<commit_message>
docs: record DEC-009 as decided in the Decision Log and mark ADR-001 accepted
The DEC-009 row now points to ADR-001, which completes the last item under Done when on #57. The row could not change while #46 held the workbook.

The M1 entry stays visible in the same row. Each changed cell holds the M2 entry first and the M1 baseline text after it, word for word, so the assessor can see what M1 deferred and what M2 decided, as the M2 brief requires for baselined content. The identifier is unchanged because ADR-001 and the driver document both cite DEC-009.

The README count of deferred decisions is a formula, and its stored result is updated from 4 to 3 so that viewers which do not recalculate show the right figure. Excel recalculates it to 3 as well. Only those two sheet parts change. The other 59 parts are byte-identical.

Refs: #57, DEC-009, #46, #72
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -3976,7 +3976,7 @@
       </c>
       <c r="B27" s="6" t="n">
         <f aca="false">COUNTIF('Decision Log'!C3:C200,"DEFERRED to M2")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -4370,42 +4370,72 @@
         <v>708</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="140.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
         <v>709</v>
       </c>
       <c r="B11" s="9" t="s">
         <v>710</v>
       </c>
-      <c r="C11" s="9" t="s">
-        <v>699</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>711</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>712</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>713</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>703</v>
-      </c>
-      <c r="H11" s="9" t="s">
-        <v>714</v>
-      </c>
-      <c r="I11" s="9" t="s">
-        <v>715</v>
-      </c>
-      <c r="J11" s="9" t="s">
-        <v>716</v>
-      </c>
-      <c r="K11" s="9" t="s">
-        <v>717</v>
-      </c>
-      <c r="L11" s="9" t="s">
-        <v>718</v>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decided (M2, ADR-001)
+M1 baseline: DEFERRED to M2</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 (23 September 2026, ADR-001): ADR-001 in docs/decisions records the context. The drivers in docs/architecture/asr-quality-drivers.md (#56) answer the first evidence condition: NFR-005, NFR-001, NFR-002, NFR-011, NFR-012, NFR-013 and NFR-003 proved architecturally significant, with CON-06 carried as a bound on complexity.
+M1 baseline: Architecture must follow from the architecturally significant requirements, and those are only being baselined in this document.</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 (23 September 2026, ADR-001): Drivers ASR-01 to ASR-06 (#56), which carry NFR-001, NFR-002, NFR-003, NFR-005, NFR-011, NFR-012 and NFR-013. Constraints CON-02 schedule; CON-03 cost; CON-06 capability; CON-07 platform availability; CON-08 governance.
+M1 baseline: NFR-001 performance; NFR-003 availability; NFR-005 authorisation; NFR-012 maintainability; CON-06 capability.</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 (23 September 2026, ADR-001): (a) Modular monolith: one deployable application in modules with explicit interfaces over one relational store. (b) Service per capability. (c) Function per operation. (d) Client application over a hosted data service.
+M1 baseline: Not yet evaluated.</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 (23 September 2026, ADR-001): Option (a), with reporting reading the transactional store for now. Five boundary rules: one server-side entry point; authorisation and read scope decided in the policy module; a status change and its audit entry written in one transaction; notification through an in-process interface; module dependencies through declared interfaces only.
+M1 baseline: Deliberately not decided.</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 (23 September 2026, ADR-001): ASR-01, ASR-03 and ASR-04 favour one enforcement point, one write path and one testable surface, which are cheaper to hold inside a process boundary. ASR-05 and ASR-06 penalise every additional deployable unit, in free-tier quota and in learning time. No baselined requirement asks for independent deployment, independent scaling or a second consumer of the data, so the evidence for (b), (c) and (d) is absent.
+M1 baseline: The quality attributes that should drive the choice are baselined here for the first time. Choosing before they were agreed would invert the dependency.</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 (23 September 2026, ADR-001): Module boundaries inside one process can erode, and review is the control until #67 adds a dependency check. One deployable unit is a single point of failure, accepted against NFR-003's 98 percent within published service hours. Reporting shares the transactional store while volume and retention are unknown (FEC-06). Scaling is whole-application scaling.
+M1 baseline: None while requirements work continues.</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 (23 September 2026, ADR-001): Two risks proposed to the Risk Register under #68: module boundaries eroding under schedule pressure (related to RSK-01 and CON-02), and reporting growth degrading the staff queue before it is measured (FEC-06, related to NFR-001 and RSK-09). DEC-008 (#59) and DEC-010 (#60) are taken against this decision, which answers the M1 risk below.
+M1 baseline: The choice interacts with DEC-008 and DEC-010; deciding any one in isolation constrains the other two.</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 (23 September 2026, ADR-001): ADR-001, approved under #72; drivers in docs/architecture/asr-quality-drivers.md (#56); module and deployment views in docs/architecture/diagrams. ADR-001 answers the three M1 conditions: the significant NFRs are identified; FEC-01 is partly answered, with scope held in the policy module; FEC-06 is answered for now, with the conditions for revisiting it recorded.
+M1 baseline: Evidence still required: which NFRs prove architecturally significant; the record-level authorisation shape from FEC-01; the reporting load position from FEC-06.</t>
+        </is>
+      </c>
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 (23 September 2026, ADR-001): Input to DEC-011 (#58), DEC-008 (#59), DEC-010 (#60) and design decisions #61 and #62. Reporting's use of the transactional store is revisited on the NFR-001 measurement or when volume and retention arrive under #2.
+M1 baseline: Sets the structure that maintainability and change cost depend on for the rest of the project.</t>
+        </is>
       </c>
     </row>
     <row r="12" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
docs: record DEC-009 as decided in the Decision Log and mark ADR-001 accepted (#82)
The DEC-009 row now points to ADR-001, which completes the last item under Done when on #57. The row could not change while #46 held the workbook.

The M1 entry stays visible in the same row. Each changed cell holds the M2 entry first and the M1 baseline text after it, word for word, so the assessor can see what M1 deferred and what M2 decided, as the M2 brief requires for baselined content. The identifier is unchanged because ADR-001 and the driver document both cite DEC-009.

The README count of deferred decisions is a formula, and its stored result is updated from 4 to 3 so that viewers which do not recalculate show the right figure. Excel recalculates it to 3 as well. Only those two sheet parts change. The other 59 parts are byte-identical.

Refs: #57, DEC-009, #46, #72
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -3976,7 +3976,7 @@
       </c>
       <c r="B27" s="6" t="n">
         <f aca="false">COUNTIF('Decision Log'!C3:C200,"DEFERRED to M2")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -4370,42 +4370,72 @@
         <v>708</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="140.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
         <v>709</v>
       </c>
       <c r="B11" s="9" t="s">
         <v>710</v>
       </c>
-      <c r="C11" s="9" t="s">
-        <v>699</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>711</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>712</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>713</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>703</v>
-      </c>
-      <c r="H11" s="9" t="s">
-        <v>714</v>
-      </c>
-      <c r="I11" s="9" t="s">
-        <v>715</v>
-      </c>
-      <c r="J11" s="9" t="s">
-        <v>716</v>
-      </c>
-      <c r="K11" s="9" t="s">
-        <v>717</v>
-      </c>
-      <c r="L11" s="9" t="s">
-        <v>718</v>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decided (M2, ADR-001)
+M1 baseline: DEFERRED to M2</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 (23 September 2026, ADR-001): ADR-001 in docs/decisions records the context. The drivers in docs/architecture/asr-quality-drivers.md (#56) answer the first evidence condition: NFR-005, NFR-001, NFR-002, NFR-011, NFR-012, NFR-013 and NFR-003 proved architecturally significant, with CON-06 carried as a bound on complexity.
+M1 baseline: Architecture must follow from the architecturally significant requirements, and those are only being baselined in this document.</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 (23 September 2026, ADR-001): Drivers ASR-01 to ASR-06 (#56), which carry NFR-001, NFR-002, NFR-003, NFR-005, NFR-011, NFR-012 and NFR-013. Constraints CON-02 schedule; CON-03 cost; CON-06 capability; CON-07 platform availability; CON-08 governance.
+M1 baseline: NFR-001 performance; NFR-003 availability; NFR-005 authorisation; NFR-012 maintainability; CON-06 capability.</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 (23 September 2026, ADR-001): (a) Modular monolith: one deployable application in modules with explicit interfaces over one relational store. (b) Service per capability. (c) Function per operation. (d) Client application over a hosted data service.
+M1 baseline: Not yet evaluated.</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 (23 September 2026, ADR-001): Option (a), with reporting reading the transactional store for now. Five boundary rules: one server-side entry point; authorisation and read scope decided in the policy module; a status change and its audit entry written in one transaction; notification through an in-process interface; module dependencies through declared interfaces only.
+M1 baseline: Deliberately not decided.</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 (23 September 2026, ADR-001): ASR-01, ASR-03 and ASR-04 favour one enforcement point, one write path and one testable surface, which are cheaper to hold inside a process boundary. ASR-05 and ASR-06 penalise every additional deployable unit, in free-tier quota and in learning time. No baselined requirement asks for independent deployment, independent scaling or a second consumer of the data, so the evidence for (b), (c) and (d) is absent.
+M1 baseline: The quality attributes that should drive the choice are baselined here for the first time. Choosing before they were agreed would invert the dependency.</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 (23 September 2026, ADR-001): Module boundaries inside one process can erode, and review is the control until #67 adds a dependency check. One deployable unit is a single point of failure, accepted against NFR-003's 98 percent within published service hours. Reporting shares the transactional store while volume and retention are unknown (FEC-06). Scaling is whole-application scaling.
+M1 baseline: None while requirements work continues.</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 (23 September 2026, ADR-001): Two risks proposed to the Risk Register under #68: module boundaries eroding under schedule pressure (related to RSK-01 and CON-02), and reporting growth degrading the staff queue before it is measured (FEC-06, related to NFR-001 and RSK-09). DEC-008 (#59) and DEC-010 (#60) are taken against this decision, which answers the M1 risk below.
+M1 baseline: The choice interacts with DEC-008 and DEC-010; deciding any one in isolation constrains the other two.</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 (23 September 2026, ADR-001): ADR-001, approved under #72; drivers in docs/architecture/asr-quality-drivers.md (#56); module and deployment views in docs/architecture/diagrams. ADR-001 answers the three M1 conditions: the significant NFRs are identified; FEC-01 is partly answered, with scope held in the policy module; FEC-06 is answered for now, with the conditions for revisiting it recorded.
+M1 baseline: Evidence still required: which NFRs prove architecturally significant; the record-level authorisation shape from FEC-01; the reporting load position from FEC-06.</t>
+        </is>
+      </c>
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 (23 September 2026, ADR-001): Input to DEC-011 (#58), DEC-008 (#59), DEC-010 (#60) and design decisions #61 and #62. Reporting's use of the transactional store is revisited on the NFR-001 measurement or when volume and retention arrive under #2.
+M1 baseline: Sets the structure that maintainability and change cost depend on for the rest of the project.</t>
+        </is>
       </c>
     </row>
     <row r="12" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
docs: record the first secret scan run in the NFR-007 RTM row
The Actions billing lock has cleared, and the Gitleaks workflow ran on #87 on 29 September 2026:
2 commits scanned, no leaks found. The NFR-007 implementation and verification cells said the
scan was blocked by the lock, and now record the run.

Refs: #54, #67, NFR-007
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -11413,12 +11413,12 @@
       </c>
       <c r="L38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">#87, open. Actions are blocked by an account billing lock</t>
+          <t xml:space="preserve">Gitleaks workflow in #87, open. It ran on #87 on 29 September 2026 and passed</t>
         </is>
       </c>
       <c r="M38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned: the scan runs on every pull request once #87 merges</t>
+          <t xml:space="preserve">Secret scan run on #87 (29 September 2026): 2 commits scanned, no leaks found. Runs on every pull request once #87 merges</t>
         </is>
       </c>
       <c r="N38" s="10" t="inlineStr">

</xml_diff>

<commit_message>
docs: add Darius Mushi's M2 AI Usage Register rows
Two rows for #70, as Darius Mushi supplied them on 30 September 2026: the #90 environment
troubleshooting, and the RSK-01 proof-of-concept test. The second row's fix is on #90 at 29eb422,
where the test file now parses.

Refs: #70, #90
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -28,7 +28,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="13" name="_xlnm._FilterDatabase" vbProcedure="false">'Access Matrix'!$A$2:$E$17</definedName>
-    <definedName function="false" hidden="true" localSheetId="10" name="_xlnm._FilterDatabase" vbProcedure="false">'AI Usage Register'!$A$2:$H$26</definedName>
+    <definedName function="false" hidden="true" localSheetId="10" name="_xlnm._FilterDatabase" vbProcedure="false">'AI Usage Register'!$A$2:$H$28</definedName>
     <definedName function="false" hidden="true" localSheetId="16" name="_xlnm._FilterDatabase" vbProcedure="false">'Baseline Sign-off'!$A$2:$B$19</definedName>
     <definedName function="false" hidden="true" localSheetId="11" name="_xlnm._FilterDatabase" vbProcedure="false">'Change Requests'!$A$2:$P$5</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">Constraints!$A$2:$D$10</definedName>
@@ -4822,7 +4822,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -5743,7 +5743,7 @@
         </is>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="47.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="59.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">29 September 2026</t>
@@ -5751,42 +5751,126 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
+          <t xml:space="preserve">Darius Mushi</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude 3.5 (Anthropic)</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diagnosing local node environment execution crash during dev runtime and client schema generations on branch #90.</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Suggested configuration mapping using custom initialization wrapper layers (src/lib/env.js).</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manually generated local client instances via "npm run prisma:generate" and checked runtime limits on local Node engine (v25.9.0).</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adopted custom path mapping patterns to resolve application bootstrap issues across varying runtime scopes.</t>
+        </is>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">My own initial local commit introduced an incorrect double nested path string (src/lib/src/lib/env.js) into prisma.js that broke text compilation; caught it on code review and fixed it back to standard relative imports.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="95.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30 September 2026</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Darius Mushi</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude 3.5 (Anthropic)</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Construction of automated integration test runner sequences to satisfy RSK-01 and ADR-002 authentication/persistence criteria.</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Provided layout structures for executing raw SQL queries and tracking validation state assertions.</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Run test runner tool locally ("npm test") using live PostgreSQL targets to check baseline passes on local host Node engine runtime environment (v25.9.0).</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Replaced generic token logs with an active argon2.hash and argon2.verify loop executing inside ephemeral temporary tables to establish robust authentication validations.</t>
+        </is>
+      </c>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A markdown parsing mismatch repeatedly inserted hidden escape backslashes (\$) before Prisma calls into the physical test script file during copy-pasting, causing syntax errors on external checkouts. Resolved by running an automated regex string replace pattern directly through the shell terminal workspace.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="47.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">29 September 2026</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">Jean Smit</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Claude Code (Anthropic)</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr">
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">M2 register changes: RTM restructure, Decision Log, change requests, RSK-12 and this register (#54, #68, #70)</t>
         </is>
       </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="E28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Drafted the RTM mapping for 42 requirements, the Decision Log rows from the ADRs, and the change requests</t>
         </is>
       </c>
-      <c r="F26" s="9" t="inlineStr">
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Every identifier checked against the ADRs, the requirements and the drivers record; the workbook parts compared before and after, with every unchanged part byte-identical; the workbook opened and recalculated in Excel and the formula values compared</t>
         </is>
       </c>
-      <c r="G26" s="9" t="inlineStr">
+      <c r="G28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Accepted after revision</t>
         </is>
       </c>
-      <c r="H26" s="9" t="inlineStr">
+      <c r="H28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">[To be completed by Jean Smit after review of this pull request.]</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:H26"/>
+  <autoFilter ref="A2:H28"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs: add Darius Mushi's A2 AI row and record DEC-008 as merged
AI Usage Register (#70): Darius Mushi's row for A2 Task 4 section 4.2, which the A2 file left for
him to supply. As supplied on 30 September 2026, with the review findings attributed to the review
that made them.

Decision Log: ADR-002 merged under #91 on 30 September 2026 with two approvals, and the DEC-008
status now records the merge.

Kept apart from #101 so its approvals were not dismissed. Only the AI Usage Register, the Decision
Log and the workbook's filter range change.

Refs: #70, #59, DEC-008
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -28,7 +28,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="13" name="_xlnm._FilterDatabase" vbProcedure="false">'Access Matrix'!$A$2:$E$17</definedName>
-    <definedName function="false" hidden="true" localSheetId="10" name="_xlnm._FilterDatabase" vbProcedure="false">'AI Usage Register'!$A$2:$H$28</definedName>
+    <definedName function="false" hidden="true" localSheetId="10" name="_xlnm._FilterDatabase" vbProcedure="false">'AI Usage Register'!$A$2:$H$29</definedName>
     <definedName function="false" hidden="true" localSheetId="16" name="_xlnm._FilterDatabase" vbProcedure="false">'Baseline Sign-off'!$A$2:$B$19</definedName>
     <definedName function="false" hidden="true" localSheetId="11" name="_xlnm._FilterDatabase" vbProcedure="false">'Change Requests'!$A$2:$P$5</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">Constraints!$A$2:$D$10</definedName>
@@ -4344,7 +4344,7 @@
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decided (M2, ADR-002 under #91), conditional on gate 3 and the RSK-01 proof of concept
+          <t xml:space="preserve">Decided (M2, ADR-002, merged under #91 on 30 September 2026), conditional on gate 3 and the RSK-01 proof of concept
 M1 baseline: DEFERRED to M2</t>
         </is>
       </c>
@@ -4822,7 +4822,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -5239,129 +5239,129 @@
         </is>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="71.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="119.0" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="inlineStr">
         <is>
+          <t xml:space="preserve">15 September 2026</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Darius Mushi</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude 3.5 (Anthropic)</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drafting Section 4.2 infrastructure text concerning automated code quality controls, code style linters, and verification warning gates.</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Provided layout structures for integrating code syntax checkers into development pipelines and proposed text outlining validation tracking strategies.</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cross-checked the generated recommendations against the local assignment criteria to ensure linting profiles were configured to issue non-blocking alerts (warnings) during early implementation blocks rather than completely failing pipeline compilation passes.</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adopted the non-blocking "warn-only" style validation constraint for initial pushes to minimize early setup friction, while explicitly deferring hard gate failures for later implementation.</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The initial automated text contained tracking errors that were caught and corrected during team review typesetting: the referenced arXiv preprint was mistakenly misattributed as Wang et al. instead of Yang et al. (2026); an unrelated cicd-sec-6 security reference point was incorrectly appended onto the OWASP CI/CD Security Cheat Sheet reference; and the review pass successfully removed two off-topic paragraphs, including one featuring an unedited, conversational AI-generated output layout structure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="71.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">21 September 2026</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Jean Smit</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Claude (Anthropic), through Claude Code</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">A3 Question 2: structuring the research, drafting the threat chains and the traceability table, and finding sources</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E15" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Structured the research, drafted the threat chains and the traceability table, and found sources</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Every cited page opened and each attributed claim found in it; the figures from Pearce et al. (2022) and Perry et al. (2023) read in the papers themselves; every reference link returned its page on 21 September 2026; citations reconciled with the reference list in both directions</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
+      <c r="G15" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Accepted after revision</t>
         </is>
       </c>
-      <c r="H14" s="9" t="inlineStr">
+      <c r="H15" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Two studies cited through Yang et al. (2026) were split across a semicolon and read as uncited sources, so the citation was rewritten to show that both are cited through Yang. The Microsoft threat modelling page is cited as 2017, the date the page states.</t>
         </is>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="154.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="inlineStr">
+    <row r="16" customFormat="false" ht="154.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">21 September 2026</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Jean Smit</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Claude (Anthropic), through Claude Code</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">A3 Question 4 and assembly (21, 22 and 28 September 2026)</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Drafted the map from Questions 1 to 3 and the registers, checked the sources of Questions 1 and 3, merged the sections, consolidated the references and built the document</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Every source cited in Questions 1 and 3 opened on 28 September 2026 and its date checked against the page; the Dijkstra (1972) point in Question 1 checked against the published text of the lecture; each map row checked against the question it summarises; every project identifier checked against the M1 registers workbook; citations reconciled in both directions across the document; the built document rendered and checked page by page</t>
         </is>
       </c>
-      <c r="G15" s="9" t="inlineStr">
+      <c r="G16" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Accepted after revision</t>
         </is>
       </c>
-      <c r="H15" s="9" t="inlineStr">
+      <c r="H16" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">The ISTQB link in Question 1 opened no entry, and the sentence citing it attributed more to the definition than it states, so the link was corrected and the citation narrowed to the definition. The NIST DOI in Question 3 did not resolve and was corrected. One Microsoft page is dated 2025 on the page itself, so the Microsoft letters were reassigned. The OWASP Secrets Management Cheat Sheet was cited under two names and dates and now has one entry. The claims Question 1 attributes to ISO/IEC/IEEE 29119-1 could not be checked against the standard, which is not freely available, and stand as the author stated them.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="71.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23 September 2026</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jean Smit</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Claude Code (Anthropic)</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Finalising ADR-002 (DEC-008) from Darius Mushi's three drafts, at his request, and amending it after review on #91 (28 September 2026)</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fact-checked the drafts against the registers and #56, checked each version, release date and licence, and drafted the finalised record and its amendments</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Versions, release dates and licences checked against the npm registry and PyPI on 23 September 2026; the Node.js release schedule and Prisma issue #30295 read directly; each member's account of their experience confirmed with them before it was recorded; the record reviewed by Darius Mushi on #91</t>
-        </is>
-      </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Accepted after revision</t>
-        </is>
-      </c>
-      <c r="H16" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The author's own Node.js experience was first recorded as tooling only, from an earlier note, and was corrected once confirmed as backend Node and Express. The first pull request description credited findings from the author's review to Darius Mushi; his review on #91 caught it and it was corrected.</t>
         </is>
       </c>
     </row>
@@ -5383,111 +5383,111 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
+          <t xml:space="preserve">Finalising ADR-002 (DEC-008) from Darius Mushi's three drafts, at his request, and amending it after review on #91 (28 September 2026)</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fact-checked the drafts against the registers and #56, checked each version, release date and licence, and drafted the finalised record and its amendments</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Versions, release dates and licences checked against the npm registry and PyPI on 23 September 2026; the Node.js release schedule and Prisma issue #30295 read directly; each member's account of their experience confirmed with them before it was recorded; the record reviewed by Darius Mushi on #91</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted after revision</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The author's own Node.js experience was first recorded as tooling only, from an earlier note, and was corrected once confirmed as backend Node and Express. The first pull request description credited findings from the author's review to Darius Mushi; his review on #91 caught it and it was corrected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="71.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">23 September 2026</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jean Smit</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code (Anthropic)</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">Moving the PED source to markdown with a Word build in the v1.0 house style (#55, CR-001)</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Wrote the conversion, the fidelity check and the build scripts, and the README</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">The fidelity check converted the markdown back to Word and compared it with v1.0: 1504 blocks, no differences, 18,169 identical words. v1.0 was rebuilt from the markdown and its 48 content pages compared with v1.0 as rendered PDF pages</t>
         </is>
       </c>
-      <c r="G17" s="9" t="inlineStr">
+      <c r="G18" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Accepted after revision</t>
         </is>
       </c>
-      <c r="H17" s="9" t="inlineStr">
+      <c r="H18" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Page comparison found build defects that were fixed before the pull request: numbered paragraphs losing their numbering, new tables wider than the page, lost bold in headings and table headers, redundant page breaks that produced blank pages, landscape margins, and Word compatibility mode.</t>
         </is>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="59.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9" t="inlineStr">
+    <row r="19" customFormat="false" ht="59.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">28 September 2026</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Jean Smit</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Claude Code (Anthropic)</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Design decisions 1 and 2: ADR-005 and ADR-006 with their code and tests (#61, #62, #93, #94)</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E19" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Drafted both records from A2 Task 1, wrote the transition table, the policy module and their tests, and exported the fixtures from the registers</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Tests generated from fixtures exported from the Status Model and Access Matrix sheets; deliberate faults introduced one at a time, three in the table and four in the policy, each failed the suite; both reviewed and approved by Darius Mushi and Tristan Roets</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="G19" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Accepted after revision</t>
         </is>
       </c>
-      <c r="H18" s="9" t="inlineStr">
+      <c r="H19" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">The tests exposed four Access Matrix cells that grant what FR-015, FR-016, FR-020 and FR-021 refuse, raised as #92 and CR-002. A risk cited as RSK-11 was RSK-05, and a Decision Log number claimed before it was assigned was removed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="47.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">28 September 2026</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jean Smit</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Claude Code (Anthropic)</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PED v2.0, sections 18 to 26 (#95)</t>
-        </is>
-      </c>
-      <c r="E19" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Drafted the M2 sections from the ADRs and pull requests, and the reading notes in the M1 sections</t>
-        </is>
-      </c>
-      <c r="F19" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Each section checked against its ADR; the M1 sections compared with v1.0 so that only the changes recorded in the v2.0 row differ; the built document rendered and checked; reviewed by Darius Mushi on #95</t>
-        </is>
-      </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Accepted after revision</t>
-        </is>
-      </c>
-      <c r="H19" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Darius Mushi's review found the cover contradicting s16 on the M1 sign-off, s8.3 conflicting with s22.2, a miscount in s19 and uncited facts in s20. All were corrected on 29 September 2026.</t>
         </is>
       </c>
     </row>
@@ -5509,368 +5509,410 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
+          <t xml:space="preserve">PED v2.0, sections 18 to 26 (#95)</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drafted the M2 sections from the ADRs and pull requests, and the reading notes in the M1 sections</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Each section checked against its ADR; the M1 sections compared with v1.0 so that only the changes recorded in the v2.0 row differ; the built document rendered and checked; reviewed by Darius Mushi on #95</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted after revision</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Darius Mushi's review found the cover contradicting s16 on the M1 sign-off, s8.3 conflicting with s22.2, a miscount in s19 and uncited facts in s20. All were corrected on 29 September 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="47.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">28 September 2026</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jean Smit</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code (Anthropic)</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">Reviewing pull requests #88, #89, #90, #97, #98 and #99 (28 and 29 September 2026)</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E21" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Checked each pull request against the requirements, ADRs and cited sources, ran the bootstrap, and drafted the review text</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">The bootstrap installed from clean and run on Node 24.14.0: npm test, the health endpoint and npm audit; each cited source opened; requirement claims checked against the workbook</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="G21" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Accepted after revision</t>
         </is>
       </c>
-      <c r="H20" s="9" t="inlineStr">
+      <c r="H21" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">A claim that the undeclared dotenv package would crash a production install was tested with npm ci --omit=dev, found wrong, and narrowed before the review was posted.</t>
         </is>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="142.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="inlineStr">
+    <row r="22" customFormat="false" ht="142.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">28 September 2026</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Tristan Roets</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">ChatGPT (OpenAI, GPT-5.6 Sol)</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">DEC-011 / #58: data and persistence design</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="E22" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Used as a review and drafting aid while I developed the data and persistence decision. It helped me organise parts of the ADR and check that I had covered the required areas.</t>
         </is>
       </c>
-      <c r="F21" s="9" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I checked the final design against FR-005 to FR-009, FR-011, FR-012, FR-017, FR-018, FR-020, FR-021, FR-025, FR-026, ADR-001, ADR-005 and ADR-006, including requester/category scope, ActionEntry visibility, status history and structured audit requirements.</t>
         </is>
       </c>
-      <c r="G21" s="9" t="inlineStr">
+      <c r="G22" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I selected and documented the final PostgreSQL relational model, Prisma as the authoritative application schema, request reference approach, transaction boundaries and integrity controls. AI suggestions were only used where they agreed with the project evidence.</t>
         </is>
       </c>
-      <c r="H21" s="9" t="inlineStr">
+      <c r="H22" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">PR review found that the first draft did not fully separate RequestStatusHistory, ActionEntry and AuditEntry responsibilities; it was missing some required Request fields and clearer transaction semantics; and it was ambiguous about the authoritative Prisma versus SQL schema. I corrected those points in ADR-007 and aligned the initial SQL/schema wording before review continued.</t>
         </is>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="119.0" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9" t="inlineStr">
+    <row r="23" customFormat="false" ht="119.0" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">28 September 2026</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Tristan Roets</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">ChatGPT (OpenAI, GPT-5.6 Sol)</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">#63: request status notification interface</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="E23" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Used to help review and organise my notification-interface ADR and check that the main interface concerns were covered.</t>
         </is>
       </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I checked the final interface against FR-017, FR-029, DEC-005, SC-D-01, FEC-03, ADR-001, ADR-005, ADR-006 and ADR-007.</t>
         </is>
       </c>
-      <c r="G22" s="9" t="inlineStr">
+      <c r="G23" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I retained the in-process M2 notification interface, derived requester indications from persisted RequestStatusHistory and requester-visible ActionEntry evidence, and kept email/SMS and asynchronous external delivery deferred.</t>
         </is>
       </c>
-      <c r="H22" s="9" t="inlineStr">
+      <c r="H23" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">PR review found that the original version did not map all four FR-029 events precisely enough, mixed visibility into the wrong contract, had unclear next-sign-in persistence/failure behaviour and used outdated persistence references. I corrected the event mapping, limited visibility to requester-visible ActionEntries, based indications on persisted evidence, and updated the ADR references.</t>
         </is>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="71.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9" t="inlineStr">
+    <row r="24" customFormat="false" ht="71.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">28 September 2026</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Tristan Roets</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">ChatGPT (OpenAI, GPT-5.6 Sol)</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">#95/#99: PED v2.0 sections 21 and 23</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="E24" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Used as a writing and checking aid while I converted my #58 and #63 work into shorter PED sections and followed the required Markdown format.</t>
         </is>
       </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I compared s21 with ADR-007 and s23 with ADR-008 to make sure the PED accurately summarised the underlying decisions without adding new ones.</t>
         </is>
       </c>
-      <c r="G23" s="9" t="inlineStr">
+      <c r="G24" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I wrote the final PED contribution and submitted it in #99.</t>
         </is>
       </c>
-      <c r="H23" s="9" t="inlineStr">
+      <c r="H24" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Review identified that visibility had initially been described on the wrong entity, ADR references needed to be explicit, unsupported notification wording had to be removed and the section boundary before s24 needed correcting. I updated #99 accordingly.</t>
         </is>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="83.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="9" t="inlineStr">
+    <row r="25" customFormat="false" ht="83.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">29 September 2026</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Tristan Roets</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">ChatGPT (OpenAI, GPT-5.6 Sol)</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">#68: M2 risk, assumption and FEC review</t>
         </is>
       </c>
-      <c r="E24" s="9" t="inlineStr">
+      <c r="E25" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Used to help organise my review of which register entries were affected by the M2 work and to cross-check related issue and ADR references.</t>
         </is>
       </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I checked the proposed updates against the actual Risk Register descriptions, the relevant M2 ADR Risks created sections and current repository evidence, including the Prisma dependency finding.</t>
         </is>
       </c>
-      <c r="G24" s="9" t="inlineStr">
+      <c r="G25" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I determined which existing risks/FECs needed updated ratings or status and supplied Jean with the new ADR-created risk rows for the combined registers PR.</t>
         </is>
       </c>
-      <c r="H24" s="9" t="inlineStr">
+      <c r="H25" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">My first pass linked several IDs to the wrong concerns. After checking the register, I corrected RSK-05, RSK-10, RSK-13 and FEC-07, kept FEC-01 only partly answered, rescored RSK-12 as materialised-active, and added the new ADR-created risks.</t>
         </is>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="95.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="9" t="inlineStr">
+    <row r="26" customFormat="false" ht="95.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">21 September 2026</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Tristan Roets</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">ChatGPT (OpenAI, GPT-5.6 Sol)</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Assignment 3 Question 3 / #76/#89: production readiness research (21 to 29 September 2026)</t>
         </is>
       </c>
-      <c r="E25" s="9" t="inlineStr">
+      <c r="E26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Used as a research and writing aid to help organise my research, identify possible sources and review wording.</t>
         </is>
       </c>
-      <c r="F25" s="9" t="inlineStr">
+      <c r="F26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I checked the technical claims against the sources used in my research, including Twelve-Factor, OWASP, GitHub Docs, Microsoft Learn, Google SRE and NIST.</t>
         </is>
       </c>
-      <c r="G25" s="9" t="inlineStr">
+      <c r="G26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I selected the final content and sources and kept the research separate from actual CivicConnect M3 implementation decisions.</t>
         </is>
       </c>
-      <c r="H25" s="9" t="inlineStr">
+      <c r="H26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">PR review found an incorrect nested file location, the NIST DOI was wrong, several reference names/dates and in-text citations did not match A3_CHANGES.md, the evidence matrix/AI record needed GitHub Markdown pipe-table formatting, and stale working-draft wording needed removal. I corrected those items on #89; the PR is still awaiting final review/merge.</t>
         </is>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="59.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="9" t="inlineStr">
+    <row r="27" customFormat="false" ht="59.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">29 September 2026</t>
         </is>
       </c>
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Darius Mushi</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
+      <c r="C27" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Claude 3.5 (Anthropic)</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Diagnosing local node environment execution crash during dev runtime and client schema generations on branch #90.</t>
         </is>
       </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="E27" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Suggested configuration mapping using custom initialization wrapper layers (src/lib/env.js).</t>
         </is>
       </c>
-      <c r="F26" s="9" t="inlineStr">
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Manually generated local client instances via "npm run prisma:generate" and checked runtime limits on local Node engine (v25.9.0).</t>
         </is>
       </c>
-      <c r="G26" s="9" t="inlineStr">
+      <c r="G27" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Adopted custom path mapping patterns to resolve application bootstrap issues across varying runtime scopes.</t>
         </is>
       </c>
-      <c r="H26" s="9" t="inlineStr">
+      <c r="H27" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">My own initial local commit introduced an incorrect double nested path string (src/lib/src/lib/env.js) into prisma.js that broke text compilation; caught it on code review and fixed it back to standard relative imports.</t>
         </is>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="95.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="9" t="inlineStr">
+    <row r="28" customFormat="false" ht="95.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">30 September 2026</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Darius Mushi</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Claude 3.5 (Anthropic)</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Construction of automated integration test runner sequences to satisfy RSK-01 and ADR-002 authentication/persistence criteria.</t>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
+      <c r="E28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Provided layout structures for executing raw SQL queries and tracking validation state assertions.</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Run test runner tool locally ("npm test") using live PostgreSQL targets to check baseline passes on local host Node engine runtime environment (v25.9.0).</t>
         </is>
       </c>
-      <c r="G27" s="9" t="inlineStr">
+      <c r="G28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Replaced generic token logs with an active argon2.hash and argon2.verify loop executing inside ephemeral temporary tables to establish robust authentication validations.</t>
         </is>
       </c>
-      <c r="H27" s="9" t="inlineStr">
+      <c r="H28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">A markdown parsing mismatch repeatedly inserted hidden escape backslashes (\$) before Prisma calls into the physical test script file during copy-pasting, causing syntax errors on external checkouts. Resolved by running an automated regex string replace pattern directly through the shell terminal workspace.</t>
         </is>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="47.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="9" t="inlineStr">
+    <row r="29" customFormat="false" ht="47.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">29 September 2026</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Jean Smit</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="C29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Claude Code (Anthropic)</t>
         </is>
       </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">M2 register changes: RTM restructure, Decision Log, change requests, RSK-12 and this register (#54, #68, #70)</t>
         </is>
       </c>
-      <c r="E28" s="9" t="inlineStr">
+      <c r="E29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Drafted the RTM mapping for 42 requirements, the Decision Log rows from the ADRs, and the change requests</t>
         </is>
       </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="F29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Every identifier checked against the ADRs, the requirements and the drivers record; the workbook parts compared before and after, with every unchanged part byte-identical; the workbook opened and recalculated in Excel and the formula values compared</t>
         </is>
       </c>
-      <c r="G28" s="9" t="inlineStr">
+      <c r="G29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Accepted after revision</t>
         </is>
       </c>
-      <c r="H28" s="9" t="inlineStr">
+      <c r="H29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">[To be completed by Jean Smit after review of this pull request.]</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:H28"/>
+  <autoFilter ref="A2:H29"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs: add RSK-24 to RSK-29 from ADR-001, ADR-002 and ADR-008
The remaining risks the M2 ADRs propose under #68, as Tristan Roets supplied them on 30 September
2026:
- RSK-24, ADR-001: module boundaries erode under schedule pressure (12, High). Owner Jean Smit.
- RSK-25, ADR-002: Prisma version drift (8, Medium). Owner Darius Mushi.
- RSK-26, ADR-002: duplicate scheduled jobs from more than one instance (8, Medium). Owner Darius
  Mushi.
- RSK-27 to RSK-29, ADR-008: the FR-029 mapping drifting from the workflow, derived notification
  queries slowing as history grows, and external delivery added without retry and idempotency
  (6, 6 and 8, Medium). Owner Tristan Roets. ADR-008's second risk is RSK-23.

README risk counts recomputed from the sheet: 2 Critical, 10 High, 17 Medium, matching Excel's
recalculation.

Refs: #68, ADR-001, ADR-002, ADR-008
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -37,7 +37,7 @@
     <definedName function="false" hidden="true" localSheetId="15" name="_xlnm._FilterDatabase" vbProcedure="false">'GitHub Governance'!$A$2:$C$14</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Requirements (FR)'!$A$2:$F$31</definedName>
     <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">'Requirements (NFR)'!$A$2:$G$15</definedName>
-    <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">'Risk Register'!$A$2:$L$25</definedName>
+    <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">'Risk Register'!$A$2:$L$31</definedName>
     <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">RTM!$A$2:$O$44</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Scope Baseline'!$A$2:$E$27</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Stakeholders!$A$2:$G$11</definedName>
@@ -3934,7 +3934,7 @@
       </c>
       <c r="B22" s="6" t="n">
         <f aca="false">COUNTIF('Risk Register'!G3:G200,"High")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3943,7 +3943,7 @@
       </c>
       <c r="B23" s="6" t="n">
         <f aca="false">COUNTIF('Risk Register'!G3:G200,"Medium")</f>
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11955,7 +11955,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -13085,8 +13085,344 @@
         </is>
       </c>
     </row>
+    <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RSK-24</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module boundaries inside the modular monolith erode under schedule pressure until the application becomes a tangled unit, increasing later change cost and threatening NFR-012.</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule pressure causes developers to bypass declared module interfaces and call another module directly because it is quicker.</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E26" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="F26" s="13" t="n">
+        <f aca="false">D26*E26</f>
+        <v>12</v>
+      </c>
+      <c r="G26" s="13" t="str">
+        <f aca="false">IF(F26&gt;=20,"Critical",IF(F26&gt;=12,"High",IF(F26&gt;=6,"Medium","Low")))</f>
+        <v>High</v>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Keep dependencies behind declared module interfaces, enforce boundaries through review, and add the dependency check under #67 when the structure exists to check automatically.</t>
+        </is>
+      </c>
+      <c r="I26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stop further feature work on the affected path and refactor the coupled modules back behind their declared interfaces before continuing.</t>
+        </is>
+      </c>
+      <c r="J26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jean Smit</t>
+        </is>
+      </c>
+      <c r="K26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="L26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-001, NFR-012, CON-02, RSK-01, #57, #67</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RSK-25</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An unpinned Prisma install can mix incompatible Prisma versions, such as the Prisma 8 release candidate with the Prisma 7 client.</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prisma packages are installed without the exact controlled pins, allowing Prisma 8 release-candidate or otherwise mismatched versions to drift from the approved Prisma 7 stack.</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F27" s="11" t="n">
+        <f aca="false">D27*E27</f>
+        <v>8</v>
+      </c>
+      <c r="G27" s="11" t="str">
+        <f aca="false">IF(F27&gt;=20,"Critical",IF(F27&gt;=12,"High",IF(F27&gt;=6,"Medium","Low")))</f>
+        <v>Medium</v>
+      </c>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pin all Prisma packages to the same exact version, keep the lockfile committed, and use npm ci. Prisma 8 should only be adopted through a later controlled decision after stable release.</t>
+        </is>
+      </c>
+      <c r="I27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Restore the exact approved Prisma version pins and committed lockfile, run npm ci, regenerate the Prisma client and rerun the build and tests before continuing.</t>
+        </is>
+      </c>
+      <c r="J27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Darius Mushi</t>
+        </is>
+      </c>
+      <c r="K27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="L27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-002, RSK-12, DEC-008, #59, #90</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RSK-26</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">node-cron runs inside the application process, so if more than one application instance is running, every scheduled job can execute more than once.</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">More than one application instance runs while node-cron scheduling is enabled, causing every instance to fire the same scheduled job.</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="F28" s="13" t="n">
+        <f aca="false">D28*E28</f>
+        <v>8</v>
+      </c>
+      <c r="G28" s="13" t="str">
+        <f aca="false">IF(F28&gt;=20,"Critical",IF(F28&gt;=12,"High",IF(F28&gt;=6,"Medium","Low")))</f>
+        <v>Medium</v>
+      </c>
+      <c r="H28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEC-010 must run exactly one instance while in-process scheduling is in use. Revisit the scheduling approach before introducing multiple application instances or asynchronous workers.</t>
+        </is>
+      </c>
+      <c r="I28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stop the duplicate scheduled execution and ensure exactly one application instance performs scheduling until a controlled alternative scheduler design is approved.</t>
+        </is>
+      </c>
+      <c r="J28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Darius Mushi</t>
+        </is>
+      </c>
+      <c r="K28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="L28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-002, DEC-010, FEC-03, RSK-02, #59, #60</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RSK-27</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FR-029 notification event mapping becomes inconsistent with workflow changes.</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-005 status transitions are changed without the ADR-008 notification mapping being reviewed and updated at the same time.</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F29" s="11" t="n">
+        <f aca="false">D29*E29</f>
+        <v>6</v>
+      </c>
+      <c r="G29" s="11" t="str">
+        <f aca="false">IF(F29&gt;=20,"Critical",IF(F29&gt;=12,"High",IF(F29&gt;=6,"Medium","Low")))</f>
+        <v>Medium</v>
+      </c>
+      <c r="H29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-005 remains the status-transition authority; every change to a transition used by accepted, rejected or completed notifications must review ADR-008 and the FR-029 mapping before merge.</t>
+        </is>
+      </c>
+      <c r="I29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stop release of the affected workflow change, correct the notification mapping and tests or evidence, and re-review the affected ADR and RTM references before continuing.</t>
+        </is>
+      </c>
+      <c r="J29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tristan Roets</t>
+        </is>
+      </c>
+      <c r="K29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="L29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-008, ADR-005, FR-029, #63, #68</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RSK-28</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Derived notification queries become inefficient as request history grows.</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 derives notifications from RequestStatusHistory and requester-visible ActionEntry evidence rather than using a dedicated notification read model or Notification table.</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F30" s="13" t="n">
+        <f aca="false">D30*E30</f>
+        <v>6</v>
+      </c>
+      <c r="G30" s="13" t="str">
+        <f aca="false">IF(F30&gt;=20,"Critical",IF(F30&gt;=12,"High",IF(F30&gt;=6,"Medium","Low")))</f>
+        <v>Medium</v>
+      </c>
+      <c r="H30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-007 owns indexes and query measurement; measure the notification query path as data volume grows and keep requester-scoped queries indexed.</t>
+        </is>
+      </c>
+      <c r="I30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If measured evidence shows the derived-query path is inadequate, introduce a dedicated notification read model or persisted Notification entity through a controlled persistence and interface decision.</t>
+        </is>
+      </c>
+      <c r="J30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tristan Roets</t>
+        </is>
+      </c>
+      <c r="K30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="L30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-008, ADR-007, FR-029, #63, #68</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RSK-29</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">External notification delivery is added without durable retry and idempotency behaviour.</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Email, SMS or another asynchronous delivery path is introduced from the M2 in-process interface without first defining persistence, retries, duplicate handling, secrets and operational monitoring.</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F31" s="11" t="n">
+        <f aca="false">D31*E31</f>
+        <v>8</v>
+      </c>
+      <c r="G31" s="11" t="str">
+        <f aca="false">IF(F31&gt;=20,"Critical",IF(F31&gt;=12,"High",IF(F31&gt;=6,"Medium","Low")))</f>
+        <v>Medium</v>
+      </c>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Keep SC-D-01 deferred. Reopening external delivery requires a follow-up interface and deployment decision covering persistence, retries, duplicates, secrets and monitoring before implementation.</t>
+        </is>
+      </c>
+      <c r="I31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Disable the external delivery path, retain the in-application persisted-evidence notification behaviour, and redesign the external path with durable retry and idempotency controls before re-enabling it.</t>
+        </is>
+      </c>
+      <c r="J31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tristan Roets</t>
+        </is>
+      </c>
+      <c r="K31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="L31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-008, SC-D-01, FEC-03, ADR-001 rule 4, #63, #68</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L25"/>
+  <autoFilter ref="A2:L31"/>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs: complete the M2 registers: RSK-24 to RSK-29, Darius Mushi's A2 AI row and ADR-002 accepted (#104)
The register entries that arrived after #101 was approved, kept apart so its approvals were not
dismissed.

Risk Register: RSK-24 to RSK-29, the risks ADR-001, ADR-002 and ADR-008 propose, as Tristan Roets
supplied them. RSK-24 module boundaries (12, High, owner Jean Smit); RSK-25 Prisma version drift and
RSK-26 duplicate scheduled jobs (8, Medium, owner Darius Mushi); RSK-27 to RSK-29 from ADR-008 (6 to
8, Medium, owner Tristan Roets). README counts match Excel's recalculation: 2 Critical, 10 High,
17 Medium.

AI Usage Register: Darius Mushi's row for A2 Task 4 section 4.2.

Decision Log and ADR-002: DEC-008 records ADR-002 merging under #91, and ADR-002's status is
Accepted, conditional on gate 3 and the RSK-01 proof of concept.

Refs: #68, #70, #59, DEC-008
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -28,7 +28,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="13" name="_xlnm._FilterDatabase" vbProcedure="false">'Access Matrix'!$A$2:$E$17</definedName>
-    <definedName function="false" hidden="true" localSheetId="10" name="_xlnm._FilterDatabase" vbProcedure="false">'AI Usage Register'!$A$2:$H$28</definedName>
+    <definedName function="false" hidden="true" localSheetId="10" name="_xlnm._FilterDatabase" vbProcedure="false">'AI Usage Register'!$A$2:$H$29</definedName>
     <definedName function="false" hidden="true" localSheetId="16" name="_xlnm._FilterDatabase" vbProcedure="false">'Baseline Sign-off'!$A$2:$B$19</definedName>
     <definedName function="false" hidden="true" localSheetId="11" name="_xlnm._FilterDatabase" vbProcedure="false">'Change Requests'!$A$2:$P$5</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">Constraints!$A$2:$D$10</definedName>
@@ -37,7 +37,7 @@
     <definedName function="false" hidden="true" localSheetId="15" name="_xlnm._FilterDatabase" vbProcedure="false">'GitHub Governance'!$A$2:$C$14</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Requirements (FR)'!$A$2:$F$31</definedName>
     <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">'Requirements (NFR)'!$A$2:$G$15</definedName>
-    <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">'Risk Register'!$A$2:$L$25</definedName>
+    <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">'Risk Register'!$A$2:$L$31</definedName>
     <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">RTM!$A$2:$O$44</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Scope Baseline'!$A$2:$E$27</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Stakeholders!$A$2:$G$11</definedName>
@@ -3934,7 +3934,7 @@
       </c>
       <c r="B22" s="6" t="n">
         <f aca="false">COUNTIF('Risk Register'!G3:G200,"High")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3943,7 +3943,7 @@
       </c>
       <c r="B23" s="6" t="n">
         <f aca="false">COUNTIF('Risk Register'!G3:G200,"Medium")</f>
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4344,7 +4344,7 @@
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decided (M2, ADR-002 under #91), conditional on gate 3 and the RSK-01 proof of concept
+          <t xml:space="preserve">Decided (M2, ADR-002, merged under #91 on 30 September 2026), conditional on gate 3 and the RSK-01 proof of concept
 M1 baseline: DEFERRED to M2</t>
         </is>
       </c>
@@ -4822,7 +4822,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -5239,129 +5239,129 @@
         </is>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="71.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="119.0" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="inlineStr">
         <is>
+          <t xml:space="preserve">15 September 2026</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Darius Mushi</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude 3.5 (Anthropic)</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drafting Section 4.2 infrastructure text concerning automated code quality controls, code style linters, and verification warning gates.</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Provided layout structures for integrating code syntax checkers into development pipelines and proposed text outlining validation tracking strategies.</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cross-checked the generated recommendations against the local assignment criteria to ensure linting profiles were configured to issue non-blocking alerts (warnings) during early implementation blocks rather than completely failing pipeline compilation passes.</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adopted the non-blocking "warn-only" style validation constraint for initial pushes to minimize early setup friction, while explicitly deferring hard gate failures for later implementation.</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The initial automated text contained tracking errors that were caught and corrected during team review typesetting: the referenced arXiv preprint was mistakenly misattributed as Wang et al. instead of Yang et al. (2026); an unrelated cicd-sec-6 security reference point was incorrectly appended onto the OWASP CI/CD Security Cheat Sheet reference; and the review pass successfully removed two off-topic paragraphs, including one featuring an unedited, conversational AI-generated output layout structure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="71.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">21 September 2026</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Jean Smit</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Claude (Anthropic), through Claude Code</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">A3 Question 2: structuring the research, drafting the threat chains and the traceability table, and finding sources</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E15" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Structured the research, drafted the threat chains and the traceability table, and found sources</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Every cited page opened and each attributed claim found in it; the figures from Pearce et al. (2022) and Perry et al. (2023) read in the papers themselves; every reference link returned its page on 21 September 2026; citations reconciled with the reference list in both directions</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
+      <c r="G15" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Accepted after revision</t>
         </is>
       </c>
-      <c r="H14" s="9" t="inlineStr">
+      <c r="H15" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Two studies cited through Yang et al. (2026) were split across a semicolon and read as uncited sources, so the citation was rewritten to show that both are cited through Yang. The Microsoft threat modelling page is cited as 2017, the date the page states.</t>
         </is>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="154.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="inlineStr">
+    <row r="16" customFormat="false" ht="154.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">21 September 2026</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Jean Smit</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Claude (Anthropic), through Claude Code</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">A3 Question 4 and assembly (21, 22 and 28 September 2026)</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Drafted the map from Questions 1 to 3 and the registers, checked the sources of Questions 1 and 3, merged the sections, consolidated the references and built the document</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Every source cited in Questions 1 and 3 opened on 28 September 2026 and its date checked against the page; the Dijkstra (1972) point in Question 1 checked against the published text of the lecture; each map row checked against the question it summarises; every project identifier checked against the M1 registers workbook; citations reconciled in both directions across the document; the built document rendered and checked page by page</t>
         </is>
       </c>
-      <c r="G15" s="9" t="inlineStr">
+      <c r="G16" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Accepted after revision</t>
         </is>
       </c>
-      <c r="H15" s="9" t="inlineStr">
+      <c r="H16" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">The ISTQB link in Question 1 opened no entry, and the sentence citing it attributed more to the definition than it states, so the link was corrected and the citation narrowed to the definition. The NIST DOI in Question 3 did not resolve and was corrected. One Microsoft page is dated 2025 on the page itself, so the Microsoft letters were reassigned. The OWASP Secrets Management Cheat Sheet was cited under two names and dates and now has one entry. The claims Question 1 attributes to ISO/IEC/IEEE 29119-1 could not be checked against the standard, which is not freely available, and stand as the author stated them.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="71.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23 September 2026</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jean Smit</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Claude Code (Anthropic)</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Finalising ADR-002 (DEC-008) from Darius Mushi's three drafts, at his request, and amending it after review on #91 (28 September 2026)</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fact-checked the drafts against the registers and #56, checked each version, release date and licence, and drafted the finalised record and its amendments</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Versions, release dates and licences checked against the npm registry and PyPI on 23 September 2026; the Node.js release schedule and Prisma issue #30295 read directly; each member's account of their experience confirmed with them before it was recorded; the record reviewed by Darius Mushi on #91</t>
-        </is>
-      </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Accepted after revision</t>
-        </is>
-      </c>
-      <c r="H16" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The author's own Node.js experience was first recorded as tooling only, from an earlier note, and was corrected once confirmed as backend Node and Express. The first pull request description credited findings from the author's review to Darius Mushi; his review on #91 caught it and it was corrected.</t>
         </is>
       </c>
     </row>
@@ -5383,111 +5383,111 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
+          <t xml:space="preserve">Finalising ADR-002 (DEC-008) from Darius Mushi's three drafts, at his request, and amending it after review on #91 (28 September 2026)</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fact-checked the drafts against the registers and #56, checked each version, release date and licence, and drafted the finalised record and its amendments</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Versions, release dates and licences checked against the npm registry and PyPI on 23 September 2026; the Node.js release schedule and Prisma issue #30295 read directly; each member's account of their experience confirmed with them before it was recorded; the record reviewed by Darius Mushi on #91</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted after revision</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The author's own Node.js experience was first recorded as tooling only, from an earlier note, and was corrected once confirmed as backend Node and Express. The first pull request description credited findings from the author's review to Darius Mushi; his review on #91 caught it and it was corrected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="71.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">23 September 2026</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jean Smit</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code (Anthropic)</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">Moving the PED source to markdown with a Word build in the v1.0 house style (#55, CR-001)</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Wrote the conversion, the fidelity check and the build scripts, and the README</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">The fidelity check converted the markdown back to Word and compared it with v1.0: 1504 blocks, no differences, 18,169 identical words. v1.0 was rebuilt from the markdown and its 48 content pages compared with v1.0 as rendered PDF pages</t>
         </is>
       </c>
-      <c r="G17" s="9" t="inlineStr">
+      <c r="G18" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Accepted after revision</t>
         </is>
       </c>
-      <c r="H17" s="9" t="inlineStr">
+      <c r="H18" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Page comparison found build defects that were fixed before the pull request: numbered paragraphs losing their numbering, new tables wider than the page, lost bold in headings and table headers, redundant page breaks that produced blank pages, landscape margins, and Word compatibility mode.</t>
         </is>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="59.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9" t="inlineStr">
+    <row r="19" customFormat="false" ht="59.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">28 September 2026</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Jean Smit</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Claude Code (Anthropic)</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Design decisions 1 and 2: ADR-005 and ADR-006 with their code and tests (#61, #62, #93, #94)</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E19" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Drafted both records from A2 Task 1, wrote the transition table, the policy module and their tests, and exported the fixtures from the registers</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Tests generated from fixtures exported from the Status Model and Access Matrix sheets; deliberate faults introduced one at a time, three in the table and four in the policy, each failed the suite; both reviewed and approved by Darius Mushi and Tristan Roets</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="G19" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Accepted after revision</t>
         </is>
       </c>
-      <c r="H18" s="9" t="inlineStr">
+      <c r="H19" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">The tests exposed four Access Matrix cells that grant what FR-015, FR-016, FR-020 and FR-021 refuse, raised as #92 and CR-002. A risk cited as RSK-11 was RSK-05, and a Decision Log number claimed before it was assigned was removed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="47.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">28 September 2026</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jean Smit</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Claude Code (Anthropic)</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PED v2.0, sections 18 to 26 (#95)</t>
-        </is>
-      </c>
-      <c r="E19" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Drafted the M2 sections from the ADRs and pull requests, and the reading notes in the M1 sections</t>
-        </is>
-      </c>
-      <c r="F19" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Each section checked against its ADR; the M1 sections compared with v1.0 so that only the changes recorded in the v2.0 row differ; the built document rendered and checked; reviewed by Darius Mushi on #95</t>
-        </is>
-      </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Accepted after revision</t>
-        </is>
-      </c>
-      <c r="H19" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Darius Mushi's review found the cover contradicting s16 on the M1 sign-off, s8.3 conflicting with s22.2, a miscount in s19 and uncited facts in s20. All were corrected on 29 September 2026.</t>
         </is>
       </c>
     </row>
@@ -5509,368 +5509,410 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
+          <t xml:space="preserve">PED v2.0, sections 18 to 26 (#95)</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drafted the M2 sections from the ADRs and pull requests, and the reading notes in the M1 sections</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Each section checked against its ADR; the M1 sections compared with v1.0 so that only the changes recorded in the v2.0 row differ; the built document rendered and checked; reviewed by Darius Mushi on #95</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted after revision</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Darius Mushi's review found the cover contradicting s16 on the M1 sign-off, s8.3 conflicting with s22.2, a miscount in s19 and uncited facts in s20. All were corrected on 29 September 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="47.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">28 September 2026</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jean Smit</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code (Anthropic)</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">Reviewing pull requests #88, #89, #90, #97, #98 and #99 (28 and 29 September 2026)</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E21" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Checked each pull request against the requirements, ADRs and cited sources, ran the bootstrap, and drafted the review text</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">The bootstrap installed from clean and run on Node 24.14.0: npm test, the health endpoint and npm audit; each cited source opened; requirement claims checked against the workbook</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="G21" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Accepted after revision</t>
         </is>
       </c>
-      <c r="H20" s="9" t="inlineStr">
+      <c r="H21" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">A claim that the undeclared dotenv package would crash a production install was tested with npm ci --omit=dev, found wrong, and narrowed before the review was posted.</t>
         </is>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="142.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="inlineStr">
+    <row r="22" customFormat="false" ht="142.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">28 September 2026</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Tristan Roets</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">ChatGPT (OpenAI, GPT-5.6 Sol)</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">DEC-011 / #58: data and persistence design</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="E22" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Used as a review and drafting aid while I developed the data and persistence decision. It helped me organise parts of the ADR and check that I had covered the required areas.</t>
         </is>
       </c>
-      <c r="F21" s="9" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I checked the final design against FR-005 to FR-009, FR-011, FR-012, FR-017, FR-018, FR-020, FR-021, FR-025, FR-026, ADR-001, ADR-005 and ADR-006, including requester/category scope, ActionEntry visibility, status history and structured audit requirements.</t>
         </is>
       </c>
-      <c r="G21" s="9" t="inlineStr">
+      <c r="G22" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I selected and documented the final PostgreSQL relational model, Prisma as the authoritative application schema, request reference approach, transaction boundaries and integrity controls. AI suggestions were only used where they agreed with the project evidence.</t>
         </is>
       </c>
-      <c r="H21" s="9" t="inlineStr">
+      <c r="H22" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">PR review found that the first draft did not fully separate RequestStatusHistory, ActionEntry and AuditEntry responsibilities; it was missing some required Request fields and clearer transaction semantics; and it was ambiguous about the authoritative Prisma versus SQL schema. I corrected those points in ADR-007 and aligned the initial SQL/schema wording before review continued.</t>
         </is>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="119.0" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9" t="inlineStr">
+    <row r="23" customFormat="false" ht="119.0" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">28 September 2026</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Tristan Roets</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">ChatGPT (OpenAI, GPT-5.6 Sol)</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">#63: request status notification interface</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="E23" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Used to help review and organise my notification-interface ADR and check that the main interface concerns were covered.</t>
         </is>
       </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I checked the final interface against FR-017, FR-029, DEC-005, SC-D-01, FEC-03, ADR-001, ADR-005, ADR-006 and ADR-007.</t>
         </is>
       </c>
-      <c r="G22" s="9" t="inlineStr">
+      <c r="G23" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I retained the in-process M2 notification interface, derived requester indications from persisted RequestStatusHistory and requester-visible ActionEntry evidence, and kept email/SMS and asynchronous external delivery deferred.</t>
         </is>
       </c>
-      <c r="H22" s="9" t="inlineStr">
+      <c r="H23" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">PR review found that the original version did not map all four FR-029 events precisely enough, mixed visibility into the wrong contract, had unclear next-sign-in persistence/failure behaviour and used outdated persistence references. I corrected the event mapping, limited visibility to requester-visible ActionEntries, based indications on persisted evidence, and updated the ADR references.</t>
         </is>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="71.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9" t="inlineStr">
+    <row r="24" customFormat="false" ht="71.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">28 September 2026</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Tristan Roets</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">ChatGPT (OpenAI, GPT-5.6 Sol)</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">#95/#99: PED v2.0 sections 21 and 23</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="E24" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Used as a writing and checking aid while I converted my #58 and #63 work into shorter PED sections and followed the required Markdown format.</t>
         </is>
       </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I compared s21 with ADR-007 and s23 with ADR-008 to make sure the PED accurately summarised the underlying decisions without adding new ones.</t>
         </is>
       </c>
-      <c r="G23" s="9" t="inlineStr">
+      <c r="G24" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I wrote the final PED contribution and submitted it in #99.</t>
         </is>
       </c>
-      <c r="H23" s="9" t="inlineStr">
+      <c r="H24" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Review identified that visibility had initially been described on the wrong entity, ADR references needed to be explicit, unsupported notification wording had to be removed and the section boundary before s24 needed correcting. I updated #99 accordingly.</t>
         </is>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="83.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="9" t="inlineStr">
+    <row r="25" customFormat="false" ht="83.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">29 September 2026</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Tristan Roets</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">ChatGPT (OpenAI, GPT-5.6 Sol)</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">#68: M2 risk, assumption and FEC review</t>
         </is>
       </c>
-      <c r="E24" s="9" t="inlineStr">
+      <c r="E25" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Used to help organise my review of which register entries were affected by the M2 work and to cross-check related issue and ADR references.</t>
         </is>
       </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I checked the proposed updates against the actual Risk Register descriptions, the relevant M2 ADR Risks created sections and current repository evidence, including the Prisma dependency finding.</t>
         </is>
       </c>
-      <c r="G24" s="9" t="inlineStr">
+      <c r="G25" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I determined which existing risks/FECs needed updated ratings or status and supplied Jean with the new ADR-created risk rows for the combined registers PR.</t>
         </is>
       </c>
-      <c r="H24" s="9" t="inlineStr">
+      <c r="H25" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">My first pass linked several IDs to the wrong concerns. After checking the register, I corrected RSK-05, RSK-10, RSK-13 and FEC-07, kept FEC-01 only partly answered, rescored RSK-12 as materialised-active, and added the new ADR-created risks.</t>
         </is>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="95.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="9" t="inlineStr">
+    <row r="26" customFormat="false" ht="95.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">21 September 2026</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Tristan Roets</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">ChatGPT (OpenAI, GPT-5.6 Sol)</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Assignment 3 Question 3 / #76/#89: production readiness research (21 to 29 September 2026)</t>
         </is>
       </c>
-      <c r="E25" s="9" t="inlineStr">
+      <c r="E26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Used as a research and writing aid to help organise my research, identify possible sources and review wording.</t>
         </is>
       </c>
-      <c r="F25" s="9" t="inlineStr">
+      <c r="F26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I checked the technical claims against the sources used in my research, including Twelve-Factor, OWASP, GitHub Docs, Microsoft Learn, Google SRE and NIST.</t>
         </is>
       </c>
-      <c r="G25" s="9" t="inlineStr">
+      <c r="G26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">I selected the final content and sources and kept the research separate from actual CivicConnect M3 implementation decisions.</t>
         </is>
       </c>
-      <c r="H25" s="9" t="inlineStr">
+      <c r="H26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">PR review found an incorrect nested file location, the NIST DOI was wrong, several reference names/dates and in-text citations did not match A3_CHANGES.md, the evidence matrix/AI record needed GitHub Markdown pipe-table formatting, and stale working-draft wording needed removal. I corrected those items on #89; the PR is still awaiting final review/merge.</t>
         </is>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="59.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="9" t="inlineStr">
+    <row r="27" customFormat="false" ht="59.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">29 September 2026</t>
         </is>
       </c>
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Darius Mushi</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
+      <c r="C27" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Claude 3.5 (Anthropic)</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Diagnosing local node environment execution crash during dev runtime and client schema generations on branch #90.</t>
         </is>
       </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="E27" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Suggested configuration mapping using custom initialization wrapper layers (src/lib/env.js).</t>
         </is>
       </c>
-      <c r="F26" s="9" t="inlineStr">
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Manually generated local client instances via "npm run prisma:generate" and checked runtime limits on local Node engine (v25.9.0).</t>
         </is>
       </c>
-      <c r="G26" s="9" t="inlineStr">
+      <c r="G27" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Adopted custom path mapping patterns to resolve application bootstrap issues across varying runtime scopes.</t>
         </is>
       </c>
-      <c r="H26" s="9" t="inlineStr">
+      <c r="H27" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">My own initial local commit introduced an incorrect double nested path string (src/lib/src/lib/env.js) into prisma.js that broke text compilation; caught it on code review and fixed it back to standard relative imports.</t>
         </is>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="95.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="9" t="inlineStr">
+    <row r="28" customFormat="false" ht="95.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">30 September 2026</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Darius Mushi</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Claude 3.5 (Anthropic)</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Construction of automated integration test runner sequences to satisfy RSK-01 and ADR-002 authentication/persistence criteria.</t>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
+      <c r="E28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Provided layout structures for executing raw SQL queries and tracking validation state assertions.</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Run test runner tool locally ("npm test") using live PostgreSQL targets to check baseline passes on local host Node engine runtime environment (v25.9.0).</t>
         </is>
       </c>
-      <c r="G27" s="9" t="inlineStr">
+      <c r="G28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Replaced generic token logs with an active argon2.hash and argon2.verify loop executing inside ephemeral temporary tables to establish robust authentication validations.</t>
         </is>
       </c>
-      <c r="H27" s="9" t="inlineStr">
+      <c r="H28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">A markdown parsing mismatch repeatedly inserted hidden escape backslashes (\$) before Prisma calls into the physical test script file during copy-pasting, causing syntax errors on external checkouts. Resolved by running an automated regex string replace pattern directly through the shell terminal workspace.</t>
         </is>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="47.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="9" t="inlineStr">
+    <row r="29" customFormat="false" ht="47.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">29 September 2026</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Jean Smit</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="C29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Claude Code (Anthropic)</t>
         </is>
       </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">M2 register changes: RTM restructure, Decision Log, change requests, RSK-12 and this register (#54, #68, #70)</t>
         </is>
       </c>
-      <c r="E28" s="9" t="inlineStr">
+      <c r="E29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Drafted the RTM mapping for 42 requirements, the Decision Log rows from the ADRs, and the change requests</t>
         </is>
       </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="F29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Every identifier checked against the ADRs, the requirements and the drivers record; the workbook parts compared before and after, with every unchanged part byte-identical; the workbook opened and recalculated in Excel and the formula values compared</t>
         </is>
       </c>
-      <c r="G28" s="9" t="inlineStr">
+      <c r="G29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Accepted after revision</t>
         </is>
       </c>
-      <c r="H28" s="9" t="inlineStr">
+      <c r="H29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">[To be completed by Jean Smit after review of this pull request.]</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:H28"/>
+  <autoFilter ref="A2:H29"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -11913,7 +11955,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -13043,8 +13085,344 @@
         </is>
       </c>
     </row>
+    <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RSK-24</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module boundaries inside the modular monolith erode under schedule pressure until the application becomes a tangled unit, increasing later change cost and threatening NFR-012.</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule pressure causes developers to bypass declared module interfaces and call another module directly because it is quicker.</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E26" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="F26" s="13" t="n">
+        <f aca="false">D26*E26</f>
+        <v>12</v>
+      </c>
+      <c r="G26" s="13" t="str">
+        <f aca="false">IF(F26&gt;=20,"Critical",IF(F26&gt;=12,"High",IF(F26&gt;=6,"Medium","Low")))</f>
+        <v>High</v>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Keep dependencies behind declared module interfaces, enforce boundaries through review, and add the dependency check under #67 when the structure exists to check automatically.</t>
+        </is>
+      </c>
+      <c r="I26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stop further feature work on the affected path and refactor the coupled modules back behind their declared interfaces before continuing.</t>
+        </is>
+      </c>
+      <c r="J26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jean Smit</t>
+        </is>
+      </c>
+      <c r="K26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="L26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-001, NFR-012, CON-02, RSK-01, #57, #67</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RSK-25</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An unpinned Prisma install can mix incompatible Prisma versions, such as the Prisma 8 release candidate with the Prisma 7 client.</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prisma packages are installed without the exact controlled pins, allowing Prisma 8 release-candidate or otherwise mismatched versions to drift from the approved Prisma 7 stack.</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F27" s="11" t="n">
+        <f aca="false">D27*E27</f>
+        <v>8</v>
+      </c>
+      <c r="G27" s="11" t="str">
+        <f aca="false">IF(F27&gt;=20,"Critical",IF(F27&gt;=12,"High",IF(F27&gt;=6,"Medium","Low")))</f>
+        <v>Medium</v>
+      </c>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pin all Prisma packages to the same exact version, keep the lockfile committed, and use npm ci. Prisma 8 should only be adopted through a later controlled decision after stable release.</t>
+        </is>
+      </c>
+      <c r="I27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Restore the exact approved Prisma version pins and committed lockfile, run npm ci, regenerate the Prisma client and rerun the build and tests before continuing.</t>
+        </is>
+      </c>
+      <c r="J27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Darius Mushi</t>
+        </is>
+      </c>
+      <c r="K27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="L27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-002, RSK-12, DEC-008, #59, #90</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RSK-26</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">node-cron runs inside the application process, so if more than one application instance is running, every scheduled job can execute more than once.</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">More than one application instance runs while node-cron scheduling is enabled, causing every instance to fire the same scheduled job.</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="F28" s="13" t="n">
+        <f aca="false">D28*E28</f>
+        <v>8</v>
+      </c>
+      <c r="G28" s="13" t="str">
+        <f aca="false">IF(F28&gt;=20,"Critical",IF(F28&gt;=12,"High",IF(F28&gt;=6,"Medium","Low")))</f>
+        <v>Medium</v>
+      </c>
+      <c r="H28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEC-010 must run exactly one instance while in-process scheduling is in use. Revisit the scheduling approach before introducing multiple application instances or asynchronous workers.</t>
+        </is>
+      </c>
+      <c r="I28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stop the duplicate scheduled execution and ensure exactly one application instance performs scheduling until a controlled alternative scheduler design is approved.</t>
+        </is>
+      </c>
+      <c r="J28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Darius Mushi</t>
+        </is>
+      </c>
+      <c r="K28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="L28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-002, DEC-010, FEC-03, RSK-02, #59, #60</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RSK-27</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FR-029 notification event mapping becomes inconsistent with workflow changes.</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-005 status transitions are changed without the ADR-008 notification mapping being reviewed and updated at the same time.</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F29" s="11" t="n">
+        <f aca="false">D29*E29</f>
+        <v>6</v>
+      </c>
+      <c r="G29" s="11" t="str">
+        <f aca="false">IF(F29&gt;=20,"Critical",IF(F29&gt;=12,"High",IF(F29&gt;=6,"Medium","Low")))</f>
+        <v>Medium</v>
+      </c>
+      <c r="H29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-005 remains the status-transition authority; every change to a transition used by accepted, rejected or completed notifications must review ADR-008 and the FR-029 mapping before merge.</t>
+        </is>
+      </c>
+      <c r="I29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stop release of the affected workflow change, correct the notification mapping and tests or evidence, and re-review the affected ADR and RTM references before continuing.</t>
+        </is>
+      </c>
+      <c r="J29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tristan Roets</t>
+        </is>
+      </c>
+      <c r="K29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="L29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-008, ADR-005, FR-029, #63, #68</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RSK-28</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Derived notification queries become inefficient as request history grows.</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 derives notifications from RequestStatusHistory and requester-visible ActionEntry evidence rather than using a dedicated notification read model or Notification table.</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F30" s="13" t="n">
+        <f aca="false">D30*E30</f>
+        <v>6</v>
+      </c>
+      <c r="G30" s="13" t="str">
+        <f aca="false">IF(F30&gt;=20,"Critical",IF(F30&gt;=12,"High",IF(F30&gt;=6,"Medium","Low")))</f>
+        <v>Medium</v>
+      </c>
+      <c r="H30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-007 owns indexes and query measurement; measure the notification query path as data volume grows and keep requester-scoped queries indexed.</t>
+        </is>
+      </c>
+      <c r="I30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If measured evidence shows the derived-query path is inadequate, introduce a dedicated notification read model or persisted Notification entity through a controlled persistence and interface decision.</t>
+        </is>
+      </c>
+      <c r="J30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tristan Roets</t>
+        </is>
+      </c>
+      <c r="K30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="L30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-008, ADR-007, FR-029, #63, #68</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RSK-29</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">External notification delivery is added without durable retry and idempotency behaviour.</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Email, SMS or another asynchronous delivery path is introduced from the M2 in-process interface without first defining persistence, retries, duplicate handling, secrets and operational monitoring.</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F31" s="11" t="n">
+        <f aca="false">D31*E31</f>
+        <v>8</v>
+      </c>
+      <c r="G31" s="11" t="str">
+        <f aca="false">IF(F31&gt;=20,"Critical",IF(F31&gt;=12,"High",IF(F31&gt;=6,"Medium","Low")))</f>
+        <v>Medium</v>
+      </c>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Keep SC-D-01 deferred. Reopening external delivery requires a follow-up interface and deployment decision covering persistence, retries, duplicates, secrets and monitoring before implementation.</t>
+        </is>
+      </c>
+      <c r="I31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Disable the external delivery path, retain the in-application persisted-evidence notification behaviour, and redesign the external path with durable retry and idempotency controls before re-enabling it.</t>
+        </is>
+      </c>
+      <c r="J31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tristan Roets</t>
+        </is>
+      </c>
+      <c r="K31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="L31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-008, SC-D-01, FEC-03, ADR-001 rule 4, #63, #68</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L25"/>
+  <autoFilter ref="A2:L31"/>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs: record ADR-005 to ADR-008 as decided in the registers and the ADRs (#105)
#97 (ADR-007) and #98 (ADR-008) merged on 30 September 2026, so the registers and the ADR files are
brought up to date. DEC-011 and DEC-015 are Decided, following the ADRs as merged. The Decision Log's
risk pointers name RSK-16 to RSK-29. 49 RTM cells cite ADR-007 and ADR-008 as decided and record
what review settled, and NFR-007 records #87 as merged. FEC-03 cites ADR-008 as decided. ADR-005 to
ADR-008 are marked Accepted with their approvals, each naming its Decision Log entry.

Refs: #58, #63, #54, DEC-011, DEC-015
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -4386,7 +4386,7 @@
       </c>
       <c r="J10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2 (28 September 2026, ADR-002): Two proposed under #68: Prisma version drift, and duplicate scheduled jobs if more than one instance runs node-cron. RSK-12 materialised on 28 September 2026 (Prisma issue #30295) and is re-scored in the Risk Register.
+          <t xml:space="preserve">M2 (28 September 2026, ADR-002): RSK-25 Prisma version drift and RSK-26 duplicate scheduled jobs if more than one instance runs node-cron. RSK-12 materialised on 28 September 2026 (Prisma issue #30295) and is re-scored in the Risk Register.
 M1 baseline: Deferring past M2 would begin to constrain construction time. The decision point is the start of M2.</t>
         </is>
       </c>
@@ -4454,7 +4454,7 @@
       </c>
       <c r="J11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2 (23 September 2026, ADR-001): Two risks proposed to the Risk Register under #68: module boundaries eroding under schedule pressure (related to RSK-01 and CON-02), and reporting growth degrading the staff queue before it is measured (FEC-06, related to NFR-001 and RSK-09). DEC-008 (#59) and DEC-010 (#60) are taken against this decision, which answers the M1 risk below.
+          <t xml:space="preserve">M2 (23 September 2026, ADR-001): Two risks, recorded under #68: RSK-24 module boundaries eroding under schedule pressure (related to RSK-01 and CON-02), and RSK-18 reporting load degrading the staff queue (FEC-06, related to NFR-001 and RSK-09). DEC-008 (#59) and DEC-010 (#60) are taken against this decision, which answers the M1 risk below.
 M1 baseline: The choice interacts with DEC-008 and DEC-010; deciding any one in isolation constrains the other two.</t>
         </is>
       </c>
@@ -4509,7 +4509,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="128.52" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="151.88" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
         <v>728</v>
       </c>
@@ -4518,61 +4518,61 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed (M2, ADR-007 under review in #97)
+          <t xml:space="preserve">Decided (M2, ADR-007, merged under #97 on 30 September 2026)
 M1 baseline: DEFERRED to M2</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2 (28 September 2026, ADR-007, proposed): ADR-007 designs the data model for FR-005 to FR-009, FR-012 and FR-025 over the one relational store ADR-001 fixed, carrying the A2 Task 2 findings on reference generation, transactions and validation.
+          <t xml:space="preserve">M2 (30 September 2026, ADR-007): ADR-007 designs the data model for FR-005 to FR-009, FR-012 and FR-025 over the one relational store ADR-001 fixed, carrying the A2 Task 2 findings on reference generation, transactions and validation.
 M1 baseline: The data model must express FR-012 record isolation, FR-025 audit immutability and the FEC-01 authorisation scope, which are baselined here but not yet designed.</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2 (28 September 2026, ADR-007, proposed): CON-05 security; NFR-001 performance; NFR-011 auditability. Drivers ASR-01, ASR-02 and ASR-03 (#56).
+          <t xml:space="preserve">M2 (30 September 2026, ADR-007): CON-05 security; NFR-001 performance; NFR-011 auditability. Drivers ASR-01, ASR-02 and ASR-03 (#56).
 M1 baseline: CON-05 security; NFR-001 performance; NFR-011 auditability.</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2 (28 September 2026, ADR-007, proposed): ADR-001 and DEC-008 already fix one relational PostgreSQL store, so ADR-007 justifies the relational model and records no alternative store. Within it, a database sequence for the reference against reading the current maximum (A2 Task 2).
+          <t xml:space="preserve">M2 (30 September 2026, ADR-007): ADR-001 and DEC-008 fix one relational PostgreSQL store. Within it, ADR-007 compared: reading the current maximum for the next reference against a database sequence (A2 Task 2); audit evidence in the status history alone against a structured AuditEntry; action entries inside the audit trail against their own entity.
 M1 baseline: Not yet evaluated.</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2 (28 September 2026, ADR-007, proposed): PostgreSQL as the system of record, with User, Category, UserCategory, Request, RequestStatusHistory and AuditEntry. References from a database sequence with a unique constraint. Creation and each status change in one transaction. Validation in the interface, service and database. Users and categories deactivated, not deleted.
+          <t xml:space="preserve">M2 (30 September 2026, ADR-007): PostgreSQL as the system of record, with prisma/schema.prisma as the authoritative model and User, Category, UserCategory, Request, ActionEntry, RequestStatusHistory and AuditEntry. References from a database sequence with a unique constraint. Creation and each status, assignee or priority change in one transaction, with one AuditEntry per change. Validation in the interface, service and database. Users and categories deactivated, not deleted.
 M1 baseline: Deliberately not decided.</t>
         </is>
       </c>
       <c r="H13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2 (28 September 2026, ADR-007, proposed): The data is strongly related, and the main reads filter by requester, category, status, assignee and date, which foreign keys, constraints, indexes and transactions serve directly. Field names match the scope conditions in ADR-006.
+          <t xml:space="preserve">M2 (30 September 2026, ADR-007): The data is strongly related, and the main reads filter by requester, category, status, assignee and date, which foreign keys, constraints, indexes and transactions serve directly. Field names match the scope conditions in ADR-006.
 M1 baseline: Schema design is explicitly outside M1 (M1 brief, s5). The requirements it must satisfy are inside M1, and are recorded here.</t>
         </is>
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2 (28 September 2026, ADR-007, proposed): Reference numbers can have gaps after a failed transaction. Reporting shares the transactional store (FEC-06). Status is held on the Request and in its history. Relational schema changes are more controlled.
+          <t xml:space="preserve">M2 (30 September 2026, ADR-007): Reference numbers can have gaps after a failed transaction. Reporting shares the transactional store (FEC-06). Status is held on the Request and in its history. Relational schema changes are more controlled.
 M1 baseline: None while requirements work continues.</t>
         </is>
       </c>
       <c r="J13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2 (28 September 2026, ADR-007, proposed): Four in ADR-007, proposed under #68: reporting load on the queue, a query bypassing the authorisation scope, audit or history inconsistent with request state, and a backup that cannot restore.
+          <t xml:space="preserve">M2 (30 September 2026, ADR-007): Seven in ADR-007, recorded as RSK-17 to RSK-23: a query bypassing the scope, reporting load, audit inconsistent with state, a backup that cannot restore, Prisma and SQL drifting apart, urgency confused with priority, and an internal action entry disclosed.
 M1 baseline: This is the longest-lived commitment in the system, because data outlives the application. FEC-01, FEC-02 and FEC-06 all constrain it.</t>
         </is>
       </c>
       <c r="K13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2 (28 September 2026, ADR-007, proposed): ADR-007 and docs/data/initial-schema.sql (#97). Review on #97 requested the FR-005 location and urgency fields, action entries (FR-017), previous and new values (FR-025), and which of the SQL and the Prisma schema is authoritative.
+          <t xml:space="preserve">M2 (30 September 2026, ADR-007): ADR-007 and docs/data/initial-schema.sql (#97, merged 30 September 2026), revised through review: location and reported urgency, ActionEntry as its own entity, previous and new values in AuditEntry, and prisma/schema.prisma as the authoritative model.
 M1 baseline: Evidence still required: the outcome of DEC-008; expected volume and retention from the organisation (FEC-06); the final record-level scope decision (FEC-01).</t>
         </is>
       </c>
       <c r="L13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2 (28 September 2026, ADR-007, proposed): #65 implements against it. DEC-010 supplies hosting, backup and restore. FEC-06 or the NFR-001 measurement reopens the reporting path.
+          <t xml:space="preserve">M2 (30 September 2026, ADR-007): #65 implements against it. DEC-010 supplies hosting, backup and restore. FEC-06 or the NFR-001 measurement reopens the reporting path.
 M1 baseline: Constrains every later change to reporting, authorisation and migration.</t>
         </is>
       </c>
@@ -4663,7 +4663,7 @@
       </c>
       <c r="J15" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">One proposed under #68: the table and the register drift apart if the register changes without the fixture being re-exported (related to RSK-09).</t>
+          <t xml:space="preserve">RSK-16: the table and the register drift apart if the register changes without the fixture being re-exported (related to RSK-09).</t>
         </is>
       </c>
       <c r="K15" s="9" t="inlineStr">
@@ -4725,7 +4725,7 @@
       </c>
       <c r="J16" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">One proposed under #68: an unscoped query leaks records (related to RSK-05 and FEC-01). Four Access Matrix cells conflict with the requirements; the policy denies them and CR-002 (#92) takes them to change control.</t>
+          <t xml:space="preserve">RSK-17: an unscoped query leaks records (related to RSK-05 and FEC-01). Four Access Matrix cells conflict with the requirements; the policy denies them and CR-002 (#92) takes them to change control.</t>
         </is>
       </c>
       <c r="K16" s="10" t="inlineStr">
@@ -4739,7 +4739,7 @@
         </is>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="58.42" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">DEC-015</t>
@@ -4752,7 +4752,7 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed (M2, ADR-008 under review in #98)</t>
+          <t xml:space="preserve">Decided (M2, ADR-008, merged under #98 on 30 September 2026)</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
@@ -4767,32 +4767,32 @@
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">(a) An in-process interface. (b) An HTTP API between the modules. (c) A message broker or a separate notification service.</t>
+          <t xml:space="preserve">(a) Indications derived from persisted status history and requester-visible action entries. (b) A separate Notification table. (c) An external notification service or message broker.</t>
         </is>
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Option (a): the workflow calls the notification interface after a status change commits. Email and SMS stay deferred under SC-D-01.</t>
+          <t xml:space="preserve">Option (a), in process under ADR-001 rule 4. FR-029's four indications are derived from RequestStatusHistory and requester-visible ActionEntry rows, with no separate notification store. Email and SMS stay deferred under SC-D-01.</t>
         </is>
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Both ends are modules in one process, so a network boundary or a broker would add failure handling and deployment work without a requirement for it.</t>
+          <t xml:space="preserve">Both ends are modules in one process, and the evidence FR-029 needs is already persisted, so a separate store or a network boundary would add state and failure handling without a requirement for it. Indications survive the next sign-in with no separate write to fail.</t>
         </is>
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">No independent scaling and no durable asynchronous delivery. A window in which a status change commits and the notification fails.</t>
+          <t xml:space="preserve">Every notification read maps history and action entries into indications. No independent scaling or buffering of notification work. No external channel in M2.</t>
         </is>
       </c>
       <c r="J17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Five in ADR-008, proposed under #68.</t>
+          <t xml:space="preserve">Four in ADR-008, recorded as RSK-27 (mapping drifts from the workflow), RSK-23 (an internal entry disclosed), RSK-28 (derived queries slow as history grows) and RSK-29 (external delivery without retry and idempotency).</t>
         </is>
       </c>
       <c r="K17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADR-008 (#98). Review on #98 requested which FR-029 events produce an indication, and where the indication is stored.</t>
+          <t xml:space="preserve">ADR-008 (#98, merged 30 September 2026), with the FR-029 event mapping, security boundary, versioning and the conditions that reopen SC-D-01.</t>
         </is>
       </c>
       <c r="L17" s="9" t="inlineStr">
@@ -9319,7 +9319,7 @@
       </c>
       <c r="I3" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): User, with a unique email and an active flag. Credential storage not yet designed</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): User, with a unique email and an active flag. Credential storage not yet designed</t>
         </is>
       </c>
       <c r="J3" s="9" t="inlineStr">
@@ -9382,7 +9382,7 @@
       </c>
       <c r="I4" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): User.role and UserCategory</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): User.role and UserCategory</t>
         </is>
       </c>
       <c r="J4" s="10" t="inlineStr">
@@ -9445,7 +9445,7 @@
       </c>
       <c r="I5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): User.role, one role per user</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): User.role, one role per user</t>
         </is>
       </c>
       <c r="J5" s="9" t="inlineStr">
@@ -9470,7 +9470,7 @@
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADR-007 (proposed)</t>
+          <t xml:space="preserve">ADR-007</t>
         </is>
       </c>
       <c r="O5" s="9" t="s">
@@ -9571,7 +9571,7 @@
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Request. Location and reported urgency were requested on review of #97</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): Request, with location and reportedUrgency held apart from priority</t>
         </is>
       </c>
       <c r="J7" s="9" t="inlineStr">
@@ -9596,7 +9596,7 @@
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADR-007 (proposed)</t>
+          <t xml:space="preserve">ADR-007</t>
         </is>
       </c>
       <c r="O7" s="9" t="s">
@@ -9634,7 +9634,7 @@
       </c>
       <c r="I8" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Category with an active flag, referenced by a foreign key</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): Category with an active flag, referenced by a foreign key</t>
         </is>
       </c>
       <c r="J8" s="10" t="inlineStr">
@@ -9659,7 +9659,7 @@
       </c>
       <c r="N8" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">FEC-02, ADR-007 (proposed)</t>
+          <t xml:space="preserve">FEC-02, ADR-007</t>
         </is>
       </c>
       <c r="O8" s="10" t="s">
@@ -9697,12 +9697,12 @@
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Not-null and foreign-key constraints behind service validation</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): Not-null and foreign-key constraints behind service validation</t>
         </is>
       </c>
       <c r="J9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADR-007 (proposed): validation divided across interface, service and database (A2 Task 2)</t>
+          <t xml:space="preserve">ADR-007: validation divided across interface, service and database (A2 Task 2)</t>
         </is>
       </c>
       <c r="K9" s="9" t="inlineStr">
@@ -9722,7 +9722,7 @@
       </c>
       <c r="N9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADR-007 (proposed)</t>
+          <t xml:space="preserve">ADR-007</t>
         </is>
       </c>
       <c r="O9" s="9" t="s">
@@ -9760,12 +9760,12 @@
       </c>
       <c r="I10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Reference from a database sequence with a unique constraint. Gaps after a failed transaction are accepted</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): Reference from a database sequence with a unique constraint. Gaps after a failed transaction are accepted</t>
         </is>
       </c>
       <c r="J10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADR-007 (proposed): database-native atomic sequence (A2 Task 2)</t>
+          <t xml:space="preserve">ADR-007: database-native atomic sequence (A2 Task 2)</t>
         </is>
       </c>
       <c r="K10" s="10" t="inlineStr">
@@ -9785,7 +9785,7 @@
       </c>
       <c r="N10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEC-004, ADR-007 (proposed)</t>
+          <t xml:space="preserve">DEC-004, ADR-007</t>
         </is>
       </c>
       <c r="O10" s="10" t="s">
@@ -9823,7 +9823,7 @@
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Request.reference and createdAt, committed in the creation transaction</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): Request.reference and createdAt, committed in the creation transaction</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr">
@@ -9848,7 +9848,7 @@
       </c>
       <c r="N11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADR-007 (proposed)</t>
+          <t xml:space="preserve">ADR-007</t>
         </is>
       </c>
       <c r="O11" s="9" t="s">
@@ -9886,7 +9886,7 @@
       </c>
       <c r="I12" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Request fields and updatedAt, indexed on requesterId</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): Request fields and updatedAt, indexed on requesterId</t>
         </is>
       </c>
       <c r="J12" s="10" t="inlineStr">
@@ -9949,7 +9949,7 @@
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Status history, and visibility on entries. Action entries as their own entity were requested on review of #97</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): Status history, and ActionEntry with an explicit visibility</t>
         </is>
       </c>
       <c r="J13" s="9" t="inlineStr">
@@ -10012,7 +10012,7 @@
       </c>
       <c r="I14" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): requesterId, the field the scope condition filters</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): requesterId, the field the scope condition filters</t>
         </is>
       </c>
       <c r="J14" s="10" t="inlineStr">
@@ -10075,7 +10075,7 @@
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): categoryId and UserCategory, indexed on category and status</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): categoryId and UserCategory, indexed on category and status</t>
         </is>
       </c>
       <c r="J15" s="9" t="inlineStr">
@@ -10138,7 +10138,7 @@
       </c>
       <c r="I16" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Indexes on status, category, assignee and createdAt. Keyword search not yet designed</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): Indexes on status, category, assignee and createdAt. Keyword search not yet designed</t>
         </is>
       </c>
       <c r="J16" s="10" t="inlineStr">
@@ -10163,7 +10163,7 @@
       </c>
       <c r="N16" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">FEC-06, ADR-007 (proposed)</t>
+          <t xml:space="preserve">FEC-06, ADR-007</t>
         </is>
       </c>
       <c r="O16" s="10" t="s">
@@ -10201,7 +10201,7 @@
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): assigneeId on Request</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): assigneeId on Request</t>
         </is>
       </c>
       <c r="J17" s="9" t="inlineStr">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="I18" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Request.status and a RequestStatusHistory row, written in one transaction (ADR-001 rule 3)</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): Request.status, a RequestStatusHistory row and one AuditEntry, written in one transaction (ADR-001 rule 3)</t>
         </is>
       </c>
       <c r="J18" s="10" t="inlineStr">
@@ -10327,7 +10327,7 @@
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Visibility on entries, required with no default. Action entries as their own entity were requested on review of #97</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): ActionEntry, whose visibility is required with no default and limited to internal or requester-visible</t>
         </is>
       </c>
       <c r="J19" s="9" t="inlineStr">
@@ -10390,7 +10390,7 @@
       </c>
       <c r="I20" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Where the resolution summary is stored was requested on review of #97</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): resolutionSummary on Request, shown to the Requester once recorded</t>
         </is>
       </c>
       <c r="J20" s="10" t="inlineStr">
@@ -10453,7 +10453,7 @@
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Status history</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): Status history</t>
         </is>
       </c>
       <c r="J21" s="9" t="inlineStr">
@@ -10516,7 +10516,7 @@
       </c>
       <c r="I22" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Rejection reason stored on the status-history row</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): Rejection reason stored on the status-history row</t>
         </is>
       </c>
       <c r="J22" s="10" t="inlineStr">
@@ -10579,7 +10579,7 @@
       </c>
       <c r="I23" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Priority nullable until set. Reported urgency as a separate field was requested on review of #97</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): Priority nullable until set, and reportedUrgency as a separate field staff cannot edit</t>
         </is>
       </c>
       <c r="J23" s="9" t="inlineStr">
@@ -10831,7 +10831,7 @@
       </c>
       <c r="I27" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): AuditEntry. Previous and new values were requested on review of #97</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): AuditEntry with the field changed, the previous value and the new value, one per change</t>
         </is>
       </c>
       <c r="J27" s="9" t="inlineStr">
@@ -10856,7 +10856,7 @@
       </c>
       <c r="N27" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADR-001, ADR-007 (proposed)</t>
+          <t xml:space="preserve">ADR-001, ADR-007</t>
         </is>
       </c>
       <c r="O27" s="9" t="s">
@@ -10894,7 +10894,7 @@
       </c>
       <c r="I28" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Append-only. No update or delete through the application</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): Append-only. No update or delete through the application</t>
         </is>
       </c>
       <c r="J28" s="10" t="inlineStr">
@@ -10957,7 +10957,7 @@
       </c>
       <c r="I29" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Category active flag. Categories are deactivated, not deleted</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): Category active flag. Categories are deactivated, not deleted</t>
         </is>
       </c>
       <c r="J29" s="9" t="inlineStr">
@@ -10982,7 +10982,7 @@
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADR-007 (proposed)</t>
+          <t xml:space="preserve">ADR-007</t>
         </is>
       </c>
       <c r="O29" s="9" t="s">
@@ -11020,7 +11020,7 @@
       </c>
       <c r="I30" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): User active flag</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): User active flag</t>
         </is>
       </c>
       <c r="J30" s="10" t="inlineStr">
@@ -11045,7 +11045,7 @@
       </c>
       <c r="N30" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADR-007 (proposed)</t>
+          <t xml:space="preserve">ADR-007</t>
         </is>
       </c>
       <c r="O30" s="10" t="s">
@@ -11083,12 +11083,12 @@
       </c>
       <c r="I31" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet designed. Where the indication is stored was requested on review of #98</t>
+          <t xml:space="preserve">Derived from RequestStatusHistory and requester-visible ActionEntry rows, with no separate store (ADR-008)</t>
         </is>
       </c>
       <c r="J31" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-008 (DEC-015, #98, under review): in-process notification interface</t>
+          <t xml:space="preserve">ADR-008 (DEC-015, #98): in-process interface, with indications derived from persisted evidence</t>
         </is>
       </c>
       <c r="K31" s="9" t="inlineStr">
@@ -11108,7 +11108,7 @@
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEC-005, SC-D-01, FEC-03, ADR-008 (proposed)</t>
+          <t xml:space="preserve">DEC-005, SC-D-01, FEC-03, ADR-008</t>
         </is>
       </c>
       <c r="O31" s="9" t="s">
@@ -11146,7 +11146,7 @@
       </c>
       <c r="I32" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Indexes on the queue and scope fields. Reporting shares the store</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): Indexes on the queue and scope fields. Reporting shares the store</t>
         </is>
       </c>
       <c r="J32" s="10" t="inlineStr">
@@ -11209,12 +11209,12 @@
       </c>
       <c r="I33" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Creation committed in one transaction</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): Creation committed in one transaction</t>
         </is>
       </c>
       <c r="J33" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADR-007 (proposed): one creation transaction</t>
+          <t xml:space="preserve">ADR-007: one creation transaction</t>
         </is>
       </c>
       <c r="K33" s="9" t="inlineStr">
@@ -11234,7 +11234,7 @@
       </c>
       <c r="N33" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADR-007 (proposed)</t>
+          <t xml:space="preserve">ADR-007</t>
         </is>
       </c>
       <c r="O33" s="9" t="s">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="I36" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): The fields the scope conditions filter: requesterId, categoryId and visibility</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): The fields the scope conditions filter: requesterId, categoryId and visibility</t>
         </is>
       </c>
       <c r="J36" s="10" t="inlineStr">
@@ -11493,7 +11493,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="35.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="47.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
         <v>449</v>
       </c>
@@ -11534,17 +11534,17 @@
       </c>
       <c r="K38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gitleaks workflow proposed in #87</t>
+          <t xml:space="preserve">Gitleaks workflow (#87, merged)</t>
         </is>
       </c>
       <c r="L38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gitleaks workflow in #87, open. It ran on #87 on 29 September 2026 and passed</t>
+          <t xml:space="preserve">Gitleaks workflow (#87), merged on 30 September 2026</t>
         </is>
       </c>
       <c r="M38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Secret scan run on #87 (29 September 2026): 2 commits scanned, no leaks found. Runs on every pull request once #87 merges</t>
+          <t xml:space="preserve">The secret scan runs on every pull request and push to main. It passed on #87 on 29 September 2026 and on main on 30 September 2026</t>
         </is>
       </c>
       <c r="N38" s="10" t="inlineStr">
@@ -11587,7 +11587,7 @@
       </c>
       <c r="I39" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Only the fields the requirements need, read through policy-scoped queries</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): Only the fields the requirements need, read through policy-scoped queries</t>
         </is>
       </c>
       <c r="J39" s="9" t="inlineStr">
@@ -11776,7 +11776,7 @@
       </c>
       <c r="I42" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, ADR-007 (#97, under review): Status and history written in one transaction. Previous and new values in the audit entry were requested on review of #97</t>
+          <t xml:space="preserve">ADR-007 (DEC-011, #97): Status, history and one AuditEntry with the previous and new values, written in one transaction</t>
         </is>
       </c>
       <c r="J42" s="10" t="inlineStr">
@@ -13556,7 +13556,7 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2 (29 September 2026): Still open. ADR-008 (#98, under review) keeps the M2 notification path in-process and leaves asynchronous delivery deferred. DEC-010 (#60) has still to establish platform support for background processing.
+          <t xml:space="preserve">M2 (29 September 2026): Still open. ADR-008 (#98) keeps the M2 notification path in-process and leaves asynchronous delivery deferred. DEC-010 (#60) has still to establish platform support for background processing.
 M1 baseline: The background-process, scheduled-job and idle-timeout limits of each candidate platform within free-tier terms.</t>
         </is>
       </c>

</xml_diff>

<commit_message>
docs: record the M1 and M2 sign-off decisions in the registers
All three members answered the sign-off points on #69 on 30 September 2026, alike.

Baseline Sign-off: the M1 sign-off of PED v1.0, conditionally accepted, with its six checks, the
conditions #27, #36, #37, #47 and #48, and the three approvals, dated after the M1 submission. The
assessor's field is marked for the assessor. The M2 sign-off is recorded in PED s26.3.

Change Requests: CR-001, CR-002 and CR-003 approved by all three members. CR-002 corrects the
Access Matrix to the requirements for all four cells; the correction itself is M3 work under #92.

Risk Register: RSK-12's probability of 3 confirmed by its owner, Darius Mushi.

Only the Baseline Sign-off, Change Requests and Risk Register sheet parts change; the other 58
parts are byte-identical, and both cell comments are kept.

Refs: #69, #7, #92, RSK-12
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -6092,7 +6092,7 @@
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending the M2 baseline sign-off (#69).</t>
+          <t xml:space="preserve">Approved by all three members on #69, 30 September 2026.</t>
         </is>
       </c>
     </row>
@@ -6169,12 +6169,12 @@
       </c>
       <c r="O4" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACCEPT, correcting the matrix. The alternative, changing the Status Model and FR-021 to match the matrix, is the larger change and affects ADR-005.</t>
+          <t xml:space="preserve">ACCEPT, correcting the matrix to the requirements for all four cells. The correction of the Access Matrix sheet, PED s8.3 and the test fixture is M3 work under #92.</t>
         </is>
       </c>
       <c r="P4" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending the team decision at the M2 baseline sign-off (#69).</t>
+          <t xml:space="preserve">Approved by all three members on #69, 30 September 2026: fix the matrix for all four cells.</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending the M2 baseline sign-off (#69).</t>
+          <t xml:space="preserve">Approved by all three members on #69, 30 September 2026.</t>
         </is>
       </c>
     </row>
@@ -7186,104 +7186,130 @@
       <c r="A7" s="9" t="s">
         <v>749</v>
       </c>
-      <c r="B7" s="12" t="s">
-        <v>922</v>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30 September 2026, after the M1 submission. Answers recorded on #69</t>
+        </is>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
         <v>923</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>924</v>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
         <v>925</v>
       </c>
-      <c r="B9" s="9" t="s">
-        <v>924</v>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
         <v>926</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>924</v>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
         <v>927</v>
       </c>
-      <c r="B11" s="9" t="s">
-        <v>924</v>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES, noting #37 and #47</t>
+        </is>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
         <v>928</v>
       </c>
-      <c r="B12" s="10" t="s">
-        <v>924</v>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
         <v>929</v>
       </c>
-      <c r="B13" s="9" t="s">
-        <v>924</v>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
         <v>930</v>
       </c>
-      <c r="B14" s="10" t="s">
-        <v>931</v>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONDITIONALLY ACCEPTED</t>
+        </is>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
         <v>932</v>
       </c>
-      <c r="B15" s="12" t="s">
-        <v>933</v>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#27 the Figure 2 label defect; #36 figure sources not held in the repository; #37 branch naming breached on five branches; #47 checks required before any existed; #48 PED s12.4 narrower than Master Brief s14. Each is carried in PED s26.2.</t>
+        </is>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
         <v>1033</v>
       </c>
-      <c r="B16" s="10" t="s">
-        <v>935</v>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Approved, 30 September 2026 (#69)</t>
+        </is>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
         <v>1034</v>
       </c>
-      <c r="B17" s="9" t="s">
-        <v>935</v>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Approved, 30 September 2026 (#69)</t>
+        </is>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
         <v>1035</v>
       </c>
-      <c r="B18" s="10" t="s">
-        <v>935</v>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Approved, 30 September 2026 (#69)</t>
+        </is>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
         <v>938</v>
       </c>
-      <c r="B19" s="12" t="s">
-        <v>933</v>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For the assessor to complete</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -12509,7 +12535,7 @@
       </c>
       <c r="K14" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2 (29 September 2026): Materialised - active. Prisma 7.10.0 pins deepmerge-ts 7.1.5 and mysql2 3.15.3, which carry high-severity advisories no 7.x release has fixed (Prisma issue #30295, found 28 September 2026). Probability re-scored from 2 to 3 under #68, for the owner to confirm.
+          <t xml:space="preserve">M2 (29 September 2026): Materialised - active. Prisma 7.10.0 pins deepmerge-ts 7.1.5 and mysql2 3.15.3, which carry high-severity advisories no 7.x release has fixed (Prisma issue #30295, found 28 September 2026). Probability re-scored from 2 to 3 under #68, confirmed by the owner on #69, 30 September 2026.
 M1 baseline: Open</t>
         </is>
       </c>

</xml_diff>

<commit_message>
docs(#107): CR-004, amend ADR-002's merge conditions for the bootstrap
Neither ADR-002 condition could be shown as met: the two verification logs
on #64 disagree, and the #90 proof of concept persisted to a temporary
table outside the data model. CR-004 replaces the campus run with a check a
second member repeats on Node 24 against PostgreSQL 16, then CI on every
pull request (#110), and restates the proof of concept against the ADR-007
User entity.

- ADR-002: dated Amendment section; the original conditions stay
- Change Requests: CR-004
- Decision Log: DEC-016
- Risk Register: RSK-30, the unverified campus environment (3 x 3, Medium)
- README: Medium risks 17 to 18, decisions recorded 15 to 16

Workbook edited at byte level: README, Risk Register, Decision Log, Change
Requests and the workbook filter ranges change; every other part is
byte-identical. Recalculated in Excel with no exposure mismatches.
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -30,14 +30,14 @@
     <definedName function="false" hidden="true" localSheetId="13" name="_xlnm._FilterDatabase" vbProcedure="false">'Access Matrix'!$A$2:$E$17</definedName>
     <definedName function="false" hidden="true" localSheetId="10" name="_xlnm._FilterDatabase" vbProcedure="false">'AI Usage Register'!$A$2:$H$29</definedName>
     <definedName function="false" hidden="true" localSheetId="16" name="_xlnm._FilterDatabase" vbProcedure="false">'Baseline Sign-off'!$A$2:$B$19</definedName>
-    <definedName function="false" hidden="true" localSheetId="11" name="_xlnm._FilterDatabase" vbProcedure="false">'Change Requests'!$A$2:$P$5</definedName>
+    <definedName function="false" hidden="true" localSheetId="11" name="_xlnm._FilterDatabase" vbProcedure="false">'Change Requests'!$A$2:$P$6</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">Constraints!$A$2:$D$10</definedName>
-    <definedName function="false" hidden="true" localSheetId="9" name="_xlnm._FilterDatabase" vbProcedure="false">'Decision Log'!$A$2:$L$17</definedName>
+    <definedName function="false" hidden="true" localSheetId="9" name="_xlnm._FilterDatabase" vbProcedure="false">'Decision Log'!$A$2:$L$18</definedName>
     <definedName function="false" hidden="true" localSheetId="8" name="_xlnm._FilterDatabase" vbProcedure="false">'Forward Considerations'!$A$2:$G$9</definedName>
     <definedName function="false" hidden="true" localSheetId="15" name="_xlnm._FilterDatabase" vbProcedure="false">'GitHub Governance'!$A$2:$C$14</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Requirements (FR)'!$A$2:$F$31</definedName>
     <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">'Requirements (NFR)'!$A$2:$G$15</definedName>
-    <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">'Risk Register'!$A$2:$L$31</definedName>
+    <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">'Risk Register'!$A$2:$L$32</definedName>
     <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">RTM!$A$2:$O$44</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Scope Baseline'!$A$2:$E$27</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Stakeholders!$A$2:$G$11</definedName>
@@ -3943,7 +3943,7 @@
       </c>
       <c r="B23" s="6" t="n">
         <f aca="false">COUNTIF('Risk Register'!G3:G200,"Medium")</f>
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3970,7 +3970,7 @@
       </c>
       <c r="B26" s="6" t="n">
         <f aca="false">COUNTA('Decision Log'!A3:A200)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3998,7 +3998,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -4801,8 +4801,70 @@
         </is>
       </c>
     </row>
+    <row r="18" customFormat="false" ht="70.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEC-016</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bootstrap merge conditions, amending DEC-008</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decided (M3, CR-004, #107)</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-002 (DEC-008) let the bootstrap (#90) merge only after gate 3 closed on a BC Desktop machine and the RSK-01 proof of concept passed. By 5 October 2026 neither was shown: the verification logs on #64 disagree, and the proof of concept persisted to a temporary table. Every M3 implementation issue depends on the bootstrap.</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CON-07 platform availability; CON-02 schedule, with M3 due 14 October 2026; RSK-01; NFR-004.</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(a) Keep both conditions and wait for a verified campus run. (b) Replace the campus run with a check a second member repeats and CI then runs on every pull request, keep the campus check as a risk, and restate the proof of concept against the data model. (c) Remove the conditions.</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(b), recorded as CR-004 and as a dated amendment to ADR-002.</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A check another member can repeat, and that CI then repeats on every pull request, is stronger evidence than a single run nobody else can see. (a) holds all of M3 on lab access the team does not control. (c) drops the evidence ADR-002 asked for.</t>
+        </is>
+      </c>
+      <c r="I18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No verified run on the campus image before construction starts, so the campus environment can still differ.</t>
+        </is>
+      </c>
+      <c r="J18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RSK-30: the campus environment differs from the verified Node 24 and PostgreSQL 16 environment.</t>
+        </is>
+      </c>
+      <c r="K18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The #64 verification logs (30 September 2026); the reviews on #90; CR-004 and the ADR-002 amendment (#107).</t>
+        </is>
+      </c>
+      <c r="L18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#90 merges under #108 once the second member's run is posted. The CI workflow (#110) repeats the check on every pull request. The campus check is run when lab access allows and recorded on #64.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L17"/>
+  <autoFilter ref="A2:L18"/>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>
@@ -5932,7 +5994,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -6260,8 +6322,90 @@
         </is>
       </c>
     </row>
+    <row r="6" customFormat="false" ht="202.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR-004</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jean Smit</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 October 2026</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Amend the two conditions ADR-002 sets before the bootstrap (#90) merges (#107). Condition 1, gate 3 on a BC Desktop machine, becomes a reproducible check: a member other than the author runs npm ci, prisma generate, prisma migrate deploy and npm test on Node 24 against PostgreSQL 16 and posts the output on #90, and the CI workflow repeats it on every pull request once #110 merges. The campus check becomes RSK-30. Condition 2 is restated: the RSK-01 proof of concept persists a User from the ADR-007 model through Prisma and verifies an argon2 sign-in.</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Neither condition could be shown as met. The two verification logs on #64 disagree: the log with a screenshot ran on a member's own machine on Node 25.9.0 with mock data, and the log that reports a campus run has no screenshot or command output. The proof of concept in #90 persists to a table the test creates and drops, outside the data model. M3 is due 14 October 2026 and every M3 implementation issue depends on the bootstrap.</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None. NFR-004 and the substance of the RSK-01 proof of concept are unchanged.</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-002: the merge conditions under Decision, recorded as a dated amendment. The original conditions stay in the record.</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data: the proof of concept uses the User entity from ADR-007 instead of a temporary table.</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None. The argon2 check is kept.</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The environment check becomes repeatable: a second member's run on #90, then the CI workflow (#110) on every pull request, on Node 24 against PostgreSQL 16.</t>
+        </is>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="L6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unblocks #108, which merges #90 by 7 October 2026, and through it every M3 implementation issue.</t>
+        </is>
+      </c>
+      <c r="M6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="N6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adds RSK-30 for the unverified campus environment. RSK-01 and RSK-02 are unchanged.</t>
+        </is>
+      </c>
+      <c r="O6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ACCEPT</t>
+        </is>
+      </c>
+      <c r="P6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Approved when the pull request for #107 merges with the approvals of the other two members.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:P5"/>
+  <autoFilter ref="A2:P6"/>
   <mergeCells count="1">
     <mergeCell ref="A1:P1"/>
   </mergeCells>
@@ -11981,7 +12125,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -13450,8 +13594,64 @@
         </is>
       </c>
     </row>
+    <row r="32" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RSK-30</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The BC Desktop campus environment differs from the Node 24 and PostgreSQL 16 environment the stack was verified on, so the application does not install or run on campus machines.</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR-004 replaced the campus run with a check repeated by a second member and in CI, because no verified campus run exists (#64). CON-07: the campus cannot guarantee the stack is available.</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F32" s="13" t="n">
+        <f aca="false">D32*E32</f>
+        <v>9</v>
+      </c>
+      <c r="G32" s="13" t="str">
+        <f aca="false">IF(F32&gt;=20,"Critical",IF(F32&gt;=12,"High",IF(F32&gt;=6,"Medium","Low")))</f>
+        <v>Medium</v>
+      </c>
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The engines field requires Node 24 or later; npm ci installs from the committed lockfile; CI runs on Node 24 against PostgreSQL 16 on every pull request (#110). Run the campus check when lab access allows and record the Node version on #64.</t>
+        </is>
+      </c>
+      <c r="I32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Demonstrate from a team member's machine on the simulated staging environment (#122), and record the campus difference as a limitation in the release summary.</t>
+        </is>
+      </c>
+      <c r="J32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Darius Mushi</t>
+        </is>
+      </c>
+      <c r="K32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="L32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-002, CR-004, DEC-016, CON-07, RSK-01, RSK-02, #64, #90, #107</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L31"/>
+  <autoFilter ref="A2:L32"/>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs(#69): remove the unagreed risk-scoring convention from #106
From Darius Mushi's second review (6 October 2026): the README B10 rule
on scoring a risk that has happened is a new team rule, and s12.1 of the
Working Agreement records team decisions in the Decision Log after
consensus. It is taken out of this PR rather than recorded without it:

- README (sheet1) restored byte for byte from main
- RSK-12 K14 no longer cites the convention. It keeps the status
  "Materialised - mitigated" with the evidence, and probability 3 as
  re-scored under #68 and confirmed by the owner on #69. Any other score
  is the owner's decision, to be stated on #106

The rule can come back as a Decision Log entry if all three agree.
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -3828,15 +3828,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="83.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Exposure and Priority on the Risk Register are formulas. Change Probability or Impact and they recalculate. Do not overwrite them with typed values.
-A risk that has happened (#106, 6 October 2026): Status starts with Materialised - active while it is still causing harm, or Materialised - mitigated once a control is in place. Probability then means the likelihood of it happening again or causing further harm, so Exposure shows the risk that remains, not the event itself. RSK-04, RSK-07, RSK-12 and RSK-15 are scored this way.</t>
-        </is>
+      <c r="B10" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12541,7 +12538,7 @@
       </c>
       <c r="K14" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Materialised - mitigated. Found 28 September 2026: Prisma 7.10.0 pins deepmerge-ts 7.1.5 and mysql2 3.15.3, which carry high-severity advisories no 7.x release has fixed (Prisma issue #30295). The bootstrap (#90) overrides them to deepmerge-ts 8.0.2 and mysql2 3.24.4, and npm audit reports 0 vulnerabilities. Probability 3 is the likelihood of it happening again, under the convention in the README (#106); re-scored from 2 under #68 and confirmed by the owner on #69, 30 September 2026.
+          <t xml:space="preserve">Materialised - mitigated. Found 28 September 2026: Prisma 7.10.0 pins deepmerge-ts 7.1.5 and mysql2 3.15.3, which carry high-severity advisories no 7.x release has fixed (Prisma issue #30295). The bootstrap (#90) overrides them to deepmerge-ts 8.0.2 and mysql2 3.24.4, and npm audit reports 0 vulnerabilities. Probability re-scored from 2 to 3 under #68 and confirmed by the owner on #69, 30 September 2026.
 M1 baseline: Open</t>
         </is>
       </c>

</xml_diff>

<commit_message>
docs(#69): answer the third #106 review: RSK-12 active until #90 merges
Risk Register K14: RSK-12 is "Materialised - active". The overrides and the
audit result are described as on the #90 branch, which has not merged
(npm audit 0 at 9529e80 and again at fbd12e9), and the audit gate as arriving
with #110. Probability 3 is cited as confirmed by the owner on #106,
8 October 2026, replacing the #69 reference. H14 describes #90 the same way.

Baseline Sign-off B16 to B18: the approvals are "recorded on #69, not at a
gate review". Change Requests J3: the CR-001 fidelity figures are given at
3b2def7, the conversion commit.

Byte-level edit of the Risk Register, Change Requests and Baseline Sign-off
parts; every other part is unchanged.
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -6062,7 +6062,7 @@
       </c>
       <c r="J3" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">The conversion is checked by a fidelity check: 1504 blocks and 18,169 words identical to v1.0. The build is checked by rebuilding v1.0 and comparing the rendered pages.</t>
+          <t xml:space="preserve">The conversion is checked by a fidelity check: at 3b2def7, 1504 blocks and 18,169 words identical to v1.0. The build is checked by rebuilding v1.0 and comparing the rendered pages.</t>
         </is>
       </c>
       <c r="K3" s="9" t="inlineStr">
@@ -7272,33 +7272,33 @@
         </is>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15.0" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
         <v>1033</v>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Approved, 30 September 2026 (#69)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+          <t xml:space="preserve">Approved, 30 September 2026, recorded on #69, not at a gate review</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15.0" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
         <v>1034</v>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Approved, 30 September 2026 (#69)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+          <t xml:space="preserve">Approved, 30 September 2026, recorded on #69, not at a gate review</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15.0" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
         <v>1035</v>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Approved, 30 September 2026 (#69)</t>
+          <t xml:space="preserve">Approved, 30 September 2026, recorded on #69, not at a gate review</t>
         </is>
       </c>
     </row>
@@ -12497,7 +12497,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="547.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="690.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
         <v>536</v>
       </c>
@@ -12523,7 +12523,7 @@
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2 (29 September 2026): ADR-002 pins every package exactly, with a committed lockfile. #90 overrides deepmerge-ts to 8.0.2 and mysql2 to 3.24.4, and npm audit reports 0 vulnerabilities at 9529e80. The overrides are removed when a Prisma 7 release fixes issue #30295. npm audit --audit-level=high runs on every pull request once the CI workflow (#110) merges, so a new advisory fails the build.
+          <t xml:space="preserve">M2 (29 September 2026): ADR-002 pins every package exactly, with a committed lockfile. On the #90 branch, which has not merged, the bootstrap overrides deepmerge-ts to 8.0.2 and mysql2 to 3.24.4, and npm audit reports 0 vulnerabilities at 9529e80. The overrides are removed when a Prisma 7 release fixes issue #30295. npm audit --audit-level=high runs on every pull request once the CI workflow (#110) merges, so a new advisory fails the build.
 M1 baseline: Make dependency-ecosystem maturity a criterion in DEC-008. Adopt lockfiles and automated dependency and vulnerability checking from the first construction Pull Request. Require any new dependency to be justified in the Pull Request that introduces it.</t>
         </is>
       </c>
@@ -12538,7 +12538,7 @@
       </c>
       <c r="K14" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Materialised - mitigated. Found 28 September 2026: Prisma 7.10.0 pins deepmerge-ts 7.1.5 and mysql2 3.15.3, which carry high-severity advisories no 7.x release has fixed (Prisma issue #30295). The bootstrap (#90) overrides them to deepmerge-ts 8.0.2 and mysql2 3.24.4, and npm audit reports 0 vulnerabilities. Probability re-scored from 2 to 3 under #68 and confirmed by the owner on #69, 30 September 2026.
+          <t xml:space="preserve">Materialised - active. Found 28 September 2026: Prisma 7.10.0 pins deepmerge-ts 7.1.5 and mysql2 3.15.3, which carry high-severity advisories no 7.x release has fixed (Prisma issue #30295). On the #90 branch, which has not merged, the bootstrap overrides them to deepmerge-ts 8.0.2 and mysql2 3.24.4, and npm audit reports 0 vulnerabilities (9529e80; again at fbd12e9 on 9 October 2026). The audit gate arrives once the CI workflow (#110) merges. The status becomes Materialised - mitigated when both have merged. Probability re-scored from 2 to 3 under #68 and confirmed by the owner, Darius Mushi, on #106, 8 October 2026.
 M1 baseline: Open</t>
         </is>
       </c>

</xml_diff>

<commit_message>
docs: record the M1 baseline sign-off decisions in the registers (#106)
Closes #69. Refs #7. The M1 sign-off of PED v1.0 in the Baseline Sign-off sheet, recorded on #69 rather than at a gate review, with the outcome as the team's recommendation and the assessor's decision pending; CR-001 and CR-003 approved, CR-002 approved and not yet implemented; RSK-12 materialised and active until #90 and #110 merge, probability 3 confirmed by its owner. Approved by Darius Mushi and Tristan Roets.
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -6062,7 +6062,7 @@
       </c>
       <c r="J3" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">The conversion is checked by a fidelity check: 1504 blocks and 18,169 words identical to v1.0. The build is checked by rebuilding v1.0 and comparing the rendered pages.</t>
+          <t xml:space="preserve">The conversion is checked by a fidelity check: at 3b2def7, 1504 blocks and 18,169 words identical to v1.0. The build is checked by rebuilding v1.0 and comparing the rendered pages.</t>
         </is>
       </c>
       <c r="K3" s="9" t="inlineStr">
@@ -6092,7 +6092,7 @@
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending the M2 baseline sign-off (#69).</t>
+          <t xml:space="preserve">Approved by all three members on #69, 30 September 2026.</t>
         </is>
       </c>
     </row>
@@ -6169,12 +6169,12 @@
       </c>
       <c r="O4" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACCEPT, correcting the matrix. The alternative, changing the Status Model and FR-021 to match the matrix, is the larger change and affects ADR-005.</t>
+          <t xml:space="preserve">ACCEPT, correcting the matrix to the requirements for all four cells. The correction of the Access Matrix sheet, PED s8.3 and the test fixture is M3 work under #92.</t>
         </is>
       </c>
       <c r="P4" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending the team decision at the M2 baseline sign-off (#69).</t>
+          <t xml:space="preserve">Approved, not implemented. Approved by all three members on #69, 30 September 2026: fix the matrix for all four cells. The Access Matrix sheet, PED s8.3 and the test fixture still show the four cells until #92 corrects them in M3.</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending the M2 baseline sign-off (#69).</t>
+          <t xml:space="preserve">Approved by all three members on #69, 30 September 2026.</t>
         </is>
       </c>
     </row>
@@ -7186,104 +7186,130 @@
       <c r="A7" s="9" t="s">
         <v>749</v>
       </c>
-      <c r="B7" s="12" t="s">
-        <v>922</v>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30 September 2026, after the M1 submission. Answers recorded on #69</t>
+        </is>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
         <v>923</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>924</v>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
         <v>925</v>
       </c>
-      <c r="B9" s="9" t="s">
-        <v>924</v>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
         <v>926</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>924</v>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
         <v>927</v>
       </c>
-      <c r="B11" s="9" t="s">
-        <v>924</v>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES, noting #37 and #47</t>
+        </is>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
         <v>928</v>
       </c>
-      <c r="B12" s="10" t="s">
-        <v>924</v>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
         <v>929</v>
       </c>
-      <c r="B13" s="9" t="s">
-        <v>924</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="23.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
         <v>930</v>
       </c>
-      <c r="B14" s="10" t="s">
-        <v>931</v>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONDITIONALLY ACCEPTED, as the team's recommendation (30 September 2026, #69). The gate decision is the assessor's, recorded in B19, and is pending.</t>
+        </is>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
         <v>932</v>
       </c>
-      <c r="B15" s="12" t="s">
-        <v>933</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#27 the Figure 2 label defect; #36 figure sources not held in the repository; #37 branch naming breached on five branches; #47 checks required before any existed; #48 PED s12.4 narrower than Master Brief s14. Each is carried in PED s26.2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15.0" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
         <v>1033</v>
       </c>
-      <c r="B16" s="10" t="s">
-        <v>935</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Approved, 30 September 2026, recorded on #69, not at a gate review</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15.0" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
         <v>1034</v>
       </c>
-      <c r="B17" s="9" t="s">
-        <v>935</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Approved, 30 September 2026, recorded on #69, not at a gate review</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15.0" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
         <v>1035</v>
       </c>
-      <c r="B18" s="10" t="s">
-        <v>935</v>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Approved, 30 September 2026, recorded on #69, not at a gate review</t>
+        </is>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
         <v>938</v>
       </c>
-      <c r="B19" s="12" t="s">
-        <v>933</v>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For the assessor to complete</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -12471,7 +12497,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="323.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="690.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
         <v>536</v>
       </c>
@@ -12497,19 +12523,22 @@
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2 (29 September 2026): ADR-002 pins every package exactly, with a committed lockfile. #90 overrides deepmerge-ts to 8.0.2 and mysql2 to 3.24.4, and npm audit reports 0 vulnerabilities at 9529e80. The overrides are removed when a Prisma 7 release fixes issue #30295. Automated dependency checking arrives with #67.
+          <t xml:space="preserve">M2 (29 September 2026): ADR-002 pins every package exactly, with a committed lockfile. On the #90 branch, which has not merged, the bootstrap overrides deepmerge-ts to 8.0.2 and mysql2 to 3.24.4, and npm audit reports 0 vulnerabilities at 9529e80. The overrides are removed when a Prisma 7 release fixes issue #30295. npm audit --audit-level=high runs on every pull request once the CI workflow (#110) merges, so a new advisory fails the build.
 M1 baseline: Make dependency-ecosystem maturity a criterion in DEC-008. Adopt lockfiles and automated dependency and vulnerability checking from the first construction Pull Request. Require any new dependency to be justified in the Pull Request that introduces it.</t>
         </is>
       </c>
-      <c r="I14" s="10" t="s">
-        <v>540</v>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 (6 October 2026): Keep the overrides while Prisma 7 pins the affected versions, and remove them when a Prisma 7 release fixes #30295. If an override breaks Prisma, return to the last working set, record the advisory as an accepted residual risk with the owner's reasons, and raise a change to the stack under ADR-002. If a new advisory has no override, replace the component.
+M1 baseline: Remove or replace the affected component, assess exposure, and record the residual risk rather than claiming the system is clean.</t>
+        </is>
       </c>
       <c r="J14" s="10" t="s">
         <v>1009</v>
       </c>
       <c r="K14" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2 (29 September 2026): Materialised - active. Prisma 7.10.0 pins deepmerge-ts 7.1.5 and mysql2 3.15.3, which carry high-severity advisories no 7.x release has fixed (Prisma issue #30295, found 28 September 2026). Probability re-scored from 2 to 3 under #68, for the owner to confirm.
+          <t xml:space="preserve">Materialised - active. Found 28 September 2026: Prisma 7.10.0 pins deepmerge-ts 7.1.5 and mysql2 3.15.3, which carry high-severity advisories no 7.x release has fixed (Prisma issue #30295). On the #90 branch, which has not merged, the bootstrap overrides them to deepmerge-ts 8.0.2 and mysql2 3.24.4, and npm audit reports 0 vulnerabilities (9529e80; again at fbd12e9 on 9 October 2026). The audit gate arrives once the CI workflow (#110) merges. The status becomes Materialised - mitigated when both have merged. Probability re-scored from 2 to 3 under #68 and confirmed by the owner, Darius Mushi, on #106, 8 October 2026.
 M1 baseline: Open</t>
         </is>
       </c>

</xml_diff>

<commit_message>
docs(#107): CR-004 approved by both members; rebuilt on #136
Tristan Roets approved CR-004 on #129 on 12 October 2026, after Darius
Mushi on 8 October. CR-004 P6 reads Approved and cites both; DEC-016 is
Decided; DEC-008's M3 entries say DEC-016 replaces the conditions; ADR-002's
status lines and the passages that said CR-004 "proposes" now record the
amendment as approved.

Rebuilt on #136 (07df332), which merges first: each commit's workbook was
regenerated by its version of cr004_registers.py on #136's workbook, and
the fixtures re-exported, since their source line holds the workbook's
hash (tests/README.md). Once #136 is on main this branch moves onto main
with no change to its content.
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -4368,7 +4368,7 @@
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">M3 (5 October 2026, CR-004): DEC-016 proposes replacing the two conditions below with an environment check repeated by a member other than the author and then by CI, and a proof of concept that persists a User from the ADR-007 model. Gate 3 is carried as RSK-30.
+          <t xml:space="preserve">M3 (CR-004, approved 12 October 2026): DEC-016 replaces the two conditions below with an environment check repeated by a member other than the author and then by CI, and a proof of concept that persists a User from the ADR-007 model. Gate 3 is carried as RSK-30.
 M2 (28 September 2026, ADR-002): Option (a) at exact pins: Express 5.2.1; Prisma CLI, client and PostgreSQL adapter 7.10.0; pg 8.23.0; argon2 0.45.1; node-cron 4.6.0; node:test; React 19.3.0 and Vite 8.3.0 with the first client work. Conditional: gate 3 on a BC Desktop machine and the RSK-01 proof of concept must pass before #90 merges.
 M1 baseline: Deliberately not decided.</t>
         </is>
@@ -4393,14 +4393,14 @@
       </c>
       <c r="K10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">M3 (5 October 2026, CR-004): under DEC-016, once CR-004 is approved, what is still required is the amended conditions, not gate 3; see DEC-016.
+          <t xml:space="preserve">M3 (CR-004, approved 12 October 2026): under DEC-016, what is still required is the amended conditions, not gate 3; see DEC-016.
 M2 (28 September 2026, ADR-002): ADR-002 (#91). npm registry and PyPI metadata, the Node.js release schedule and Prisma issue #30295; team capability as reported by each member. Still required: gate 3 and the RSK-01 proof of concept.
 M1 baseline: Evidence still required: requirement and architecture fit; realistic learning curve for these three members; availability and compatibility on the BC Desktop platform; dependency ecosystem maturity; testing and automation support; deployment compatibility; free-tier limits and likely operational cost; lock-in and unavailability consequences.</t>
         </is>
       </c>
       <c r="L10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">M3 (5 October 2026, CR-004): under DEC-016, once CR-004 is approved, #90 merges after the amended conditions instead; see DEC-016.
+          <t xml:space="preserve">M3 (CR-004, approved 12 October 2026): under DEC-016, #90 merges after the amended conditions instead; see DEC-016.
 M2 (28 September 2026, ADR-002): DEC-010 (#60) must provide a Node 24 runtime and PostgreSQL, and run one instance while node-cron is used. Upgrading to Prisma 8 is a separate decision once it is stable. #90 merges only after both conditions.
 M1 baseline: Determines construction, testing and deployment for the remainder of the project.</t>
         </is>
@@ -4804,7 +4804,7 @@
         </is>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="81.78" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="70.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">DEC-016</t>
@@ -4817,7 +4817,7 @@
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed (M3, CR-004, #107); decided when CR-004 is approved on #129. Approved by Darius Mushi on 8 October 2026; Tristan Roets to answer</t>
+          <t xml:space="preserve">Decided (M3, CR-004, #107). CR-004 approved on #129 by Darius Mushi on 8 October 2026 and Tristan Roets on 12 October 2026</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -6403,7 +6403,7 @@
       </c>
       <c r="P6" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed, partly approved. Darius Mushi approved CR-004 on #129 on 8 October 2026, subject to DEC-016's later consequence naming both amended conditions, which it now does. Tristan Roets's decision is still to be recorded on #129. This cell then cites it and its date before #129 merges, as CR-001 to CR-003 cite theirs on #69.</t>
+          <t xml:space="preserve">Approved. Darius Mushi approved CR-004 on #129 on 8 October 2026, subject to DEC-016's later consequence naming both amended conditions, which it does. Tristan Roets approved it on #129 on 12 October 2026.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: implement CR-002, correct the four Access Matrix cells (#136)
Closes #92. CR-002, approved on #69: the Access Matrix no longer grants the four cells FR-015, FR-016, FR-020 and FR-021 refuse; the fixtures are exported from the workbook by tools/export_register_fixtures.py, MATRIX_CONFLICTS is empty, and the PED's s8.3 reading note records the correction. Approved by Darius Mushi and Tristan Roets.
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -6174,7 +6174,7 @@
       </c>
       <c r="P4" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Approved, not implemented. Approved by all three members on #69, 30 September 2026: fix the matrix for all four cells. The Access Matrix sheet, PED s8.3 and the test fixture still show the four cells until #92 corrects them in M3.</t>
+          <t xml:space="preserve">Approved and implemented. Approved by all three members on #69, 30 September 2026: fix the matrix for all four cells. Implemented under #92 (6 October 2026): the Access Matrix sheet now refuses the four cells, the test fixture is re-exported from it, and the policy's list of conflicts is empty. PED s8.3 is corrected in PED v3.0 (#127); until then its reading note records the correction.</t>
         </is>
       </c>
     </row>
@@ -6618,7 +6618,7 @@
         <v>831</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>831</v>
+        <v>834</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6632,7 +6632,7 @@
         <v>831</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>831</v>
+        <v>834</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>834</v>
@@ -6703,7 +6703,7 @@
         <v>831</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>831</v>
+        <v>834</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6720,7 +6720,7 @@
         <v>831</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>831</v>
+        <v>834</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
docs: CR-004, amend ADR-002's merge conditions for the bootstrap (#129)
Part of #107. CR-004 replaces ADR-002's verified campus run with two conditions on #90: an environment check repeated by a member other than the author, and CI repeating it once #110 merges. DEC-016 is Decided, RSK-30 carries the campus environment risk, and the fixtures are re-exported. Approved by Darius Mushi and Tristan Roets.
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -30,14 +30,14 @@
     <definedName function="false" hidden="true" localSheetId="13" name="_xlnm._FilterDatabase" vbProcedure="false">'Access Matrix'!$A$2:$E$17</definedName>
     <definedName function="false" hidden="true" localSheetId="10" name="_xlnm._FilterDatabase" vbProcedure="false">'AI Usage Register'!$A$2:$H$29</definedName>
     <definedName function="false" hidden="true" localSheetId="16" name="_xlnm._FilterDatabase" vbProcedure="false">'Baseline Sign-off'!$A$2:$B$19</definedName>
-    <definedName function="false" hidden="true" localSheetId="11" name="_xlnm._FilterDatabase" vbProcedure="false">'Change Requests'!$A$2:$P$5</definedName>
+    <definedName function="false" hidden="true" localSheetId="11" name="_xlnm._FilterDatabase" vbProcedure="false">'Change Requests'!$A$2:$P$6</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">Constraints!$A$2:$D$10</definedName>
-    <definedName function="false" hidden="true" localSheetId="9" name="_xlnm._FilterDatabase" vbProcedure="false">'Decision Log'!$A$2:$L$17</definedName>
+    <definedName function="false" hidden="true" localSheetId="9" name="_xlnm._FilterDatabase" vbProcedure="false">'Decision Log'!$A$2:$L$18</definedName>
     <definedName function="false" hidden="true" localSheetId="8" name="_xlnm._FilterDatabase" vbProcedure="false">'Forward Considerations'!$A$2:$G$9</definedName>
     <definedName function="false" hidden="true" localSheetId="15" name="_xlnm._FilterDatabase" vbProcedure="false">'GitHub Governance'!$A$2:$C$14</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Requirements (FR)'!$A$2:$F$31</definedName>
     <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">'Requirements (NFR)'!$A$2:$G$15</definedName>
-    <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">'Risk Register'!$A$2:$L$31</definedName>
+    <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">'Risk Register'!$A$2:$L$32</definedName>
     <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">RTM!$A$2:$O$44</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Scope Baseline'!$A$2:$E$27</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Stakeholders!$A$2:$G$11</definedName>
@@ -3943,7 +3943,7 @@
       </c>
       <c r="B23" s="6" t="n">
         <f aca="false">COUNTIF('Risk Register'!G3:G200,"Medium")</f>
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3970,7 +3970,7 @@
       </c>
       <c r="B26" s="6" t="n">
         <f aca="false">COUNTA('Decision Log'!A3:A200)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3998,7 +3998,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -4368,7 +4368,8 @@
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2 (28 September 2026, ADR-002): Option (a) at exact pins: Express 5.2.1; Prisma CLI, client and PostgreSQL adapter 7.10.0; pg 8.23.0; argon2 0.45.1; node-cron 4.6.0; node:test; React 19.3.0 and Vite 8.3.0 with the first client work. Conditional: gate 3 on a BC Desktop machine and the RSK-01 proof of concept must pass before #90 merges.
+          <t xml:space="preserve">M3 (CR-004, approved 12 October 2026): DEC-016 replaces the two conditions below with an environment check repeated by a member other than the author and then by CI, and a proof of concept that persists a User from the ADR-007 model. Gate 3 is carried as RSK-30.
+M2 (28 September 2026, ADR-002): Option (a) at exact pins: Express 5.2.1; Prisma CLI, client and PostgreSQL adapter 7.10.0; pg 8.23.0; argon2 0.45.1; node-cron 4.6.0; node:test; React 19.3.0 and Vite 8.3.0 with the first client work. Conditional: gate 3 on a BC Desktop machine and the RSK-01 proof of concept must pass before #90 merges.
 M1 baseline: Deliberately not decided.</t>
         </is>
       </c>
@@ -4392,13 +4393,15 @@
       </c>
       <c r="K10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2 (28 September 2026, ADR-002): ADR-002 (#91). npm registry and PyPI metadata, the Node.js release schedule and Prisma issue #30295; team capability as reported by each member. Still required: gate 3 and the RSK-01 proof of concept.
+          <t xml:space="preserve">M3 (CR-004, approved 12 October 2026): under DEC-016, what is still required is the amended conditions, not gate 3; see DEC-016.
+M2 (28 September 2026, ADR-002): ADR-002 (#91). npm registry and PyPI metadata, the Node.js release schedule and Prisma issue #30295; team capability as reported by each member. Still required: gate 3 and the RSK-01 proof of concept.
 M1 baseline: Evidence still required: requirement and architecture fit; realistic learning curve for these three members; availability and compatibility on the BC Desktop platform; dependency ecosystem maturity; testing and automation support; deployment compatibility; free-tier limits and likely operational cost; lock-in and unavailability consequences.</t>
         </is>
       </c>
       <c r="L10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2 (28 September 2026, ADR-002): DEC-010 (#60) must provide a Node 24 runtime and PostgreSQL, and run one instance while node-cron is used. Upgrading to Prisma 8 is a separate decision once it is stable. #90 merges only after both conditions.
+          <t xml:space="preserve">M3 (CR-004, approved 12 October 2026): under DEC-016, #90 merges after the amended conditions instead; see DEC-016.
+M2 (28 September 2026, ADR-002): DEC-010 (#60) must provide a Node 24 runtime and PostgreSQL, and run one instance while node-cron is used. Upgrading to Prisma 8 is a separate decision once it is stable. #90 merges only after both conditions.
 M1 baseline: Determines construction, testing and deployment for the remainder of the project.</t>
         </is>
       </c>
@@ -4801,8 +4804,70 @@
         </is>
       </c>
     </row>
+    <row r="18" customFormat="false" ht="70.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEC-016</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bootstrap merge conditions, amending DEC-008</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decided (M3, CR-004, #107). CR-004 approved on #129 by Darius Mushi on 8 October 2026 and Tristan Roets on 12 October 2026</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-002 (DEC-008) let the bootstrap (#90) merge only after gate 3 closed on a BC Desktop machine and the RSK-01 proof of concept passed. By 5 October 2026 neither was shown: the verification logs on #64 disagree, and the proof of concept persisted to a temporary table. Every M3 implementation issue depends on the bootstrap.</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CON-07 platform availability; CON-02 schedule, with M3 due 14 October 2026; RSK-01; NFR-004.</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(a) Keep both conditions and wait for a verified campus run. (b) Replace the campus run with a check a second member repeats and CI then runs on every pull request, keep the campus check as a risk, and restate the proof of concept against the data model. (c) Remove the conditions.</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(b), recorded as CR-004 and as a dated amendment to ADR-002.</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A check another member can repeat, and that CI then repeats on every pull request, is stronger evidence than a single run nobody else can see. (a) holds all of M3 on lab access the team does not control. (c) drops the evidence ADR-002 asked for.</t>
+        </is>
+      </c>
+      <c r="I18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No verified run on the campus image before construction starts, so the campus environment can still differ.</t>
+        </is>
+      </c>
+      <c r="J18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RSK-30: the campus environment differs from the verified Node 24 and PostgreSQL 16 environment.</t>
+        </is>
+      </c>
+      <c r="K18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The #64 verification logs (30 September 2026); the reviews on #90; CR-004 and the ADR-002 amendment (#107).</t>
+        </is>
+      </c>
+      <c r="L18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#90 merges under #108 once both amended conditions are shown on it: the environment check, run by a member other than the author and posted on #90, and the proof of concept persisting a User from the ADR-007 model. Once #110 merges, the CI workflow repeats the check on every pull request. The campus check is run when lab access allows and recorded on #64.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L17"/>
+  <autoFilter ref="A2:L18"/>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>
@@ -5932,7 +5997,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -6260,8 +6325,90 @@
         </is>
       </c>
     </row>
+    <row r="6" customFormat="false" ht="226.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR-004</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jean Smit</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 October 2026</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Amend the two conditions ADR-002 sets before the bootstrap (#90) merges (#107). Condition 1, gate 3 on a BC Desktop machine, becomes a reproducible check: a member other than the author runs npm ci, prisma generate, prisma migrate deploy and npm test from a fresh clone with no node_modules, on Node 24 against PostgreSQL 16, and posts the output on #90 with the operating system, node -v and where PostgreSQL ran. The CI workflow repeats it on every pull request once #110 merges. The campus check becomes RSK-30. Condition 2 is restated: the RSK-01 proof of concept persists a User from the ADR-007 model through Prisma and verifies an argon2 sign-in.</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Neither condition could be shown as met. The two verification logs on #64 disagree: the log with a screenshot ran on a member's own machine on Node 25.9.0 with mock data, and the log that reports a campus run has no screenshot or command output. The proof of concept in #90 persists to a table the test creates and drops, outside the data model. M3 is due 14 October 2026 and every M3 implementation issue depends on the bootstrap.</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None. NFR-004 and the substance of the RSK-01 proof of concept are unchanged.</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-002: the merge conditions under Decision, recorded as a dated amendment. The original conditions stay in the record.</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data: the proof of concept uses the User entity from ADR-007 instead of a temporary table.</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None. The argon2 check is kept.</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The environment check becomes repeatable: a second member's run on #90, then the CI workflow (#110) on every pull request, on Node 24 against PostgreSQL 16.</t>
+        </is>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="L6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unblocks #108, and through it every M3 implementation issue. The timebox was #108's due date, 7 October 2026. The proof of concept on the User model was pushed to #90 on 11 October 2026 (e162f28), four days after it; the second member's environment check is still to be posted. The date is not moved: the delay is recorded here and in ADR-002's amendment.</t>
+        </is>
+      </c>
+      <c r="M6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="N6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adds RSK-30 for the unverified campus environment. RSK-01 and RSK-02 are unchanged.</t>
+        </is>
+      </c>
+      <c r="O6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ACCEPT</t>
+        </is>
+      </c>
+      <c r="P6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Approved. Darius Mushi approved CR-004 on #129 on 8 October 2026, subject to DEC-016's later consequence naming both amended conditions, which it does. Tristan Roets approved it on #129 on 12 October 2026.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:P5"/>
+  <autoFilter ref="A2:P6"/>
   <mergeCells count="1">
     <mergeCell ref="A1:P1"/>
   </mergeCells>
@@ -11981,7 +12128,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -13450,8 +13597,64 @@
         </is>
       </c>
     </row>
+    <row r="32" customFormat="false" ht="46.73" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RSK-30</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The BC Desktop campus environment differs from the Node 24 and PostgreSQL 16 environment the stack was verified on, so the application does not install or run on campus machines.</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR-004 replaced the campus run with a check repeated by a second member and in CI, because no verified campus run exists (#64). CON-07: the campus cannot guarantee the stack is available.</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F32" s="13" t="n">
+        <f aca="false">D32*E32</f>
+        <v>9</v>
+      </c>
+      <c r="G32" s="13" t="str">
+        <f aca="false">IF(F32&gt;=20,"Critical",IF(F32&gt;=12,"High",IF(F32&gt;=6,"Medium","Low")))</f>
+        <v>Medium</v>
+      </c>
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">npm ci installs from the committed lockfile. #90's engines field is to limit Node to version 24 (&gt;=24 &lt;25, with engine-strict), as agreed on #90. Once the CI workflow (#110) merges, it runs the check on Node 24 against PostgreSQL 16 on every pull request. Run the campus check when lab access allows and record the Node version on #64.</t>
+        </is>
+      </c>
+      <c r="I32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Demonstrate from a team member's machine on the simulated staging environment (#122), and record the campus difference as a limitation in the release summary.</t>
+        </is>
+      </c>
+      <c r="J32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Darius Mushi</t>
+        </is>
+      </c>
+      <c r="K32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="L32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-002, CR-004, DEC-016, CON-07, RSK-01, RSK-02, #64, #90, #107</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L31"/>
+  <autoFilter ref="A2:L32"/>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs(#126): record DEC-017, and CR-005 and CR-006 as proposed, in the registers (#154)
Part of #126. DEC-017 is recorded as Decided in the Decision Log, from all three members' answers on #131. CR-005 and CR-006 are recorded as Proposed, with Tristan Roets's agreement and Darius Mushi's answer pending. The fixtures are re-exported for the workbook's new hash, and the test catalogue cites DEC-017 as decided. Approved by Darius Mushi and Tristan Roets.
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -30,9 +30,9 @@
     <definedName function="false" hidden="true" localSheetId="13" name="_xlnm._FilterDatabase" vbProcedure="false">'Access Matrix'!$A$2:$E$17</definedName>
     <definedName function="false" hidden="true" localSheetId="10" name="_xlnm._FilterDatabase" vbProcedure="false">'AI Usage Register'!$A$2:$H$29</definedName>
     <definedName function="false" hidden="true" localSheetId="16" name="_xlnm._FilterDatabase" vbProcedure="false">'Baseline Sign-off'!$A$2:$B$19</definedName>
-    <definedName function="false" hidden="true" localSheetId="11" name="_xlnm._FilterDatabase" vbProcedure="false">'Change Requests'!$A$2:$P$6</definedName>
+    <definedName function="false" hidden="true" localSheetId="11" name="_xlnm._FilterDatabase" vbProcedure="false">'Change Requests'!$A$2:$P$8</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">Constraints!$A$2:$D$10</definedName>
-    <definedName function="false" hidden="true" localSheetId="9" name="_xlnm._FilterDatabase" vbProcedure="false">'Decision Log'!$A$2:$L$18</definedName>
+    <definedName function="false" hidden="true" localSheetId="9" name="_xlnm._FilterDatabase" vbProcedure="false">'Decision Log'!$A$2:$L$19</definedName>
     <definedName function="false" hidden="true" localSheetId="8" name="_xlnm._FilterDatabase" vbProcedure="false">'Forward Considerations'!$A$2:$G$9</definedName>
     <definedName function="false" hidden="true" localSheetId="15" name="_xlnm._FilterDatabase" vbProcedure="false">'GitHub Governance'!$A$2:$C$14</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Requirements (FR)'!$A$2:$F$31</definedName>
@@ -3970,7 +3970,7 @@
       </c>
       <c r="B26" s="6" t="n">
         <f aca="false">COUNTA('Decision Log'!A3:A200)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3998,7 +3998,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -4866,8 +4866,70 @@
         </is>
       </c>
     </row>
+    <row r="19" customFormat="false" ht="175.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEC-017</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Submission and workflow details the M1 baseline leaves open: the reference format, the urgency scale, the field limits and who sees priority</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decided (M3, #131). Agreed by all three members: Jean Smit and Tristan Roets on 7 October 2026, Darius Mushi on 8 October 2026</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FR-008's acceptance criterion refers to "the agreed format" for the reference, and no baseline artefact states one. FR-005 and FR-021 require a reported urgency and a priority, with no scale. The schema limits the title (VARCHAR(200)) and leaves description and location unlimited. FR-021 says Coordinators see both values and is silent on the Requester. The submission and workflow services (#131, #132) and the screens (#133 to #135) each need these fixed.</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEC-004: the reference is issued at submission, unique, never reused, and not a visible counter. ADR-007: the reference sequence and its unique constraint. FR-012. NFR-007: no secret in the source. DEC-002.</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reference: (a) a visible counter, which DEC-004 rejects because it reveals volume and invites guessing; (b) a random reference retried on collision, which gives up the sequence's guarantee of uniqueness; (c) the sequence passed through a keyed permutation into a fixed format. Urgency and priority: a numeric scale, or three named levels.</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Reference: CC- and eight digits in two groups of four, for example CC-4829-1573, from ADR-007's sequence through a keyed permutation. The key (REFERENCE_KEY) is configuration, never in the source, and stays fixed for the life of the data. DEC-004 is unchanged. 2. Reported urgency: Low, Medium, High, with the descriptions shown on the form. 3. Field limits: title 200 characters, description 4,000, location 300, each counted after trimming, and every field at least one non-blank character. 4. Priority: the same Low, Medium, High scale, set only by a Coordinator (FR-021). Staff, Coordinators and Managers see priority and assignee; a Requester sees the urgency they reported.</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(c) keeps the uniqueness the sequence and the unique constraint give, while one reference, or a run of them, reveals neither its position nor the volume. Three named levels are a choice a requester can make without guidance, and one scale for urgency and priority lets a Coordinator compare them directly (DEC-002). The title limit is the schema's; the others are what a request needs. Showing the Requester only what they supplied keeps FR-021's separation of urgency and priority.</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The key cannot change once there is data: a different key is a different permutation, so a new request could land on an existing reference and the insert would be refused. Capacity is 99,999,999 references. A Requester does not see how their request was prioritised.</t>
+        </is>
+      </c>
+      <c r="J19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If the key leaks, the volume DEC-004 guards is exposed, but access is still governed by FR-012's scope check on every lookup. A Requester may feel their urgency was ignored, which DEC-002 records.</t>
+        </is>
+      </c>
+      <c r="K19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The proposal on #131 (issuecomment-6010035116, 6 October 2026); the answers of Jean Smit and Tristan Roets on #131 (7 October 2026) and of Darius Mushi in his review of #131 (8 October 2026); the tests in #131 and #132.</t>
+        </is>
+      </c>
+      <c r="L19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Each value is held in one place in the code (reference.js, validation.js, views.js and the workflow service), so a change is one line and the tests follow it. Changing any of the four is a new decision.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L18"/>
+  <autoFilter ref="A2:L19"/>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>
@@ -5997,7 +6059,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -6407,8 +6469,172 @@
         </is>
       </c>
     </row>
+    <row r="7" customFormat="false" ht="297.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR-005</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jean Smit</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7 October 2026</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Record the changes PED v2.0 makes to M1 sections (1 to 17) that CR-001 to CR-003 do not cover (#95). 1. The cover updated for each version: title, milestone, document line and baseline status. 2. A Milestone 2 boundary note added under the M1 one. 3. A paragraph added to s2 on how the M1 and M2 sections relate. 4. Reading notes added to s10, s13 and s14.2, each saying the section shows the register as at M1 and pointing to the live register in the workbook. 5. Four references added to s17, for s20, s24 and s26.2. 6. The M1 template instruction left under the version table in v1.0 removed. 7. The team's M1 sign-off recorded in s16 as its recommendation (#69), with the assessor's gate decision pending. Item 1 was widened on 8 October 2026 from the v2.0 cover alone, so that v3.0 (#145) and v4.0 update the same cover rows under this change.</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v2.0 continues the same document (Master Brief s6), so the M1 sections must stay readable next to the M2 ones without being rewritten. Items 1 to 4 tell a reader what changed and where the live versions are; item 5 supports claims made in the M2 sections; item 6 removes text that was never meant to be submitted; item 7 records a decision the team took on #69. A change request per version for the cover would add records without adding control, and the version row in s1 records each cover change.</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None. Every M1 table keeps its content.</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tools/ped_fidelity.py --m1-only lists every difference from v1.0 in sections 1 to 17, so a reviewer can compare it with the version row: 55 lines on v2.0, 60 on v3.0.</t>
+        </is>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="M7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="N7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None. The reading notes point to registers changed under their own pull requests.</t>
+        </is>
+      </c>
+      <c r="O7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ACCEPT</t>
+        </is>
+      </c>
+      <c r="P7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proposed, partly answered. Tristan Roets agreed to the seven items on #95 on 7 October 2026, and to item 1 as widened on 12 October 2026. Darius Mushi's answer is still to be recorded on #95; this cell is then changed to cite it and its date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="357.0" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR-006</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jean Smit</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7 October 2026</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add five columns to the RTM after column N, so that Status stays the last column (#126). 1. Test cases (M3): the IDs of the records in docs/quality/test-catalogue.md that verify the requirement's acceptance criterion. 2. Expected result (M3): one sentence stating what those tests must show for the criterion to be met, written from the criterion before the result is known. 3. Execution evidence (M3): the run that shows the result, the CI run once #110 merges or until then a dated local run with its commit, and the count of checks passed. 4. Defects (M3): the Defect Register IDs (#125) that affect the criterion, or None. 5. Acceptance criterion status (M3): one of Met, Partially met, Not met, Not yet verified, or Changed or removed under CR-nnn. Not yet verified is used only during M3, and no row may hold it at the Final. The title cell is updated to describe the five columns and their values. Column F keeps its pointer to the requirements registers, and column M (CR-003) keeps naming the test files and pull requests.</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The M3 brief (s12) requires the RTM to carry each implemented requirement through to its test cases, expected result, execution evidence and defect status. The Final brief (s9) calculates Scope Completion from a status for each M1 acceptance criterion (Met 1.0, Partially met 0.5, Not met 0.0). With these columns every one of the 42 criteria (29 FR, 13 NFR) has a status from M3 onwards, and the percentage is a calculation over one column rather than a reconstruction at the end.</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None. Every requirement keeps its row and its criterion.</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Each criterion is tied to designed test cases and a run, and an unverified criterion is visible as such.</t>
+        </is>
+      </c>
+      <c r="K8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None. Changed or removed criteria are counted against the changed baseline with their CR reference, as the Final brief requires.</t>
+        </is>
+      </c>
+      <c r="L8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Part of #126.</t>
+        </is>
+      </c>
+      <c r="M8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="N8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None new. Gaps in verification show up during M3, while there is time to close them.</t>
+        </is>
+      </c>
+      <c r="O8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ACCEPT</t>
+        </is>
+      </c>
+      <c r="P8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proposed, partly answered. Proposed on #126 on 7 October 2026; Tristan Roets agreed there on 12 October 2026. Darius Mushi's answer is still to be recorded on #126. The columns are added and filled under #126 once he has answered, and this cell is then changed to cite the answers and their dates.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:P6"/>
+  <autoFilter ref="A2:P8"/>
   <mergeCells count="1">
     <mergeCell ref="A1:P1"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs(#127): AI Usage Register, Darius Mushi's row for drafting s28, s30 and s31
Row 30, in Darius Mushi's own words as he sent them on 16 October 2026,
so s30.5's statement that the entry exists is true. Byte-level edit:
only the AI Usage Register sheet (row 30, its dimension and autoFilter)
and workbook.xml (its _FilterDatabase range) change. The fixtures are
re-exported for the workbook's new hash, with no matrix or status cell
changed; export_register_fixtures.py --check passes, and the policy and
status-model tests pass, 23 of 23.
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -28,7 +28,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="13" name="_xlnm._FilterDatabase" vbProcedure="false">'Access Matrix'!$A$2:$E$17</definedName>
-    <definedName function="false" hidden="true" localSheetId="10" name="_xlnm._FilterDatabase" vbProcedure="false">'AI Usage Register'!$A$2:$H$29</definedName>
+    <definedName function="false" hidden="true" localSheetId="10" name="_xlnm._FilterDatabase" vbProcedure="false">'AI Usage Register'!$A$2:$H$30</definedName>
     <definedName function="false" hidden="true" localSheetId="16" name="_xlnm._FilterDatabase" vbProcedure="false">'Baseline Sign-off'!$A$2:$B$19</definedName>
     <definedName function="false" hidden="true" localSheetId="11" name="_xlnm._FilterDatabase" vbProcedure="false">'Change Requests'!$A$2:$P$8</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">Constraints!$A$2:$D$10</definedName>
@@ -4949,7 +4949,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -6038,8 +6038,50 @@
         </is>
       </c>
     </row>
+    <row r="30" customFormat="false" ht="140" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16 October 2026</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Darius Mushi</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Sonnet 5.5 (Anthropic)</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drafting PED v3.0 s28 (M2 baseline conformance), s30 (construction and configuration) and s31 (CI and automated verification) for the M3 submission (#127).</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proposed the structure and text of the three sections from the PED, the M3 brief and pull request #145, and listed the facts it could not confirm as open questions. Wrote the final text after I supplied repository evidence, and gave the PowerShell commands used to insert it into the PED markdown.</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cross-checked each statement against live repository output: the src/modules listing, package.json, .npmrc, ruleset 22248862 read back from the GitHub API, a full-history gitleaks detect (267 commits, no leaks), the state of issues #27, #36, #37, #48 and #49, the merged pull requests, the workflow file, and the review history of #90 and #129. Checked the insertion with Select-String for leftover placeholders and with git diff --stat (176 insertions, 3 deletions, one file).</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted after revision. Facts that could not be confirmed were kept as open questions until the repository evidence was supplied, instead of being guessed.</t>
+        </is>
+      </c>
+      <c r="H30" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The first draft left unverified facts in brackets. Checking the repository corrected three errors: the persistence module only re-exports the Prisma client, the first migration creates only the User table, and a PostgreSQL 18.6 run does not meet the ADR-002 amendment, which needs 16. The FR-004 deviation (a Manager-assisted one-time code, not a reset link) was added after checking #146 against the requirement. Three points are still to be confirmed by the team: the production database decision, that a109702 is the head that merged #90, and the reason for the FR-004 deviation</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:H29"/>
+  <autoFilter ref="A2:H30"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs(#127): Darius Mushi's revised AI Usage Register row; #144 cited as elsewhere
Row 30 now holds the text Darius Mushi sent after the team's check: the
verification adds Jean Smit's check of the three assumptions, and the
issues found record the corrected debt-register statement in s28.2. The
row is rebuilt on the workbook as before ee841dc, so only the AI Usage
Register sheet and workbook.xml differ from it; the fixtures are
re-exported for the new hash and --check passes. s28.2 item 5 cites #144
as the rest of the document does.
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -6066,17 +6066,17 @@
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cross-checked each statement against live repository output: the src/modules listing, package.json, .npmrc, ruleset 22248862 read back from the GitHub API, a full-history gitleaks detect (267 commits, no leaks), the state of issues #27, #36, #37, #48 and #49, the merged pull requests, the workflow file, and the review history of #90 and #129. Checked the insertion with Select-String for leftover placeholders and with git diff --stat (176 insertions, 3 deletions, one file).</t>
+          <t xml:space="preserve">Cross-checked each statement against live repository output: the src/modules listing, package.json, .npmrc, ruleset 22248862 read back from the GitHub API, a full-history gitleaks detect (267 commits, no leaks), the state of issues #27, #36, #37, #48 and #49, the merged pull requests, the workflow file, and the review history of #90 and #129. Checked the insertion with Select-String for leftover placeholders and with git diff --stat. Jean Smit then checked the three assumptions the repository could not show.</t>
         </is>
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted after revision. Facts that could not be confirmed were kept as open questions until the repository evidence was supplied, instead of being guessed.</t>
+          <t xml:space="preserve">Accepted after revision. Facts that could not be confirmed were kept as open questions until the repository evidence or Jean's check was supplied, instead of being guessed.</t>
         </is>
       </c>
       <c r="H30" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">The first draft left unverified facts in brackets. Checking the repository corrected three errors: the persistence module only re-exports the Prisma client, the first migration creates only the User table, and a PostgreSQL 18.6 run does not meet the ADR-002 amendment, which needs 16. The FR-004 deviation (a Manager-assisted one-time code, not a reset link) was added after checking #146 against the requirement. Three points are still to be confirmed by the team: the production database decision, that a109702 is the head that merged #90, and the reason for the FR-004 deviation</t>
+          <t xml:space="preserve">The first draft left unverified facts in brackets. Checking the repository corrected three errors: the persistence module only re-exports the Prisma client, the first migration creates only the User table, and a PostgreSQL 18.6 run does not meet the ADR-002 amendment, which needs 16. The FR-004 deviation (a Manager-assisted one-time code, not a reset link) was added after checking #146 against the requirement. Jean's check corrected one statement: the draft said both reset limitations were in the Technical Debt Register, but only the Manager-assisted reset is recorded (TD-004, #144, in review) and the missing rate limit is not, so s28.2 now says that.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(#126): AI Usage Register rows 31 and 32 for Jean Smit's M3 work, and the README sheet's owner
Row 31: the M3 implementation and tests (#130 to #153). Row 32: PED v3.0 s27, s32 to s36 and s29.
Each states what the AI did, how it was verified and the issues review found. README B5, a placeholder
since M1, names the three members. Byte-level edits to sheet11, sheet1 and workbook.xml; fixtures
re-exported.
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -28,7 +28,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="13" name="_xlnm._FilterDatabase" vbProcedure="false">'Access Matrix'!$A$2:$E$17</definedName>
-    <definedName function="false" hidden="true" localSheetId="10" name="_xlnm._FilterDatabase" vbProcedure="false">'AI Usage Register'!$A$2:$H$30</definedName>
+    <definedName function="false" hidden="true" localSheetId="10" name="_xlnm._FilterDatabase" vbProcedure="false">'AI Usage Register'!$A$2:$H$32</definedName>
     <definedName function="false" hidden="true" localSheetId="16" name="_xlnm._FilterDatabase" vbProcedure="false">'Baseline Sign-off'!$A$2:$B$19</definedName>
     <definedName function="false" hidden="true" localSheetId="11" name="_xlnm._FilterDatabase" vbProcedure="false">'Change Requests'!$A$2:$P$8</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">Constraints!$A$2:$D$10</definedName>
@@ -3798,8 +3798,10 @@
       <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>6</v>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jean Smit - 600368 | Tristan Roets - 601764 | Darius Mushi - 577982</t>
+        </is>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4949,7 +4951,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -6080,8 +6082,92 @@
         </is>
       </c>
     </row>
+    <row r="31" customFormat="false" ht="160" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16 October 2026</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jean Smit</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code (Anthropic)</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M3 implementation and tests, 6 to 16 October 2026: sign-in and sessions (#130), request submission, the requester's views and the workflow service (#131, #132), the client screens (#133 to #135), CR-002 (#136), the test catalogue and its check (#137), the browser journeys (#138), the performance scripts (#139), the password reset (#146), the API suites (#147) and the review follow-ups (#149 to #153).</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrote the code and the tests from the requirements, the ADRs, DEC-017 and the registers, ran the suites, and drafted the commit messages and the pull request descriptions.</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Each new test for the services, the API suites and the scripts was shown to fail with the defect it guards against put back (s32.2). The suites were run on each branch and on main at d1af49a, and tools/check_test_catalogue.mjs --strict ties each test to its catalogue record. The RSK-01 test and the draft migrations were run against a local PostgreSQL 16.13. Every pull request is reviewed by the other two members before it merges.</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted after revision. #147 and #149 to #153 are still in review.</t>
+        </is>
+      </c>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Review and testing found real defects in the output, each fixed with a regression test: an emoji counted as two characters in the length limits (968a44f), a NUL character in a text field causing a server error (0efac6a), and the assignee id sent in the wrong form (c84b7c1). In the follow-ups, the performance scripts first waited on /api/health where the server serves /health, the catalogue check treated any .env file as a configured database, and a fault in the password-reset concurrency limit went undetected until a test for it was added. One commit message stated 76 tests where 72 ran, and was corrected before it was pushed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="160" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16 October 2026</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jean Smit</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code (Anthropic)</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drafting PED v3.0 s27 and s32 to s36, completing the submission information on 16 October 2026, and drafting s29 in place of Tristan Roets for the submitted build (#127, #145).</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drafted the sections from the M3 brief, the registers, the test catalogue and the repository, filled the placeholders at submission, and built the Word document and the PDF.</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Each count, date, commit and pull request number was read back from the repository or GitHub: merge dates and states with gh, test counts from the runs on main at d1af49a, and register text from the workbook. tools/ped_fidelity.py --m1-only confirmed that sections 1 to 17 differ only where the 3.0 row says (68 lines). The PDF was rendered page by page and checked for placeholders, layout and where each section starts.</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted after revision.</t>
+        </is>
+      </c>
+      <c r="H32" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Three statements were wrong and were corrected before submission: s36 said both reset limitations were in the Technical Debt Register, where only TD-004 is (#144); the run instructions in s27.1 left out the database steps the RSK-01 test needs; and the first draft of s29 said all five changes were made in M3, where two are still proposed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:H30"/>
+  <autoFilter ref="A2:H32"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs(#126): AI Usage Register row 33, Tristan Roets's M3 and Final use of ChatGPT
From Tristan Roets's own text of 17 October 2026: a supporting tool for understanding and checking
requirements, working through problems, reviewing work and the wording of documentation and review
comments; every change reviewed and every decision taken by Tristan Roets; none found in review.
Byte-level edit to sheet11 and workbook.xml; fixtures re-exported.
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -28,7 +28,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="13" name="_xlnm._FilterDatabase" vbProcedure="false">'Access Matrix'!$A$2:$E$17</definedName>
-    <definedName function="false" hidden="true" localSheetId="10" name="_xlnm._FilterDatabase" vbProcedure="false">'AI Usage Register'!$A$2:$H$32</definedName>
+    <definedName function="false" hidden="true" localSheetId="10" name="_xlnm._FilterDatabase" vbProcedure="false">'AI Usage Register'!$A$2:$H$33</definedName>
     <definedName function="false" hidden="true" localSheetId="16" name="_xlnm._FilterDatabase" vbProcedure="false">'Baseline Sign-off'!$A$2:$B$19</definedName>
     <definedName function="false" hidden="true" localSheetId="11" name="_xlnm._FilterDatabase" vbProcedure="false">'Change Requests'!$A$2:$P$8</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">Constraints!$A$2:$D$10</definedName>
@@ -4951,7 +4951,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -6166,8 +6166,50 @@
         </is>
       </c>
     </row>
+    <row r="33" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">17 October 2026</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tristan Roets</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ChatGPT (OpenAI)</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Supporting work during M3 and the Final Project: understanding and checking requirements, working through problems, reviewing parts of the work, and the wording of documentation and review comments.</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Helped to understand and check requirements, to work through problems and to review parts of the work, improved the wording of documentation and review comments, checked whether work matched the project requirements, and pointed out things that may have been overlooked.</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reviewed the changes personally, checked the results and the evidence, and made the final decision on everything submitted or approved.</t>
+        </is>
+      </c>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Used as a supporting tool only. The AI made no project decision and completed no task on its own.</t>
+        </is>
+      </c>
+      <c r="H33" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None found in review.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:H32"/>
+  <autoFilter ref="A2:H33"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs(#126): the final RTM, CR-006's five columns, counted per acceptance criterion
CR-006 (approved 18 October 2026) applied to the RTM sheet: columns O to S after N hold the test cases,
the expected result written from the criterion, the execution evidence, the defects, and the status of
each acceptance criterion in the requirement's row, counted per criterion as Darius Mushi's condition on
#126 asks. Status moves from O to T. Columns L and M (CR-003) now name the final implementation and the
test files and pull requests. The title states the Scope Completion: 64 of 69 criteria, 92.8 percent.

Not fully met: FR-004 (two criteria, the Manager-assisted reset), FR-022's target defined in the status
model, NFR-003, NFR-008, NFR-009, NFR-012 and NFR-013, each with its reason in the row. The statuses
assume #147 and #157 merge before the tag; they are rechecked there.

Byte-level edit: sheet7.xml and workbook.xml only; Excel opens it with no repair, used range A1:T44.
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -38,7 +38,7 @@
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Requirements (FR)'!$A$2:$F$31</definedName>
     <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">'Requirements (NFR)'!$A$2:$G$15</definedName>
     <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">'Risk Register'!$A$2:$L$32</definedName>
-    <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">RTM!$A$2:$O$44</definedName>
+    <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">RTM!$A$2:$T$44</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Scope Baseline'!$A$2:$E$27</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Stakeholders!$A$2:$G$11</definedName>
     <definedName function="false" hidden="true" localSheetId="12" name="_xlnm._FilterDatabase" vbProcedure="false">'Status Model'!$A$2:$D$14</definedName>
@@ -9753,7 +9753,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O44"/>
+  <dimension ref="A1:T44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -9770,13 +9770,18 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Requirements Traceability Matrix. From M2 (#54, CR-003), columns G to N trace each requirement to its quality driver, module, data, design, technology, implementation and verification evidence. A cell with no evidence yet holds a controlled status: Planned (M3), Not yet designed, Not yet decided, Not yet implemented or Not applicable. FR-016 is traced end to end.</t>
+          <t xml:space="preserve">Requirements Traceability Matrix. From M2 (#54, CR-003), columns G to N trace each requirement to its quality driver, module, data, design, technology, implementation and verification evidence. From the Final (CR-006, #126), columns O to S give the M3 and final trace: the test cases from docs/quality/test-catalogue.md, the expected result written from the criterion, the execution evidence, the defects, and the status of each acceptance criterion in the requirement's row, counted per criterion as CR-006's approval asks (Met 1.0, Partially met 0.5, Not met 0.0). Scope Completion: 64 of 69 criteria, 92.8 percent, at the release tag (PED v4.0 s38).</t>
         </is>
       </c>
       <c r="B1" s="7"/>
@@ -9792,7 +9797,7 @@
       <c r="L1" s="7"/>
       <c r="M1" s="7"/>
       <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
+      <c r="T1" s="7"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
@@ -9853,7 +9858,32 @@
           <t xml:space="preserve">ADR, change or risk reference</t>
         </is>
       </c>
-      <c r="O2" s="8" t="s">
+      <c r="O2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Test cases (M3 and Final)</t>
+        </is>
+      </c>
+      <c r="P2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Expected result</t>
+        </is>
+      </c>
+      <c r="Q2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Execution evidence</t>
+        </is>
+      </c>
+      <c r="R2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Defects</t>
+        </is>
+      </c>
+      <c r="S2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Acceptance criterion status (per criterion)</t>
+        </is>
+      </c>
+      <c r="T2" s="8" t="s">
         <v>176</v>
       </c>
     </row>
@@ -9903,12 +9933,12 @@
       </c>
       <c r="L3" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">src/modules/identity-access (sign-in.js, session.js, http.js) and the client's sign-in (#130, #133), wired in src/app.js (#155)</t>
         </is>
       </c>
       <c r="M3" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">tests/identity-access.test.js (#130), tests/api-decision-table.test.js (#147), tests/api-postgres.test.js (#155), client/test/api-and-router.test.js (#133), e2e journeys (#138)</t>
         </is>
       </c>
       <c r="N3" s="9" t="inlineStr">
@@ -9916,7 +9946,32 @@
           <t xml:space="preserve">RSK-05, RSK-01, ADR-002</t>
         </is>
       </c>
-      <c r="O3" s="9" t="s">
+      <c r="O3" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-08, TC-09, TC-10, TC-11, TC-23, TC-27, TC-32, TC-33</t>
+        </is>
+      </c>
+      <c r="P3" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No request data without a session and the visitor is sent to sign in; valid credentials give a session; every failed sign-in gets one answer that reveals nothing.</t>
+        </is>
+      </c>
+      <c r="Q3" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R3" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEF-001 (fixed)</t>
+        </is>
+      </c>
+      <c r="S3" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 of 3. AC1. unauthenticated: no data, redirected to sign-in: Met. 401 with no data (TC-23, TC-32); the client sends the visitor to sign in (TC-27) AC2. valid credentials: a session: Met. TC-10, TC-32, TC-33 AC3. invalid credentials: one generic message: Met. TC-09, TC-32</t>
+        </is>
+      </c>
+      <c r="T3" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -9966,12 +10021,12 @@
       </c>
       <c r="L4" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/authorisation-policy/policy.js (#94, merged)</t>
+          <t xml:space="preserve">src/modules/authorisation-policy/policy.js (#94, #136) and requirePermission in identity-access/http.js (#130)</t>
         </is>
       </c>
       <c r="M4" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/authorisation-policy.test.js (#94): every Access Matrix cell. Endpoint negative tests planned (M3)</t>
+          <t xml:space="preserve">tests/authorisation-policy.test.js (#94), tests/api-decision-table.test.js (#147), tests/api-postgres.test.js (#155)</t>
         </is>
       </c>
       <c r="N4" s="10" t="inlineStr">
@@ -9979,7 +10034,32 @@
           <t xml:space="preserve">RSK-05, FEC-01, ADR-006, CR-002 (#92)</t>
         </is>
       </c>
-      <c r="O4" s="10" t="s">
+      <c r="O4" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-01, TC-11, TC-22, TC-32</t>
+        </is>
+      </c>
+      <c r="P4" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Every role and function pair in the Access Matrix is permitted or refused as the register says, also when called directly at the endpoint.</t>
+        </is>
+      </c>
+      <c r="Q4" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R4" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEF-002 to DEF-005 (fixed by CR-002)</t>
+        </is>
+      </c>
+      <c r="S4" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 of 1. AC1. every pair permitted or refused, directly at the endpoint: Met. TC-01 all 60 cells; TC-22: 56 cells through their own endpoint, editAuditEntry's 4 at the permission check, since FR-026 forbids an endpoint</t>
+        </is>
+      </c>
+      <c r="T4" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -10029,12 +10109,12 @@
       </c>
       <c r="L5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">src/modules/administration (#155)</t>
         </is>
       </c>
       <c r="M5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">tests/administration.test.js, tests/api-postgres.test.js (#155)</t>
         </is>
       </c>
       <c r="N5" s="9" t="inlineStr">
@@ -10042,7 +10122,32 @@
           <t xml:space="preserve">ADR-007</t>
         </is>
       </c>
-      <c r="O5" s="9" t="s">
+      <c r="O5" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-43, TC-32, TC-31</t>
+        </is>
+      </c>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A Manager's new account authenticates with only its role's permissions; anyone else is refused.</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R5" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEF-008 (fixed)</t>
+        </is>
+      </c>
+      <c r="S5" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 of 2. AC1. Manager creates an account: it authenticates with only that role: Met. TC-43; TC-32 from the setup code to sign-in AC2. a non-Manager is refused: Met. TC-43, TC-22</t>
+        </is>
+      </c>
+      <c r="T5" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -10092,12 +10197,12 @@
       </c>
       <c r="L6" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">src/modules/identity-access/reset.js and concurrency.js (#146, #153); Manager-assisted, since email is deferred (SC-D-01)</t>
         </is>
       </c>
       <c r="M6" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">tests/password-reset.test.js (#146, #153), tests/api-postgres.test.js (#155)</t>
         </is>
       </c>
       <c r="N6" s="10" t="inlineStr">
@@ -10105,7 +10210,32 @@
           <t xml:space="preserve">RSK-05</t>
         </is>
       </c>
-      <c r="O6" s="10" t="s">
+      <c r="O6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-36, TC-32, TC-44</t>
+        </is>
+      </c>
+      <c r="P6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">One answer whatever the identifier; a reset credential works once and expires.</t>
+        </is>
+      </c>
+      <c r="Q6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 of 2. AC1. same message whether or not the account exists: Partially met. every failed reset gets one answer and a dummy check (TC-36), but there is no self-service reset request, because the reset is Manager-assisted AC2. a reset link is single-use and expires: Partially met. the Manager-issued code that replaces the link is single-use, expires after 24 hours and is withdrawn after five wrong tries (TC-36, TC-32); there is no link. Not changed through a change request (PED s29 item 6)</t>
+        </is>
+      </c>
+      <c r="T6" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -10155,12 +10285,12 @@
       </c>
       <c r="L7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">src/modules/request-capture (#131), client submit screen (#133)</t>
         </is>
       </c>
       <c r="M7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">tests/request-submission.test.js (#131), tests/api-postgres.test.js (#155), e2e (#138)</t>
         </is>
       </c>
       <c r="N7" s="9" t="inlineStr">
@@ -10168,7 +10298,32 @@
           <t xml:space="preserve">ADR-007</t>
         </is>
       </c>
-      <c r="O7" s="9" t="s">
+      <c r="O7" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-14, TC-15, TC-32, TC-33</t>
+        </is>
+      </c>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A complete submission is saved as New, appears in the requester's list, and every field shows unchanged.</t>
+        </is>
+      </c>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R7" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S7" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 of 2. AC1. persisted as New and in the requester's list: Met. TC-14, TC-32, TC-33 AC2. every field displayed unchanged on the detail: Met. TC-33, TC-15</t>
+        </is>
+      </c>
+      <c r="T7" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -10218,12 +10373,12 @@
       </c>
       <c r="L8" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">request-capture/validation.js (#131), categories.activeIds and listActive (#155), administration (#155)</t>
         </is>
       </c>
       <c r="M8" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">tests/request-submission.test.js, tests/api-submission-boundaries.test.js (#147), tests/api-postgres.test.js</t>
         </is>
       </c>
       <c r="N8" s="10" t="inlineStr">
@@ -10231,7 +10386,32 @@
           <t xml:space="preserve">FEC-02, ADR-007</t>
         </is>
       </c>
-      <c r="O8" s="10" t="s">
+      <c r="O8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-13, TC-26, TC-43, TC-32</t>
+        </is>
+      </c>
+      <c r="P8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Only active categories are offered, and any other value is refused, also directly at the endpoint.</t>
+        </is>
+      </c>
+      <c r="Q8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 of 2. AC1. only active categories offered: Met. GET /api/categories lists active ones; a deactivated category disappears from it (TC-32, TC-43) AC2. any other value refused, also directly: Met. TC-13, TC-26, TC-32; also when deactivated during the submission</t>
+        </is>
+      </c>
+      <c r="T8" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -10281,12 +10461,12 @@
       </c>
       <c r="L9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">request-capture/validation.js and src/shared/text.js (#131), client submit screen (#133)</t>
         </is>
       </c>
       <c r="M9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">tests/request-submission.test.js, tests/api-submission-boundaries.test.js, tests/api-input-partitions.test.js (#147), e2e (#138, #157)</t>
         </is>
       </c>
       <c r="N9" s="9" t="inlineStr">
@@ -10294,7 +10474,32 @@
           <t xml:space="preserve">ADR-007</t>
         </is>
       </c>
-      <c r="O9" s="9" t="s">
+      <c r="O9" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-13, TC-25, TC-26, TC-37, TC-32, TC-33</t>
+        </is>
+      </c>
+      <c r="P9" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An invalid submission saves nothing, names each failing field, and keeps what was typed.</t>
+        </is>
+      </c>
+      <c r="Q9" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R9" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEF-011, DEF-012 (fixed)</t>
+        </is>
+      </c>
+      <c r="S9" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 of 1. AC1. not persisted, each failing field named, values retained: Met. TC-13, TC-25, TC-26, TC-37; TC-33 checks the typed values stay (#157)</t>
+        </is>
+      </c>
+      <c r="T9" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -10344,12 +10549,12 @@
       </c>
       <c r="L10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">request-capture/reference.js (#131), request_reference_seq and the unique constraint (#109, #155)</t>
         </is>
       </c>
       <c r="M10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">tests/request-submission.test.js (#131), tests/api-postgres.test.js (#155), e2e (#138)</t>
         </is>
       </c>
       <c r="N10" s="10" t="inlineStr">
@@ -10357,7 +10562,32 @@
           <t xml:space="preserve">DEC-004, ADR-007</t>
         </is>
       </c>
-      <c r="O10" s="10" t="s">
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-12, TC-32, TC-33</t>
+        </is>
+      </c>
+      <c r="P10" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Every reference matches CC-dddd-dddd, is unique, never reissued, and shows on every view.</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R10" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S10" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 of 4. AC1. matches the agreed format (DEC-017): Met. TC-12, TC-32, TC-33 AC2. two requests never share a reference: Met. keyed permutation of the sequence under a unique constraint (TC-12, TC-32) AC3. not reissued after deletion or archiving: Met. nothing deletes a request, and the sequence never reuses a value (TC-12) AC4. shown on submission and every later view: Met. TC-33, TC-34</t>
+        </is>
+      </c>
+      <c r="T10" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -10407,12 +10637,12 @@
       </c>
       <c r="L11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">request-capture/http.js (#131), client acknowledgement (#133)</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">tests/request-submission.test.js, e2e (#138)</t>
         </is>
       </c>
       <c r="N11" s="9" t="inlineStr">
@@ -10420,7 +10650,32 @@
           <t xml:space="preserve">ADR-007</t>
         </is>
       </c>
-      <c r="O11" s="9" t="s">
+      <c r="O11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-14, TC-33</t>
+        </is>
+      </c>
+      <c r="P11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The acknowledgement holds the reference and recorded time, the same as the detail.</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 of 1. AC1. reference and timestamp, the same on the detail: Met. TC-14, TC-33</t>
+        </is>
+      </c>
+      <c r="T11" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -10470,12 +10725,12 @@
       </c>
       <c r="L12" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scope in src/modules/authorisation-policy/policy.js (#94, merged). List not yet implemented</t>
+          <t xml:space="preserve">request-access/views.js (#131), client list (#133)</t>
         </is>
       </c>
       <c r="M12" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scope tested in tests/authorisation-policy.test.js (#94). List planned (M3)</t>
+          <t xml:space="preserve">tests/request-submission.test.js, e2e (#138)</t>
         </is>
       </c>
       <c r="N12" s="10" t="inlineStr">
@@ -10483,7 +10738,32 @@
           <t xml:space="preserve">ADR-006</t>
         </is>
       </c>
-      <c r="O12" s="10" t="s">
+      <c r="O12" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-15, TC-33, TC-32</t>
+        </is>
+      </c>
+      <c r="P12" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Every own request once with six fields, and nobody else's.</t>
+        </is>
+      </c>
+      <c r="Q12" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R12" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S12" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 of 1. AC1. every own request once, six fields, none of another's: Met. TC-15, TC-32, TC-33</t>
+        </is>
+      </c>
+      <c r="T12" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -10533,12 +10813,12 @@
       </c>
       <c r="L13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scope in src/modules/authorisation-policy/policy.js (#94, merged). Detail view not yet implemented</t>
+          <t xml:space="preserve">request-access/views.js (#131, #155)</t>
         </is>
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/authorisation-policy.test.js (#94). The payload negative test is planned (M3)</t>
+          <t xml:space="preserve">tests/request-submission.test.js, tests/api-postgres.test.js, e2e</t>
         </is>
       </c>
       <c r="N13" s="9" t="inlineStr">
@@ -10546,7 +10826,32 @@
           <t xml:space="preserve">RSK-05, FEC-01, DEC-003, ADR-006</t>
         </is>
       </c>
-      <c r="O13" s="9" t="s">
+      <c r="O13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-03, TC-15, TC-32, TC-34</t>
+        </is>
+      </c>
+      <c r="P13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fields, ordered history and only requester-visible entries, with no internal entry in the payload.</t>
+        </is>
+      </c>
+      <c r="Q13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEF-006 (fixed)</t>
+        </is>
+      </c>
+      <c r="S13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 of 2. AC1. fields, ordered history with times, visible entries only: Met. TC-15, TC-34 AC2. no internal entry in the payload: Met. TC-03, TC-32, also when the store ignores the condition</t>
+        </is>
+      </c>
+      <c r="T13" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -10596,12 +10901,12 @@
       </c>
       <c r="L14" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/authorisation-policy/policy.js (#94, merged)</t>
+          <t xml:space="preserve">policy.js scopedWhere (#94), used by every lookup (#131, #155)</t>
         </is>
       </c>
       <c r="M14" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/authorisation-policy.test.js (#94): the query condition and the single-request check select the same requests. Endpoint negative test planned (M3)</t>
+          <t xml:space="preserve">tests/authorisation-policy.test.js, tests/request-submission.test.js, tests/api-decision-table.test.js (#147), tests/api-postgres.test.js</t>
         </is>
       </c>
       <c r="N14" s="10" t="inlineStr">
@@ -10609,7 +10914,32 @@
           <t xml:space="preserve">RSK-05, FEC-01, ADR-006</t>
         </is>
       </c>
-      <c r="O14" s="10" t="s">
+      <c r="O14" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-02, TC-15, TC-22, TC-23, TC-32</t>
+        </is>
+      </c>
+      <c r="P14" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Another requester's record is refused with the same answer as a missing one, through any route.</t>
+        </is>
+      </c>
+      <c r="Q14" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R14" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S14" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 of 1. AC1. access refused, no field disclosed, any route: Met. same 404 as a missing reference, in PostgreSQL too (TC-32)</t>
+        </is>
+      </c>
+      <c r="T14" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -10659,12 +10989,12 @@
       </c>
       <c r="L15" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/authorisation-policy/policy.js (#94, merged)</t>
+          <t xml:space="preserve">src/modules/queue (#141, #155)</t>
         </is>
       </c>
       <c r="M15" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/authorisation-policy.test.js (#94). Queue planned (M3)</t>
+          <t xml:space="preserve">tests/queue.test.js, tests/api-decision-table.test.js (#147), tests/api-postgres.test.js</t>
         </is>
       </c>
       <c r="N15" s="9" t="inlineStr">
@@ -10672,7 +11002,32 @@
           <t xml:space="preserve">FEC-01, ADR-006</t>
         </is>
       </c>
-      <c r="O15" s="9" t="s">
+      <c r="O15" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-40, TC-22, TC-32, TC-34</t>
+        </is>
+      </c>
+      <c r="P15" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Staff see every open request in their categories and none outside; a Coordinator sees all.</t>
+        </is>
+      </c>
+      <c r="Q15" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R15" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S15" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 of 2. AC1. Staff: every open request in their categories, none outside: Met. TC-40, TC-22 scope cases, TC-32 AC2. a Coordinator sees all categories: Met. TC-40, TC-32</t>
+        </is>
+      </c>
+      <c r="T15" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -10722,12 +11077,12 @@
       </c>
       <c r="L16" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">queue/validation.js and service.js (#141, #155), client queue filters (#134)</t>
         </is>
       </c>
       <c r="M16" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">tests/queue.test.js, client/test/staff-screens.test.js, tests/api-postgres.test.js</t>
         </is>
       </c>
       <c r="N16" s="10" t="inlineStr">
@@ -10735,7 +11090,32 @@
           <t xml:space="preserve">FEC-06, ADR-007</t>
         </is>
       </c>
-      <c r="O16" s="10" t="s">
+      <c r="O16" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-40, TC-29, TC-32</t>
+        </is>
+      </c>
+      <c r="P16" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Each search, filter and sort returns only matching records, filters combine, and an empty result is reported as such.</t>
+        </is>
+      </c>
+      <c r="Q16" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R16" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S16" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 of 1. AC1. each search, filter and sort correct, combining, empty reported: Met. TC-40, TC-29, TC-32 (priority sorts in PostgreSQL)</t>
+        </is>
+      </c>
+      <c r="T16" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -10785,12 +11165,12 @@
       </c>
       <c r="L17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/workflow-status/transition-table.js and transitions.js (#93, merged); src/modules/authorisation-policy/policy.js (#94, merged)</t>
+          <t xml:space="preserve">workflow-status/service.js (#132), assignable staff (#155)</t>
         </is>
       </c>
       <c r="M17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/workflow-status.test.js (#93) and tests/authorisation-policy.test.js (#94). Endpoint tests planned (M3)</t>
+          <t xml:space="preserve">tests/workflow-service.test.js, tests/api-decision-table.test.js, tests/api-input-partitions.test.js (#147), tests/api-postgres.test.js, e2e</t>
         </is>
       </c>
       <c r="N17" s="9" t="inlineStr">
@@ -10798,7 +11178,32 @@
           <t xml:space="preserve">ADR-005, ADR-006, CR-002 (#92)</t>
         </is>
       </c>
-      <c r="O17" s="9" t="s">
+      <c r="O17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-16, TC-22, TC-37, TC-32, TC-34</t>
+        </is>
+      </c>
+      <c r="P17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment is recorded and the request reaches the assignee's queue; Staff accepting become the assignee; Staff cannot assign.</t>
+        </is>
+      </c>
+      <c r="Q17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEF-003 (fixed), DEF-007 (fixed), DEF-013 (fixed)</t>
+        </is>
+      </c>
+      <c r="S17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 of 3. AC1. Coordinator assigns: recorded, in the assignee's queue: Met. TC-16, TC-32, TC-34 AC2. Staff accept an unassigned request in scope and become the assignee: Met. TC-16, TC-22 scope cases AC3. Staff cannot assign to another user: Met. TC-22</t>
+        </is>
+      </c>
+      <c r="T17" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -10848,12 +11253,12 @@
       </c>
       <c r="L18" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/workflow-status/transition-table.js and transitions.js (#93, merged 29 September 2026)</t>
+          <t xml:space="preserve">workflow-status/transition-table.js and service.js (#93, #132)</t>
         </is>
       </c>
       <c r="M18" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/workflow-status.test.js: all 196 combinations of status pair and role against a fixture exported from the Status Model register; three deliberate faults each failed the suite (#93). Refusal at the endpoint planned (M3)</t>
+          <t xml:space="preserve">tests/workflow-status.test.js, tests/api-state-transitions.test.js (#147), tests/api-postgres.test.js</t>
         </is>
       </c>
       <c r="N18" s="10" t="inlineStr">
@@ -10861,7 +11266,32 @@
           <t xml:space="preserve">RSK-09, FEC-02, ADR-001, ADR-005, ADR-006, CR-002 (#92)</t>
         </is>
       </c>
-      <c r="O18" s="10" t="s">
+      <c r="O18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-05, TC-06, TC-07, TC-24, TC-32</t>
+        </is>
+      </c>
+      <c r="P18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Every allowed move succeeds for an authorised role, every other is refused, directly too, leaving the status unchanged.</t>
+        </is>
+      </c>
+      <c r="Q18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 of 2. AC1. allowed moves succeed, others refused, directly too: Met. TC-05 against the register, TC-24 every pair through the endpoint AC2. a refused move leaves the status unchanged: Met. TC-24; TC-32 for two concurrent moves</t>
+        </is>
+      </c>
+      <c r="T18" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -10911,12 +11341,12 @@
       </c>
       <c r="L19" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scope in src/modules/authorisation-policy/policy.js (#94, merged). Recording not yet implemented</t>
+          <t xml:space="preserve">workflow-status/service.js recordActionEntry (#132)</t>
         </is>
       </c>
       <c r="M19" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scope tested in tests/authorisation-policy.test.js (#94). Recording planned (M3)</t>
+          <t xml:space="preserve">tests/workflow-service.test.js, tests/api-postgres.test.js, e2e</t>
         </is>
       </c>
       <c r="N19" s="9" t="inlineStr">
@@ -10924,7 +11354,32 @@
           <t xml:space="preserve">RSK-05, DEC-003, ADR-006</t>
         </is>
       </c>
-      <c r="O19" s="9" t="s">
+      <c r="O19" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-20, TC-32, TC-34</t>
+        </is>
+      </c>
+      <c r="P19" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An entry is stored with author, time and visibility, and visibility has no default.</t>
+        </is>
+      </c>
+      <c r="Q19" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R19" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S19" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 of 2. AC1. stored with author, timestamp and visibility: Met. TC-20, TC-32 AC2. visibility chosen explicitly, no default: Met. TC-20, TC-32 (no choice answers 400)</t>
+        </is>
+      </c>
+      <c r="T19" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -10974,12 +11429,12 @@
       </c>
       <c r="L20" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/workflow-status/transition-table.js and transitions.js (#93, merged)</t>
+          <t xml:space="preserve">transition-table.js guard, service.js (#93, #132)</t>
         </is>
       </c>
       <c r="M20" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/workflow-status.test.js (#93)</t>
+          <t xml:space="preserve">tests/workflow-service.test.js, tests/api-postgres.test.js, e2e</t>
         </is>
       </c>
       <c r="N20" s="10" t="inlineStr">
@@ -10987,7 +11442,32 @@
           <t xml:space="preserve">ADR-005</t>
         </is>
       </c>
-      <c r="O20" s="10" t="s">
+      <c r="O20" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-17, TC-32, TC-34</t>
+        </is>
+      </c>
+      <c r="P20" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resolving without a summary is refused; the summary is stored and shown to the requester.</t>
+        </is>
+      </c>
+      <c r="Q20" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R20" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S20" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 of 2. AC1. refused without a summary: Met. TC-17, TC-32 AC2. stored and requester-visible: Met. TC-32, TC-34</t>
+        </is>
+      </c>
+      <c r="T20" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -11037,12 +11517,12 @@
       </c>
       <c r="L21" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/workflow-status/transition-table.js and transitions.js (#93, merged)</t>
+          <t xml:space="preserve">transition-table.js (#93), service.js (#132)</t>
         </is>
       </c>
       <c r="M21" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/workflow-status.test.js (#93)</t>
+          <t xml:space="preserve">tests/workflow-service.test.js, tests/api-postgres.test.js, e2e</t>
         </is>
       </c>
       <c r="N21" s="9" t="inlineStr">
@@ -11050,7 +11530,32 @@
           <t xml:space="preserve">ADR-005</t>
         </is>
       </c>
-      <c r="O21" s="9" t="s">
+      <c r="O21" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-17, TC-22, TC-32, TC-34</t>
+        </is>
+      </c>
+      <c r="P21" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coordinators and Managers close a Resolved request; Staff and Requesters are refused; closing is audited.</t>
+        </is>
+      </c>
+      <c r="Q21" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R21" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S21" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 of 3. AC1. Coordinator or Manager can close: Met. TC-17, TC-32, TC-34 AC2. Staff or Requester refused: Met. TC-22, TC-32 AC3. closing audited: Met. TC-18, TC-32 row by row</t>
+        </is>
+      </c>
+      <c r="T21" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -11100,12 +11605,12 @@
       </c>
       <c r="L22" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/workflow-status/transition-table.js and transitions.js (#93, merged)</t>
+          <t xml:space="preserve">transition-table.js guard (#93), service.js (#132), views.js (#155)</t>
         </is>
       </c>
       <c r="M22" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/workflow-status.test.js (#93)</t>
+          <t xml:space="preserve">tests/workflow-service.test.js, tests/request-submission.test.js, tests/api-postgres.test.js</t>
         </is>
       </c>
       <c r="N22" s="10" t="inlineStr">
@@ -11113,7 +11618,32 @@
           <t xml:space="preserve">ADR-005, ADR-006, CR-002 (#92)</t>
         </is>
       </c>
-      <c r="O22" s="10" t="s">
+      <c r="O22" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-17, TC-15, TC-32</t>
+        </is>
+      </c>
+      <c r="P22" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rejection needs a reason; the reason is stored, shown to the requester, and the event audited.</t>
+        </is>
+      </c>
+      <c r="Q22" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R22" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEF-004 (fixed), DEF-006 (fixed)</t>
+        </is>
+      </c>
+      <c r="S22" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 of 2. AC1. refused without a reason: Met. TC-17 AC2. Rejected, reason stored, on the requester's detail, audited: Met. TC-15, TC-32 since DEF-006 was fixed</t>
+        </is>
+      </c>
+      <c r="T22" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -11163,12 +11693,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/authorisation-policy/policy.js (#94, merged). Priority change not yet implemented</t>
+          <t xml:space="preserve">service.js setPriority (#132), policy.js (#94), views.js (#131)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/authorisation-policy.test.js (#94). Priority change planned (M3)</t>
+          <t xml:space="preserve">tests/workflow-service.test.js, tests/api-decision-table.test.js, tests/api-postgres.test.js, e2e</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -11176,7 +11706,32 @@
           <t xml:space="preserve">DEC-002, ADR-006, CR-002 (#92)</t>
         </is>
       </c>
-      <c r="O23" s="9" t="s">
+      <c r="O23" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-19, TC-22, TC-32, TC-34</t>
+        </is>
+      </c>
+      <c r="P23" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Urgency is the requester's and unchanged; priority is absent until a Coordinator sets it; others are refused; Coordinators see both.</t>
+        </is>
+      </c>
+      <c r="Q23" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R23" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEF-005 (fixed)</t>
+        </is>
+      </c>
+      <c r="S23" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 of 4. AC1. urgency captured, not editable by staff: Met. TC-19, TC-34 AC2. priority absent until a Coordinator sets it: Met. TC-19, TC-34 AC3. Requester or Staff refused: Met. TC-22, TC-32 AC4. both visible to Coordinators: Met. TC-34, TC-40</t>
+        </is>
+      </c>
+      <c r="T23" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -11226,12 +11781,12 @@
       </c>
       <c r="L24" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">src/modules/reports (#143, #155)</t>
         </is>
       </c>
       <c r="M24" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">tests/reports.test.js, tests/api-decision-table.test.js, tests/api-postgres.test.js, client/test/manager-screens.test.js</t>
         </is>
       </c>
       <c r="N24" s="10" t="inlineStr">
@@ -11239,7 +11794,32 @@
           <t xml:space="preserve">RSK-09, FEC-02, FEC-06, ADR-001</t>
         </is>
       </c>
-      <c r="O24" s="10" t="s">
+      <c r="O24" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-42, TC-30, TC-32</t>
+        </is>
+      </c>
+      <c r="P24" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Each count equals the value worked out by hand from the seeded data, overdue using the one organisation-wide target.</t>
+        </is>
+      </c>
+      <c r="Q24" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R24" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S24" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.5 of 2. AC1. each count equals the independent calculation: Met. TC-42 worked examples, including an age equal to the target AC2. overdue uses the single organisation-wide target defined in the status model: Partially met. one organisation-wide target is used, but it is configuration (OVERDUE_TARGET_DAYS), because the Status Model register defines none (FEC-02)</t>
+        </is>
+      </c>
+      <c r="T24" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -11289,12 +11869,12 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">reports/service.js (#143, #155)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">tests/reports.test.js, tests/api-postgres.test.js</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
@@ -11302,7 +11882,32 @@
           <t xml:space="preserve">FEC-06, ADR-001</t>
         </is>
       </c>
-      <c r="O25" s="9" t="s">
+      <c r="O25" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-42, TC-30, TC-32</t>
+        </is>
+      </c>
+      <c r="P25" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The breakdown reconciles exactly to the totals.</t>
+        </is>
+      </c>
+      <c r="Q25" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R25" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S25" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 of 1. AC1. breakdown reconciles to FR-022's totals: Met. TC-42, TC-32</t>
+        </is>
+      </c>
+      <c r="T25" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -11352,12 +11957,12 @@
       </c>
       <c r="L26" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">reports/service.js (#143, #155)</t>
         </is>
       </c>
       <c r="M26" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">tests/reports.test.js, tests/api-postgres.test.js</t>
         </is>
       </c>
       <c r="N26" s="10" t="inlineStr">
@@ -11365,7 +11970,32 @@
           <t xml:space="preserve">FEC-02, ADR-001</t>
         </is>
       </c>
-      <c r="O26" s="10" t="s">
+      <c r="O26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-42, TC-32</t>
+        </is>
+      </c>
+      <c r="P26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Every overdue request once with four fields, and none within the target.</t>
+        </is>
+      </c>
+      <c r="Q26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 of 1. AC1. every overdue request once with four fields, none within target: Met. TC-42, TC-32</t>
+        </is>
+      </c>
+      <c r="T26" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -11415,12 +12045,12 @@
       </c>
       <c r="L27" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">src/modules/audit/audit.js, service.js transactions (#132), persistence store.js (#155)</t>
         </is>
       </c>
       <c r="M27" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">tests/workflow-service.test.js, tests/api-state-transitions.test.js, tests/api-postgres.test.js</t>
         </is>
       </c>
       <c r="N27" s="9" t="inlineStr">
@@ -11428,7 +12058,32 @@
           <t xml:space="preserve">ADR-001, ADR-007</t>
         </is>
       </c>
-      <c r="O27" s="9" t="s">
+      <c r="O27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-04, TC-18, TC-24, TC-32</t>
+        </is>
+      </c>
+      <c r="P27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Each change of status, assignee or priority creates exactly one complete audit entry with the true previous value.</t>
+        </is>
+      </c>
+      <c r="Q27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 of 1. AC1. exactly one complete entry per change, previous value correct: Met. TC-18; TC-32 row by row in PostgreSQL</t>
+        </is>
+      </c>
+      <c r="T27" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -11478,12 +12133,12 @@
       </c>
       <c r="L28" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/authorisation-policy/policy.js (#94, merged)</t>
+          <t xml:space="preserve">no route edits or deletes an audit entry; the application's database role has no UPDATE or DELETE on audit_entries (docs/deployment/app-role.sql, #155)</t>
         </is>
       </c>
       <c r="M28" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/authorisation-policy.test.js (#94): the Access Matrix row denies every role. Endpoint test planned (M3)</t>
+          <t xml:space="preserve">tests/authorisation-policy.test.js, tests/api-decision-table.test.js (#147), simulated production check (#155)</t>
         </is>
       </c>
       <c r="N28" s="10" t="inlineStr">
@@ -11491,7 +12146,32 @@
           <t xml:space="preserve">ADR-006</t>
         </is>
       </c>
-      <c r="O28" s="10" t="s">
+      <c r="O28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-04, TC-22, TC-32</t>
+        </is>
+      </c>
+      <c r="P28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No endpoint changes an audit entry, an attempt is refused, verified by review and negative test.</t>
+        </is>
+      </c>
+      <c r="Q28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md; as civicconnect_app, UPDATE and DELETE on audit_entries answer permission denied (17 October 2026)</t>
+        </is>
+      </c>
+      <c r="R28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 of 3. AC1. no endpoint accepts update or delete: Met. TC-04 AC2. an attempt through an exposed route is refused: Met. TC-22 editAuditEntry for every role; the database role refuses it AC3. verified by review and negative test: Met. TC-04, TC-22; review of #155</t>
+        </is>
+      </c>
+      <c r="T28" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -11541,12 +12221,12 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">src/modules/administration (#155, #157)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">tests/administration.test.js, tests/api-postgres.test.js</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
@@ -11554,7 +12234,32 @@
           <t xml:space="preserve">ADR-007</t>
         </is>
       </c>
-      <c r="O29" s="9" t="s">
+      <c r="O29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-43, TC-31, TC-32</t>
+        </is>
+      </c>
+      <c r="P29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A deactivated category is not offered but still shows on its requests; deleting one is refused with the reason.</t>
+        </is>
+      </c>
+      <c r="Q29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 of 2. AC1. deactivated: not offered, still shown on existing requests: Met. TC-43, TC-32 AC2. deleting a referenced category refused with an explanation: Met. 409 with the reason and what to do instead (TC-43, TC-32, #157)</t>
+        </is>
+      </c>
+      <c r="T29" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -11604,12 +12309,12 @@
       </c>
       <c r="L30" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">administration/service.js deactivateUser (#155); authenticate reads active on every call (#130)</t>
         </is>
       </c>
       <c r="M30" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">tests/administration.test.js, tests/identity-access.test.js, tests/api-postgres.test.js</t>
         </is>
       </c>
       <c r="N30" s="10" t="inlineStr">
@@ -11617,7 +12322,32 @@
           <t xml:space="preserve">ADR-007</t>
         </is>
       </c>
-      <c r="O30" s="10" t="s">
+      <c r="O30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-43, TC-09, TC-32</t>
+        </is>
+      </c>
+      <c r="P30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A deactivated account cannot sign in or act, and what it wrote stays visible and attributed.</t>
+        </is>
+      </c>
+      <c r="Q30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEF-008 (fixed)</t>
+        </is>
+      </c>
+      <c r="S30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 of 2. AC1. cannot authenticate: Met. TC-09; TC-32 ends its session at once AC2. its requests, entries and audit entries remain, attributed: Met. TC-32 (#157)</t>
+        </is>
+      </c>
+      <c r="T30" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -11667,12 +12397,12 @@
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">src/modules/notifications (#142, #155)</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">tests/notifications.test.js, tests/api-postgres.test.js</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
@@ -11680,7 +12410,32 @@
           <t xml:space="preserve">DEC-005, SC-D-01, FEC-03, ADR-008</t>
         </is>
       </c>
-      <c r="O31" s="9" t="s">
+      <c r="O31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-41, TC-32</t>
+        </is>
+      </c>
+      <c r="P31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">After each of the four events the requester sees an indication naming the request and the event.</t>
+        </is>
+      </c>
+      <c r="Q31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 of 1. AC1. an indication for each of the four events: Met. TC-41, TC-32</t>
+        </is>
+      </c>
+      <c r="T31" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -11730,12 +12485,12 @@
       </c>
       <c r="L32" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">queue with paging and indexes (#141, #109, #155)</t>
         </is>
       </c>
       <c r="M32" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3): 20 timed retrievals against a seeded 5 000-request dataset</t>
+          <t xml:space="preserve">perf/nfr-001-queue.mjs (#139, #150)</t>
         </is>
       </c>
       <c r="N32" s="10" t="inlineStr">
@@ -11743,7 +12498,32 @@
           <t xml:space="preserve">FEC-04, FEC-06, ADR-001, ADR-006</t>
         </is>
       </c>
-      <c r="O32" s="10" t="s">
+      <c r="O32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-35</t>
+        </is>
+      </c>
+      <c r="P32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p95 of 20 first-page retrievals with 5,000 requests under 2.0 s.</t>
+        </is>
+      </c>
+      <c r="Q32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Simulated production build at rc-f47d054, 17 October 2026: p95 7.4 ms (client and server on one machine)</t>
+        </is>
+      </c>
+      <c r="R32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 of 1. AC1. p95 under 2.0 s at 5,000 requests: Met. p95 7.4 ms, no network in the path (TC-35)</t>
+        </is>
+      </c>
+      <c r="T32" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -11793,12 +12573,12 @@
       </c>
       <c r="L33" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">request-capture (#131, #155)</t>
         </is>
       </c>
       <c r="M33" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">perf/nfr-002-submission.mjs (#139, #150)</t>
         </is>
       </c>
       <c r="N33" s="9" t="inlineStr">
@@ -11806,7 +12586,32 @@
           <t xml:space="preserve">ADR-007</t>
         </is>
       </c>
-      <c r="O33" s="9" t="s">
+      <c r="O33" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-35</t>
+        </is>
+      </c>
+      <c r="P33" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p95 of 20 submissions under 3.0 s.</t>
+        </is>
+      </c>
+      <c r="Q33" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Simulated production build at rc-f47d054, 17 October 2026: p95 7.9 ms</t>
+        </is>
+      </c>
+      <c r="R33" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S33" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 of 1. AC1. p95 under 3.0 s: Met. p95 7.9 ms (TC-35)</t>
+        </is>
+      </c>
+      <c r="T33" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -11856,12 +12661,12 @@
       </c>
       <c r="L34" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Health endpoint in src/app.js (#90, open)</t>
+          <t xml:space="preserve">/health probes the database (#155)</t>
         </is>
       </c>
       <c r="M34" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/health.test.js (#90, open). Availability measurement planned (M3)</t>
+          <t xml:space="preserve">tests/http-hardening.test.js (#155)</t>
         </is>
       </c>
       <c r="N34" s="10" t="inlineStr">
@@ -11869,7 +12674,32 @@
           <t xml:space="preserve">RSK-02, FEC-05, DEC-010</t>
         </is>
       </c>
-      <c r="O34" s="10" t="s">
+      <c r="O34" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-44</t>
+        </is>
+      </c>
+      <c r="P34" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">98% availability over service hours, measured monthly.</t>
+        </is>
+      </c>
+      <c r="Q34" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not measured: no hosted service ran for a month (PED v4.0 s41)</t>
+        </is>
+      </c>
+      <c r="R34" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S34" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 1. AC1. 98% availability, assessed monthly: Not met. the probe target exists (TC-44), but no month of hosted service exists to measure</t>
+        </is>
+      </c>
+      <c r="T34" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -11919,12 +12749,12 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">argon2 in identity-access and wiring.js (#130, #155)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">tests/rsk01.test.js (#90), tests/password-reset.test.js, tests/identity-access.test.js</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
@@ -11932,7 +12762,32 @@
           <t xml:space="preserve">RSK-05, ADR-002</t>
         </is>
       </c>
-      <c r="O35" s="9" t="s">
+      <c r="O35" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-36, TC-38</t>
+        </is>
+      </c>
+      <c r="P35" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Passwords stored only as a slow, salted hash.</t>
+        </is>
+      </c>
+      <c r="Q35" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R35" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEF-001 (fixed)</t>
+        </is>
+      </c>
+      <c r="S35" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 of 1. AC1. slow, salted hash only: Met. argon2id with a per-user salt; no other storage (RSK-01 test)</t>
+        </is>
+      </c>
+      <c r="T35" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -11982,12 +12837,12 @@
       </c>
       <c r="L36" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/modules/authorisation-policy/policy.js (#94, merged)</t>
+          <t xml:space="preserve">policy.js (#94), every route behind authenticate and the policy (#155)</t>
         </is>
       </c>
       <c r="M36" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/authorisation-policy.test.js (#94): all sixty Access Matrix cells; four deliberate faults each failed the suite. Endpoint negative tests planned (M3)</t>
+          <t xml:space="preserve">tests/api-decision-table.test.js (#147), tests/authorisation-policy.test.js</t>
         </is>
       </c>
       <c r="N36" s="10" t="inlineStr">
@@ -11995,7 +12850,32 @@
           <t xml:space="preserve">RSK-05, FEC-01, ADR-006, CR-002 (#92)</t>
         </is>
       </c>
-      <c r="O36" s="10" t="s">
+      <c r="O36" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-01, TC-22, TC-32</t>
+        </is>
+      </c>
+      <c r="P36" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No access succeeds anywhere in the negative matrix, called directly at the endpoints.</t>
+        </is>
+      </c>
+      <c r="Q36" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R36" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEF-002 to DEF-005 (fixed)</t>
+        </is>
+      </c>
+      <c r="S36" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 of 1. AC1. zero successful accesses across the negative matrix, at the endpoints: Met. TC-22: 56 cells through their own endpoint and editAuditEntry's 4 at the permission check (no endpoint by FR-026), with category scope varied</t>
+        </is>
+      </c>
+      <c r="T36" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -12045,12 +12925,12 @@
       </c>
       <c r="L37" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">HTTPS, the HTTP redirect, HSTS and the content security policy (src/server.js, src/app.js, #155)</t>
         </is>
       </c>
       <c r="M37" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">tools/smoke-check.mjs (#155)</t>
         </is>
       </c>
       <c r="N37" s="9" t="inlineStr">
@@ -12058,7 +12938,32 @@
           <t xml:space="preserve">DEC-010</t>
         </is>
       </c>
-      <c r="O37" s="9" t="s">
+      <c r="O37" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-44, smoke check</t>
+        </is>
+      </c>
+      <c r="P37" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Every request over HTTPS, plain HTTP redirected, no mixed content.</t>
+        </is>
+      </c>
+      <c r="Q37" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Simulated production over HTTPS, 17 October 2026: smoke check 7 of 7, including HSTS and the redirect</t>
+        </is>
+      </c>
+      <c r="R37" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S37" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 of 1. AC1. all over HTTPS, HTTP redirected, no mixed content: Met. in simulated production, with a self-signed certificate (PED v4.0 s41)</t>
+        </is>
+      </c>
+      <c r="T37" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -12108,12 +13013,12 @@
       </c>
       <c r="L38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gitleaks workflow (#87), merged on 30 September 2026</t>
+          <t xml:space="preserve">Gitleaks on every pull request (#87); .gitignore and .env.example (#90)</t>
         </is>
       </c>
       <c r="M38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">The secret scan runs on every pull request and push to main. It passed on #87 on 29 September 2026 and on main on 30 September 2026</t>
+          <t xml:space="preserve">.github/workflows/secret-scan.yml</t>
         </is>
       </c>
       <c r="N38" s="10" t="inlineStr">
@@ -12121,7 +13026,32 @@
           <t xml:space="preserve">RSK-11</t>
         </is>
       </c>
-      <c r="O38" s="10" t="s">
+      <c r="O38" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s30.3</t>
+        </is>
+      </c>
+      <c r="P38" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No finding from secret scanning across the whole history.</t>
+        </is>
+      </c>
+      <c r="Q38" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Full-history scan at the release tag (PED v4.0 s40.2)</t>
+        </is>
+      </c>
+      <c r="R38" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S38" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 of 1. AC1. zero findings across the full history: Met. gitleaks detect on the full history (PED v3.0 s30.3; re-run at the tag)</t>
+        </is>
+      </c>
+      <c r="T38" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -12171,12 +13101,12 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Access scope in src/modules/authorisation-policy/policy.js (#94, merged)</t>
+          <t xml:space="preserve">the data model (ADR-007) and the scope in policy.js; the Personal Data Inventory (#125)</t>
         </is>
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">PED v4.0 s38</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
@@ -12184,7 +13114,32 @@
           <t xml:space="preserve">RSK-05, RSK-10, FEC-04, ADR-006</t>
         </is>
       </c>
-      <c r="O39" s="9" t="s">
+      <c r="O39" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s38</t>
+        </is>
+      </c>
+      <c r="P39" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Only name, contact detail and request content stored as personal information, each field justified, access by FR-002.</t>
+        </is>
+      </c>
+      <c r="Q39" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">See the Personal Data Inventory</t>
+        </is>
+      </c>
+      <c r="R39" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S39" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.5 of 1. AC1. only the three kinds of personal information, each justified, access governed: Partially met. access is governed and tested (TC-01, TC-22); the inventory justifying each field is in #144, not merged</t>
+        </is>
+      </c>
+      <c r="T39" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -12234,12 +13189,12 @@
       </c>
       <c r="L40" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">the client (#133 to #135)</t>
         </is>
       </c>
       <c r="M40" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">none</t>
         </is>
       </c>
       <c r="N40" s="10" t="inlineStr">
@@ -12247,7 +13202,32 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="O40" s="10" t="s">
+      <c r="O40" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">none</t>
+        </is>
+      </c>
+      <c r="P40" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">At least 4 of 5 first-time users complete a submission unaided within 3 minutes.</t>
+        </is>
+      </c>
+      <c r="Q40" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="R40" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S40" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 1. AC1. 4 of 5 first-time users within 3 minutes: Not met. the moderated task test was not run</t>
+        </is>
+      </c>
+      <c r="T40" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -12297,12 +13277,12 @@
       </c>
       <c r="L41" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">the client's markup and styles (#133 to #135, #155)</t>
         </is>
       </c>
       <c r="M41" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3)</t>
+          <t xml:space="preserve">e2e/journeys/accessibility.spec.js (#155)</t>
         </is>
       </c>
       <c r="N41" s="9" t="inlineStr">
@@ -12310,7 +13290,32 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="O41" s="9" t="s">
+      <c r="O41" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-45</t>
+        </is>
+      </c>
+      <c r="P41" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Keyboard operable with visible focus, every control labelled, body text contrast at AA.</t>
+        </is>
+      </c>
+      <c r="Q41" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R41" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEF-009 (fixed)</t>
+        </is>
+      </c>
+      <c r="S41" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 of 1. AC1. keyboard, visible focus, labels, contrast: Met. TC-45: no WCAG 2.1 A or AA violation on any screen, and the keyboard walk</t>
+        </is>
+      </c>
+      <c r="T41" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -12360,12 +13365,12 @@
       </c>
       <c r="L42" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">audit.js and the change's transaction (#132), persistence store.js (#155)</t>
         </is>
       </c>
       <c r="M42" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned (M3): an audit entry per change type, and a reconciliation query</t>
+          <t xml:space="preserve">tests/workflow-service.test.js, tests/api-postgres.test.js</t>
         </is>
       </c>
       <c r="N42" s="10" t="inlineStr">
@@ -12373,7 +13378,32 @@
           <t xml:space="preserve">RSK-09, ADR-001, ADR-005</t>
         </is>
       </c>
-      <c r="O42" s="10" t="s">
+      <c r="O42" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-18, TC-32</t>
+        </is>
+      </c>
+      <c r="P42" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Every change produces exactly one complete audit entry, with none orphaned.</t>
+        </is>
+      </c>
+      <c r="Q42" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass on main at the release tag (PED v4.0 s40.2); records in docs/quality/test-catalogue.md</t>
+        </is>
+      </c>
+      <c r="R42" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S42" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 of 1. AC1. 100% of changes, exactly one complete entry each: Met. TC-18; TC-32 compares the audit rows with the changes made</t>
+        </is>
+      </c>
+      <c r="T42" s="10" t="s">
         <v>182</v>
       </c>
     </row>
@@ -12423,12 +13453,12 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests/ (#93, #94, merged)</t>
+          <t xml:space="preserve">CI workflow .github/workflows/ci.yml (#156), required on main by the ruleset</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">22 tests pass locally. No CI check has run yet (#67)</t>
+          <t xml:space="preserve">#156 and its blocked-merge proof</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
@@ -12436,7 +13466,32 @@
           <t xml:space="preserve">RSK-03, ADR-002</t>
         </is>
       </c>
-      <c r="O43" s="9" t="s">
+      <c r="O43" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s31</t>
+        </is>
+      </c>
+      <c r="P43" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tests covering every Must requirement pass on every pull request before merge is allowed.</t>
+        </is>
+      </c>
+      <c r="Q43" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The CI run on #156; the ruleset's required check</t>
+        </is>
+      </c>
+      <c r="R43" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S43" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.5 of 1. AC1. tests gate every merge: Partially met. the workflow runs every suite (#156); it gates a merge only once it is a required check on main</t>
+        </is>
+      </c>
+      <c r="T43" s="9" t="s">
         <v>182</v>
       </c>
     </row>
@@ -12486,12 +13541,12 @@
       </c>
       <c r="L44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not yet implemented</t>
+          <t xml:space="preserve">simulated production on a member's machine (#122, #155)</t>
         </is>
       </c>
       <c r="M44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned: a recorded cost review before release</t>
+          <t xml:space="preserve">PED v2.0 s24, PED v4.0 s41</t>
         </is>
       </c>
       <c r="N44" s="10" t="inlineStr">
@@ -12499,14 +13554,39 @@
           <t xml:space="preserve">RSK-02, FEC-05, DEC-010</t>
         </is>
       </c>
-      <c r="O44" s="10" t="s">
+      <c r="O44" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s41</t>
+        </is>
+      </c>
+      <c r="P44" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Zero running cost within free-tier limits, with the limits documented and the cost beyond projected.</t>
+        </is>
+      </c>
+      <c r="Q44" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Simulated production, 17 October 2026</t>
+        </is>
+      </c>
+      <c r="R44" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S44" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.5 of 1. AC1. zero running cost, limits documented, cost beyond projected: Partially met. zero cost and the free-tier limits documented (s24); the cost beyond the educational context is not projected</t>
+        </is>
+      </c>
+      <c r="T44" s="10" t="s">
         <v>182</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:O44"/>
+  <autoFilter ref="A2:T44"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A1:T1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
docs(#128): NFR-013's projected running cost, and the RTM and s38 at 64.5 of 69
s41.5 projects the cost beyond the educational context from Render's published prices of 18 October 2026:
USD 13.30 a month at the least (Hobby workspace, a Starter web service that does not sleep, Basic 256 MB
PostgreSQL with backups and point-in-time recovery, 1 GB), or USD 52.50 with headroom and 7 days of
recovery. 5,000 requests take 12 MB. The go-live table and s41.4 point to it. The source is listed in a
new s42.8, since s17 changes only under change control.

NFR-013 is Met in the RTM and s38 (64.5 of 69, 93.5 percent). The --m1-only count for v4.0 is 77, in the
PED README.
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -9781,7 +9781,7 @@
     <row r="1" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Requirements Traceability Matrix. From M2 (#54, CR-003), columns G to N trace each requirement to its quality driver, module, data, design, technology, implementation and verification evidence. From the Final (CR-006, #126), columns O to S give the M3 and final trace: the test cases from docs/quality/test-catalogue.md, the expected result written from the criterion, the execution evidence, the defects, and the status of each acceptance criterion in the requirement's row, counted per criterion as CR-006's approval asks (Met 1.0, Partially met 0.5, Not met 0.0). Scope Completion: 64 of 69 criteria, 92.8 percent, at the release tag (PED v4.0 s38).</t>
+          <t xml:space="preserve">Requirements Traceability Matrix. From M2 (#54, CR-003), columns G to N trace each requirement to its quality driver, module, data, design, technology, implementation and verification evidence. From the Final (CR-006, #126), columns O to S give the M3 and final trace: the test cases from docs/quality/test-catalogue.md, the expected result written from the criterion, the execution evidence, the defects, and the status of each acceptance criterion in the requirement's row, counted per criterion as CR-006's approval asks (Met 1.0, Partially met 0.5, Not met 0.0). Scope Completion: 64.5 of 69 criteria, 93.5 percent, at the release tag (PED v4.0 s38).</t>
         </is>
       </c>
       <c r="B1" s="7"/>
@@ -13566,7 +13566,7 @@
       </c>
       <c r="Q44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Simulated production, 17 October 2026</t>
+          <t xml:space="preserve">Simulated production costs nothing; projection in PED v4.0 s41.5</t>
         </is>
       </c>
       <c r="R44" s="10" t="inlineStr">
@@ -13576,7 +13576,7 @@
       </c>
       <c r="S44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5 of 1. AC1. zero running cost, limits documented, cost beyond projected: Partially met. zero cost and the free-tier limits documented (s24); the cost beyond the educational context is not projected</t>
+          <t xml:space="preserve">1 of 1. AC1. zero running cost, limits documented, cost beyond projected: Met. zero cost in the assessed period; free-tier limits in PED s24; the cost beyond projected at USD 13.30 a month at the least, from Render's prices of 18 October 2026 (PED v4.0 s41.5)</t>
         </is>
       </c>
       <c r="T44" s="10" t="s">

</xml_diff>

<commit_message>
docs(#128): defects numbered as Tristan Roets's register numbers them
Tristan Roets numbered M3's three code defects DEF-006 to DEF-008 (s35, #145), so the Final's defects are
DEF-009 (the rejection reason), DEF-010 (the staff detail's moves), DEF-011 (the account-event constraint)
and DEF-012 (the date fields' focus ring), in s39.1 and in the RTM's defects column.
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -10139,7 +10139,7 @@
       </c>
       <c r="R5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEF-008 (fixed)</t>
+          <t xml:space="preserve">DEF-011 (fixed)</t>
         </is>
       </c>
       <c r="S5" s="9" t="inlineStr">
@@ -10491,7 +10491,7 @@
       </c>
       <c r="R9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEF-011, DEF-012 (fixed)</t>
+          <t xml:space="preserve">DEF-006, DEF-007 (fixed)</t>
         </is>
       </c>
       <c r="S9" s="9" t="inlineStr">
@@ -10843,7 +10843,7 @@
       </c>
       <c r="R13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEF-006 (fixed)</t>
+          <t xml:space="preserve">DEF-009 (fixed)</t>
         </is>
       </c>
       <c r="S13" s="9" t="inlineStr">
@@ -11195,7 +11195,7 @@
       </c>
       <c r="R17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEF-003 (fixed), DEF-007 (fixed), DEF-013 (fixed)</t>
+          <t xml:space="preserve">DEF-003, DEF-008, DEF-010 (fixed)</t>
         </is>
       </c>
       <c r="S17" s="9" t="inlineStr">
@@ -11635,12 +11635,12 @@
       </c>
       <c r="R22" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEF-004 (fixed), DEF-006 (fixed)</t>
+          <t xml:space="preserve">DEF-004, DEF-009 (fixed)</t>
         </is>
       </c>
       <c r="S22" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 of 2. AC1. refused without a reason: Met. TC-17 AC2. Rejected, reason stored, on the requester's detail, audited: Met. TC-15, TC-32 since DEF-006 was fixed</t>
+          <t xml:space="preserve">2 of 2. AC1. refused without a reason: Met. TC-17 AC2. Rejected, reason stored, on the requester's detail, audited: Met. TC-15, TC-32 since DEF-009 was fixed</t>
         </is>
       </c>
       <c r="T22" s="10" t="s">
@@ -12339,7 +12339,7 @@
       </c>
       <c r="R30" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEF-008 (fixed)</t>
+          <t xml:space="preserve">DEF-011 (fixed)</t>
         </is>
       </c>
       <c r="S30" s="10" t="inlineStr">
@@ -13307,7 +13307,7 @@
       </c>
       <c r="R41" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEF-009 (fixed)</t>
+          <t xml:space="preserve">DEF-012 (fixed)</t>
         </is>
       </c>
       <c r="S41" s="9" t="inlineStr">

</xml_diff>

<commit_message>
docs(#128): NFR-012 met, the CI blocker resolved, the second-machine walkthrough, and Jean Smit's risks
#158's deliberately failing test failed the required check and its merge was blocked (#110), so NFR-012
is Met in the RTM and s38 (65 of 69 with #147 and #157), and s39.2's CI blocker is resolved; the go-live
table loses its CI row. s41.2 records Tristan Roets's walkthrough on a separate machine (#155). s39.3
gives the final status of the seven risks Jean Smit owns.
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -9781,7 +9781,7 @@
     <row r="1" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Requirements Traceability Matrix. From M2 (#54, CR-003), columns G to N trace each requirement to its quality driver, module, data, design, technology, implementation and verification evidence. From the Final (CR-006, #126), columns O to S give the M3 and final trace: the test cases from docs/quality/test-catalogue.md, the expected result written from the criterion, the execution evidence, the defects, and the status of each acceptance criterion in the requirement's row, counted per criterion as CR-006's approval asks (Met 1.0, Partially met 0.5, Not met 0.0). Scope Completion: 64.5 of 69 criteria, 93.5 percent, at the release tag (PED v4.0 s38).</t>
+          <t xml:space="preserve">Requirements Traceability Matrix. From M2 (#54, CR-003), columns G to N trace each requirement to its quality driver, module, data, design, technology, implementation and verification evidence. From the Final (CR-006, #126), columns O to S give the M3 and final trace: the test cases from docs/quality/test-catalogue.md, the expected result written from the criterion, the execution evidence, the defects, and the status of each acceptance criterion in the requirement's row, counted per criterion as CR-006's approval asks (Met 1.0, Partially met 0.5, Not met 0.0). Scope Completion: 65 of 69 criteria, 94.2 percent, at the release tag (PED v4.0 s38).</t>
         </is>
       </c>
       <c r="B1" s="7"/>
@@ -13453,12 +13453,12 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">CI workflow .github/workflows/ci.yml (#156), required on main by the ruleset</t>
+          <t xml:space="preserve">CI workflow .github/workflows/ci.yml (#156); test and gitleaks required on main by the Protect main ruleset</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">#156 and its blocked-merge proof</t>
+          <t xml:space="preserve">.github/workflows/ci.yml (#156); the blocked-merge proof on #110 (#158)</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
@@ -13478,7 +13478,7 @@
       </c>
       <c r="Q43" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">The CI run on #156; the ruleset's required check</t>
+          <t xml:space="preserve">CI passed on main at e73f513, 18 October 2026; #158's deliberately failing test failed the required check and its merge was BLOCKED (actions run 39149158418)</t>
         </is>
       </c>
       <c r="R43" s="9" t="inlineStr">
@@ -13488,7 +13488,7 @@
       </c>
       <c r="S43" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5 of 1. AC1. tests gate every merge: Partially met. the workflow runs every suite (#156); it gates a merge only once it is a required check on main</t>
+          <t xml:space="preserve">1 of 1. AC1. tests gate every merge: Met. every suite runs on every pull request and push to main (#156), the check is required by the ruleset with no bypass, and a failing test blocked #158's merge (#110)</t>
         </is>
       </c>
       <c r="T43" s="9" t="s">

</xml_diff>

<commit_message>
docs(#128): Tristan Roets's final register closure: 14 risks, the defects, TD-001 to TD-009, ADR paragraphs, AI row
From Tristan Roets's final answers of 18 October 2026: the final status and reason of the 14 risks Tristan
Roets owns (s39.3); every defect closed with its regression test, DEF-013 added, and the numbering kept as
s35 has it (s39.1); TD-001 to TD-009 all kept with their costs (s39.4); the final ADR-007 and ADR-008
paragraphs (s42.4); and AI Usage Register row 33 as revised. NFR-008 is Partially met: the data
inventory is written but only in the draft #144 (s38.4).
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -6169,7 +6169,7 @@
     <row r="33" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">17 October 2026</t>
+          <t xml:space="preserve">18 October 2026</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
@@ -6184,27 +6184,27 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Supporting work during M3 and the Final Project: understanding and checking requirements, working through problems, reviewing parts of the work, and the wording of documentation and review comments.</t>
+          <t xml:space="preserve">Supporting tool during M3 and the Final Project: clarifying requirements, checking selected work against the project requirements, reviewing parts of changes and evidence, and improving the wording of documentation and review comments.</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Helped to understand and check requirements, to work through problems and to review parts of the work, improved the wording of documentation and review comments, checked whether work matched the project requirements, and pointed out things that may have been overlooked.</t>
+          <t xml:space="preserve">Suggested checks, highlighted possible omissions, helped organise wording, and helped identify missing or stale pull-request evidence and review points.</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reviewed the changes personally, checked the results and the evidence, and made the final decision on everything submitted or approved.</t>
+          <t xml:space="preserve">Checked each suggestion against the repository, the requirements, the test evidence and the current pull-request heads before using it.</t>
         </is>
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Used as a supporting tool only. The AI made no project decision and completed no task on its own.</t>
+          <t xml:space="preserve">Only suggestions matching the controlled evidence were used. The final technical and review decisions remained Tristan Roets's.</t>
         </is>
       </c>
       <c r="H33" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">None found in review.</t>
+          <t xml:space="preserve">Suggestions that did not match the controlled artefacts were corrected or discarded.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(#128): Darius Mushi's final register closure: nine risks and AI Usage Register row 34
From Darius Mushi's answers of 18 October 2026: the final status and reason of RSK-03, RSK-06, RSK-09,
RSK-12, RSK-16, RSK-20, RSK-25, RSK-26 and RSK-30 (s39.3), with his conditional answers resolved from the
repository: CR-005 and CR-006 are answered on #95 and #126, and #156 is merged and required. Row 34
records the AI use for the CI workflow (#156). No placeholder remains.
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -28,7 +28,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="13" name="_xlnm._FilterDatabase" vbProcedure="false">'Access Matrix'!$A$2:$E$17</definedName>
-    <definedName function="false" hidden="true" localSheetId="10" name="_xlnm._FilterDatabase" vbProcedure="false">'AI Usage Register'!$A$2:$H$33</definedName>
+    <definedName function="false" hidden="true" localSheetId="10" name="_xlnm._FilterDatabase" vbProcedure="false">'AI Usage Register'!$A$2:$H$34</definedName>
     <definedName function="false" hidden="true" localSheetId="16" name="_xlnm._FilterDatabase" vbProcedure="false">'Baseline Sign-off'!$A$2:$B$19</definedName>
     <definedName function="false" hidden="true" localSheetId="11" name="_xlnm._FilterDatabase" vbProcedure="false">'Change Requests'!$A$2:$P$8</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">Constraints!$A$2:$D$10</definedName>
@@ -4951,7 +4951,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -6208,8 +6208,50 @@
         </is>
       </c>
     </row>
+    <row r="34" customFormat="false" ht="160" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18 October 2026</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Darius Mushi</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Sonnet 5.5 (Anthropic)</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The GitHub Actions workflow .github/workflows/ci.yml for #110 (PR #156), plus drafting the PR description, the request to the repository owner to make the check required, and the comment text for CR-005 (#95) and CR-006 (#126).</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drafted the workflow from my specification: Node 24, a postgres:16 service with an empty database, then npm ci, prisma generate, prisma migrate deploy and npm test in the root, and npm ci and node --test in client/ and perf/, with test-only environment values. It also gave the PowerShell commands, drafted the PR text and the comment wording, and helped me set up the local walkthrough. It did not review any pull request for me.</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Compared the env block with .env.example and scanned the source for every process.env variable the code reads, which found PERF_RESULTS_DIR and its fallback in perf/lib.mjs. Read the first run's log, checked perf/package.json, and read the full git diff before committing. Confirmed in the second run (https://github.com/PVY-Smit/civicconnect/actions/runs/39092848211) that root, client and perf ran 192, 35 and 19 tests with 0 failures. Read CR-005 and CR-006 in the PED before commenting.</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted after revision.</t>
+        </is>
+      </c>
+      <c r="H34" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The first workflow had an Install (perf) step that failed because perf has no dependencies and no lockfile, so I removed it. Two AI-supplied commands were wrong (a Select-String -Recurse parameter that does not exist, and a Set-Content call that failed on this PowerShell) and were replaced. The runner was pinned to ubuntu-24.04 because ubuntu-latest moves to Ubuntu 26 on 19 October. The workflow has no lint, npm audit or client build, which #110 lists, and passing tests do not show Must-requirement coverage (NFR-012).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:H33"/>
+  <autoFilter ref="A2:H34"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs(#128): Group G as the team name, and the M1 template guidance closed
s37.1 gives the team name, Group G, as the Final brief's submission block asks, and the workbook's README
names it as owner. The template instructions left from M1 are closed: the README sheet no longer tells the
team to replace yellow placeholder cells, its version line names the final release, and the AI Usage
Register's title drops 'Highlighted cells are placeholders you must replace'. In s14.2 the M1 callout is
kept, and its reading note (CR-005, item 4) says every row is now a real entry.
</commit_message>
<xml_diff>
--- a/docs/requirements/CivicConnect_M1_Registers.xlsx
+++ b/docs/requirements/CivicConnect_M1_Registers.xlsx
@@ -3790,8 +3790,10 @@
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>4</v>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.0, baselined at the M1 engineering gate, and continued through M2, M3 and the Final Project. The final version describes release v1.0.0 (18 October 2026).</t>
+        </is>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3800,7 +3802,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jean Smit - 600368 | Tristan Roets - 601764 | Darius Mushi - 577982</t>
+          <t xml:space="preserve">Group G: Jean Smit - 600368 | Tristan Roets - 601764 | Darius Mushi - 577982</t>
         </is>
       </c>
     </row>
@@ -3815,11 +3817,15 @@
       <c r="B7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>9</v>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square brackets</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">During drafting, a value still to be completed was written in [square brackets]. None remains in the final version.</t>
+        </is>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4965,8 +4971,10 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
-        <v>748</v>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AI Usage Register (Master Brief s10.1). Complete a row at the time the work is done, not retrospectively.</t>
+        </is>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>

</xml_diff>